<commit_message>
se termina categoria de cocina
</commit_message>
<xml_diff>
--- a/BD/Catalogo_Bloopia_Estructurado.xlsx
+++ b/BD/Catalogo_Bloopia_Estructurado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimilitareduco-my.sharepoint.com/personal/est_tatiana_castillo_unimilitar_edu_co/Documents/Backup/Descargas/copiaBloopia (2)/copiaBloopia/Bloopia/BD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3597" documentId="11_39DF2C4B9F61F837F4C1046A4016A4F540A1B085" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E318E82-B307-408F-BF7A-9BCF99F78A13}"/>
+  <xr:revisionPtr revIDLastSave="3617" documentId="11_39DF2C4B9F61F837F4C1046A4016A4F540A1B085" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD541ABF-9024-4BC2-AFD7-D0C6957BFA47}"/>
   <bookViews>
     <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10295" uniqueCount="2192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10327" uniqueCount="2199">
   <si>
     <t>Codigo</t>
   </si>
@@ -39716,6 +39716,236 @@
 Deja enfriar el recipiente antes de lavarlo para prolongar la vida útil del recubrimiento.
 Usa utensilios de silicona, madera o plástico para proteger el antiadherente.
 Limpia el recipiente con una esponja suave para conservar su acabado.</t>
+    </r>
+  </si>
+  <si>
+    <t>assets/productos/cocina/ollapresion/olla.webp</t>
+  </si>
+  <si>
+    <t>assets/productos/cocina/ollapresion/olla2.webp</t>
+  </si>
+  <si>
+    <t>assets/productos/cocina/ollapresion/olla3.webp</t>
+  </si>
+  <si>
+    <t>assets/productos/cocina/ollapresion/olla4.webp</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Ahorra tiempo en la cocina con la </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Olla a Presión UNIVERSAL® de 6 Litros</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, un utensilio pensado para preparar recetas deliciosas de forma más rápida y eficiente. Gracias a su sistema de presión, conserva mejor el sabor, la textura y los nutrientes de los alimentos, reduciendo considerablemente los tiempos de cocción.
+Su sistema de cierre interno autoajustable proporciona un sellado hermético que facilita el uso y mejora la seguridad. Además, incorpora múltiples válvulas de protección para ofrecer una experiencia de cocción confiable.
+Fabricada en aluminio de alta calidad, distribuye el calor de manera uniforme para obtener resultados consistentes en cada preparación. Es ideal para cocinar carnes, fríjoles, lentejas, sopas, verduras, granos y muchas recetas más.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">La Olla a Presión UNIVERSAL® de 6 Litros </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>está diseñada para cocinar carnes, sopas, granos, verduras y muchas otras preparaciones en menos tiempo. Su sistema de cierre interno autoajustable, cuerpo de aluminio de alta resistencia y múltiples sistemas de seguridad garantizan una cocción rápida, uniforme y confiable para el uso diario.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Características principales</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Capacidad de 6 litros.
+Sistema de presión para una cocción más rápida.
+Cierre interno autoajustable para un sellado seguro.
+Cuerpo de aluminio resistente que distribuye el calor uniformemente.
+Dispositivo para liberar la presión de forma práctica y segura.
+Tres sistemas de seguridad para mayor tranquilidad.
+Ideal para carnes, sopas, granos, legumbres y verduras.
+Diseño resistente para el uso diario.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Especificaciones técnicas</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Marca: UNIVERSAL®.
+Tipo: Olla a presión.
+Capacidad: 6 litros.
+Sistema de cierre: Interno autoajustable.
+Material del cuerpo: Aluminio de 1.8 mm de espesor.
+Material de la tapa: Aluminio de 2 mm de espesor.
+Color: Según disponibilidad.
+Uso: Cocción a presión.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Sistemas de seguridad</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Válvula reguladora de presión.
+Válvula de seguridad de silicona.
+Válvula de seguridad metálica.
+Dispositivo para liberación segura de presión.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Contenido del paquete</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1 Olla a Presión UNIVERSAL® de 6 litros.
+1 Tapa con sistema de cierre interno.
+Manual de uso.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Beneficios</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Reduce significativamente los tiempos de cocción.
+Conserva mejor el sabor y la textura de los alimentos.
+Cocción uniforme gracias a su cuerpo de aluminio.
+Sistema de cierre diseñado para brindar mayor seguridad.
+Fácil de usar, abrir y cerrar.
+Materiales resistentes para una larga vida útil.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Recomendaciones de uso</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Ideal para preparar carnes más suaves en menos tiempo.
+Perfecta para cocinar fríjoles, lentejas, granos y sopas.
+Verifica que las válvulas estén limpias antes de cada uso.
+Lava y seca completamente la olla después de utilizarla para prolongar su vida útil.
+Sigue siempre las indicaciones del manual para una cocción segura.</t>
     </r>
   </si>
 </sst>
@@ -40118,7 +40348,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M912"/>
+  <dimension ref="A1:M915"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -66872,7 +67102,7 @@
         <v>25</v>
       </c>
       <c r="H714" t="s">
-        <v>19</v>
+        <v>1104</v>
       </c>
       <c r="I714" t="s">
         <v>25</v>
@@ -66910,7 +67140,7 @@
         <v>25</v>
       </c>
       <c r="H715" t="s">
-        <v>19</v>
+        <v>1104</v>
       </c>
       <c r="I715" t="s">
         <v>25</v>
@@ -66948,7 +67178,7 @@
         <v>25</v>
       </c>
       <c r="H716" t="s">
-        <v>19</v>
+        <v>1104</v>
       </c>
       <c r="I716" t="s">
         <v>25</v>
@@ -66976,14 +67206,14 @@
       <c r="D717" t="s">
         <v>533</v>
       </c>
-      <c r="E717" t="s">
-        <v>25</v>
-      </c>
-      <c r="F717" t="s">
-        <v>25</v>
+      <c r="E717">
+        <v>204998</v>
+      </c>
+      <c r="F717" s="2" t="s">
+        <v>2196</v>
       </c>
       <c r="G717" t="s">
-        <v>25</v>
+        <v>2192</v>
       </c>
       <c r="H717" t="s">
         <v>19</v>
@@ -66992,10 +67222,10 @@
         <v>25</v>
       </c>
       <c r="J717" t="s">
-        <v>25</v>
-      </c>
-      <c r="K717" t="s">
-        <v>25</v>
+        <v>2197</v>
+      </c>
+      <c r="K717" s="2" t="s">
+        <v>2198</v>
       </c>
       <c r="L717" t="s">
         <v>25</v>
@@ -67003,25 +67233,25 @@
     </row>
     <row r="718" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A718" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="B718" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="C718" t="s">
-        <v>602</v>
+        <v>443</v>
       </c>
       <c r="D718" t="s">
-        <v>25</v>
-      </c>
-      <c r="E718" t="s">
-        <v>25</v>
+        <v>533</v>
+      </c>
+      <c r="E718">
+        <v>204998</v>
       </c>
       <c r="F718" t="s">
         <v>25</v>
       </c>
       <c r="G718" t="s">
-        <v>25</v>
+        <v>2193</v>
       </c>
       <c r="H718" t="s">
         <v>19</v>
@@ -67041,25 +67271,25 @@
     </row>
     <row r="719" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A719" t="s">
-        <v>603</v>
+        <v>598</v>
       </c>
       <c r="B719" t="s">
-        <v>604</v>
+        <v>599</v>
       </c>
       <c r="C719" t="s">
-        <v>602</v>
+        <v>443</v>
       </c>
       <c r="D719" t="s">
-        <v>25</v>
-      </c>
-      <c r="E719" t="s">
-        <v>25</v>
+        <v>533</v>
+      </c>
+      <c r="E719">
+        <v>204998</v>
       </c>
       <c r="F719" t="s">
         <v>25</v>
       </c>
       <c r="G719" t="s">
-        <v>25</v>
+        <v>2194</v>
       </c>
       <c r="H719" t="s">
         <v>19</v>
@@ -67079,25 +67309,25 @@
     </row>
     <row r="720" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A720" t="s">
-        <v>605</v>
+        <v>598</v>
       </c>
       <c r="B720" t="s">
-        <v>606</v>
+        <v>599</v>
       </c>
       <c r="C720" t="s">
-        <v>602</v>
+        <v>443</v>
       </c>
       <c r="D720" t="s">
-        <v>25</v>
-      </c>
-      <c r="E720" t="s">
-        <v>25</v>
+        <v>533</v>
+      </c>
+      <c r="E720">
+        <v>204998</v>
       </c>
       <c r="F720" t="s">
         <v>25</v>
       </c>
       <c r="G720" t="s">
-        <v>25</v>
+        <v>2195</v>
       </c>
       <c r="H720" t="s">
         <v>19</v>
@@ -67117,10 +67347,10 @@
     </row>
     <row r="721" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A721" t="s">
-        <v>607</v>
+        <v>600</v>
       </c>
       <c r="B721" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="C721" t="s">
         <v>602</v>
@@ -67155,10 +67385,10 @@
     </row>
     <row r="722" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A722" t="s">
-        <v>609</v>
+        <v>603</v>
       </c>
       <c r="B722" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="C722" t="s">
         <v>602</v>
@@ -67193,10 +67423,10 @@
     </row>
     <row r="723" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A723" t="s">
-        <v>611</v>
+        <v>605</v>
       </c>
       <c r="B723" t="s">
-        <v>612</v>
+        <v>606</v>
       </c>
       <c r="C723" t="s">
         <v>602</v>
@@ -67231,10 +67461,10 @@
     </row>
     <row r="724" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A724" t="s">
-        <v>613</v>
+        <v>607</v>
       </c>
       <c r="B724" t="s">
-        <v>614</v>
+        <v>608</v>
       </c>
       <c r="C724" t="s">
         <v>602</v>
@@ -67269,10 +67499,10 @@
     </row>
     <row r="725" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A725" t="s">
-        <v>615</v>
+        <v>609</v>
       </c>
       <c r="B725" t="s">
-        <v>616</v>
+        <v>610</v>
       </c>
       <c r="C725" t="s">
         <v>602</v>
@@ -67307,16 +67537,16 @@
     </row>
     <row r="726" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A726" t="s">
-        <v>617</v>
+        <v>611</v>
       </c>
       <c r="B726" t="s">
-        <v>618</v>
+        <v>612</v>
       </c>
       <c r="C726" t="s">
-        <v>619</v>
+        <v>602</v>
       </c>
       <c r="D726" t="s">
-        <v>620</v>
+        <v>25</v>
       </c>
       <c r="E726" t="s">
         <v>25</v>
@@ -67345,16 +67575,16 @@
     </row>
     <row r="727" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A727" t="s">
-        <v>621</v>
+        <v>613</v>
       </c>
       <c r="B727" t="s">
-        <v>622</v>
+        <v>614</v>
       </c>
       <c r="C727" t="s">
-        <v>619</v>
+        <v>602</v>
       </c>
       <c r="D727" t="s">
-        <v>620</v>
+        <v>25</v>
       </c>
       <c r="E727" t="s">
         <v>25</v>
@@ -67383,16 +67613,16 @@
     </row>
     <row r="728" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A728" t="s">
-        <v>623</v>
+        <v>615</v>
       </c>
       <c r="B728" t="s">
-        <v>624</v>
+        <v>616</v>
       </c>
       <c r="C728" t="s">
-        <v>619</v>
+        <v>602</v>
       </c>
       <c r="D728" t="s">
-        <v>620</v>
+        <v>25</v>
       </c>
       <c r="E728" t="s">
         <v>25</v>
@@ -67421,10 +67651,10 @@
     </row>
     <row r="729" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A729" t="s">
-        <v>625</v>
+        <v>617</v>
       </c>
       <c r="B729" t="s">
-        <v>626</v>
+        <v>618</v>
       </c>
       <c r="C729" t="s">
         <v>619</v>
@@ -67459,16 +67689,16 @@
     </row>
     <row r="730" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A730" t="s">
-        <v>627</v>
+        <v>621</v>
       </c>
       <c r="B730" t="s">
-        <v>628</v>
+        <v>622</v>
       </c>
       <c r="C730" t="s">
         <v>619</v>
       </c>
       <c r="D730" t="s">
-        <v>138</v>
+        <v>620</v>
       </c>
       <c r="E730" t="s">
         <v>25</v>
@@ -67497,16 +67727,16 @@
     </row>
     <row r="731" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A731" t="s">
-        <v>629</v>
+        <v>623</v>
       </c>
       <c r="B731" t="s">
-        <v>630</v>
+        <v>624</v>
       </c>
       <c r="C731" t="s">
         <v>619</v>
       </c>
       <c r="D731" t="s">
-        <v>138</v>
+        <v>620</v>
       </c>
       <c r="E731" t="s">
         <v>25</v>
@@ -67535,16 +67765,16 @@
     </row>
     <row r="732" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A732" t="s">
-        <v>631</v>
+        <v>625</v>
       </c>
       <c r="B732" t="s">
-        <v>632</v>
+        <v>626</v>
       </c>
       <c r="C732" t="s">
         <v>619</v>
       </c>
       <c r="D732" t="s">
-        <v>138</v>
+        <v>620</v>
       </c>
       <c r="E732" t="s">
         <v>25</v>
@@ -67573,10 +67803,10 @@
     </row>
     <row r="733" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A733" t="s">
-        <v>633</v>
+        <v>627</v>
       </c>
       <c r="B733" t="s">
-        <v>634</v>
+        <v>628</v>
       </c>
       <c r="C733" t="s">
         <v>619</v>
@@ -67611,16 +67841,16 @@
     </row>
     <row r="734" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A734" t="s">
-        <v>635</v>
+        <v>629</v>
       </c>
       <c r="B734" t="s">
-        <v>636</v>
+        <v>630</v>
       </c>
       <c r="C734" t="s">
         <v>619</v>
       </c>
       <c r="D734" t="s">
-        <v>637</v>
+        <v>138</v>
       </c>
       <c r="E734" t="s">
         <v>25</v>
@@ -67649,16 +67879,16 @@
     </row>
     <row r="735" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A735" t="s">
-        <v>638</v>
+        <v>631</v>
       </c>
       <c r="B735" t="s">
-        <v>639</v>
+        <v>632</v>
       </c>
       <c r="C735" t="s">
         <v>619</v>
       </c>
       <c r="D735" t="s">
-        <v>637</v>
+        <v>138</v>
       </c>
       <c r="E735" t="s">
         <v>25</v>
@@ -67687,16 +67917,16 @@
     </row>
     <row r="736" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A736" t="s">
-        <v>640</v>
+        <v>633</v>
       </c>
       <c r="B736" t="s">
-        <v>641</v>
+        <v>634</v>
       </c>
       <c r="C736" t="s">
         <v>619</v>
       </c>
       <c r="D736" t="s">
-        <v>637</v>
+        <v>138</v>
       </c>
       <c r="E736" t="s">
         <v>25</v>
@@ -67725,10 +67955,10 @@
     </row>
     <row r="737" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A737" t="s">
-        <v>642</v>
+        <v>635</v>
       </c>
       <c r="B737" t="s">
-        <v>643</v>
+        <v>636</v>
       </c>
       <c r="C737" t="s">
         <v>619</v>
@@ -67763,10 +67993,10 @@
     </row>
     <row r="738" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A738" t="s">
-        <v>644</v>
+        <v>638</v>
       </c>
       <c r="B738" t="s">
-        <v>645</v>
+        <v>639</v>
       </c>
       <c r="C738" t="s">
         <v>619</v>
@@ -67801,16 +68031,16 @@
     </row>
     <row r="739" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A739" t="s">
-        <v>646</v>
+        <v>640</v>
       </c>
       <c r="B739" t="s">
-        <v>647</v>
+        <v>641</v>
       </c>
       <c r="C739" t="s">
         <v>619</v>
       </c>
       <c r="D739" t="s">
-        <v>128</v>
+        <v>637</v>
       </c>
       <c r="E739" t="s">
         <v>25</v>
@@ -67839,16 +68069,16 @@
     </row>
     <row r="740" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A740" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="B740" t="s">
-        <v>649</v>
+        <v>643</v>
       </c>
       <c r="C740" t="s">
         <v>619</v>
       </c>
       <c r="D740" t="s">
-        <v>128</v>
+        <v>637</v>
       </c>
       <c r="E740" t="s">
         <v>25</v>
@@ -67877,16 +68107,16 @@
     </row>
     <row r="741" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A741" t="s">
-        <v>650</v>
+        <v>644</v>
       </c>
       <c r="B741" t="s">
-        <v>651</v>
+        <v>645</v>
       </c>
       <c r="C741" t="s">
         <v>619</v>
       </c>
       <c r="D741" t="s">
-        <v>652</v>
+        <v>637</v>
       </c>
       <c r="E741" t="s">
         <v>25</v>
@@ -67915,16 +68145,16 @@
     </row>
     <row r="742" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A742" t="s">
-        <v>653</v>
+        <v>646</v>
       </c>
       <c r="B742" t="s">
-        <v>654</v>
+        <v>647</v>
       </c>
       <c r="C742" t="s">
         <v>619</v>
       </c>
       <c r="D742" t="s">
-        <v>652</v>
+        <v>128</v>
       </c>
       <c r="E742" t="s">
         <v>25</v>
@@ -67953,16 +68183,16 @@
     </row>
     <row r="743" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A743" t="s">
-        <v>655</v>
+        <v>648</v>
       </c>
       <c r="B743" t="s">
-        <v>656</v>
+        <v>649</v>
       </c>
       <c r="C743" t="s">
         <v>619</v>
       </c>
       <c r="D743" t="s">
-        <v>652</v>
+        <v>128</v>
       </c>
       <c r="E743" t="s">
         <v>25</v>
@@ -67991,10 +68221,10 @@
     </row>
     <row r="744" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A744" t="s">
-        <v>655</v>
+        <v>650</v>
       </c>
       <c r="B744" t="s">
-        <v>657</v>
+        <v>651</v>
       </c>
       <c r="C744" t="s">
         <v>619</v>
@@ -68029,16 +68259,16 @@
     </row>
     <row r="745" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A745" t="s">
-        <v>658</v>
+        <v>653</v>
       </c>
       <c r="B745" t="s">
-        <v>659</v>
+        <v>654</v>
       </c>
       <c r="C745" t="s">
-        <v>660</v>
+        <v>619</v>
       </c>
       <c r="D745" t="s">
-        <v>661</v>
+        <v>652</v>
       </c>
       <c r="E745" t="s">
         <v>25</v>
@@ -68067,16 +68297,16 @@
     </row>
     <row r="746" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A746" t="s">
-        <v>662</v>
+        <v>655</v>
       </c>
       <c r="B746" t="s">
-        <v>663</v>
+        <v>656</v>
       </c>
       <c r="C746" t="s">
-        <v>660</v>
+        <v>619</v>
       </c>
       <c r="D746" t="s">
-        <v>661</v>
+        <v>652</v>
       </c>
       <c r="E746" t="s">
         <v>25</v>
@@ -68105,16 +68335,16 @@
     </row>
     <row r="747" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A747" t="s">
-        <v>664</v>
+        <v>655</v>
       </c>
       <c r="B747" t="s">
-        <v>665</v>
+        <v>657</v>
       </c>
       <c r="C747" t="s">
-        <v>660</v>
+        <v>619</v>
       </c>
       <c r="D747" t="s">
-        <v>661</v>
+        <v>652</v>
       </c>
       <c r="E747" t="s">
         <v>25</v>
@@ -68143,10 +68373,10 @@
     </row>
     <row r="748" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A748" t="s">
-        <v>666</v>
+        <v>658</v>
       </c>
       <c r="B748" t="s">
-        <v>667</v>
+        <v>659</v>
       </c>
       <c r="C748" t="s">
         <v>660</v>
@@ -68181,10 +68411,10 @@
     </row>
     <row r="749" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A749" t="s">
-        <v>668</v>
+        <v>662</v>
       </c>
       <c r="B749" t="s">
-        <v>669</v>
+        <v>663</v>
       </c>
       <c r="C749" t="s">
         <v>660</v>
@@ -68219,10 +68449,10 @@
     </row>
     <row r="750" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A750" t="s">
-        <v>670</v>
+        <v>664</v>
       </c>
       <c r="B750" t="s">
-        <v>671</v>
+        <v>665</v>
       </c>
       <c r="C750" t="s">
         <v>660</v>
@@ -68257,16 +68487,16 @@
     </row>
     <row r="751" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A751" t="s">
-        <v>672</v>
+        <v>666</v>
       </c>
       <c r="B751" t="s">
-        <v>673</v>
+        <v>667</v>
       </c>
       <c r="C751" t="s">
         <v>660</v>
       </c>
       <c r="D751" t="s">
-        <v>674</v>
+        <v>661</v>
       </c>
       <c r="E751" t="s">
         <v>25</v>
@@ -68295,16 +68525,16 @@
     </row>
     <row r="752" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A752" t="s">
-        <v>675</v>
+        <v>668</v>
       </c>
       <c r="B752" t="s">
-        <v>676</v>
+        <v>669</v>
       </c>
       <c r="C752" t="s">
         <v>660</v>
       </c>
       <c r="D752" t="s">
-        <v>674</v>
+        <v>661</v>
       </c>
       <c r="E752" t="s">
         <v>25</v>
@@ -68333,16 +68563,16 @@
     </row>
     <row r="753" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A753" t="s">
-        <v>677</v>
+        <v>670</v>
       </c>
       <c r="B753" t="s">
-        <v>678</v>
+        <v>671</v>
       </c>
       <c r="C753" t="s">
         <v>660</v>
       </c>
       <c r="D753" t="s">
-        <v>674</v>
+        <v>661</v>
       </c>
       <c r="E753" t="s">
         <v>25</v>
@@ -68371,16 +68601,16 @@
     </row>
     <row r="754" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A754" t="s">
-        <v>679</v>
+        <v>672</v>
       </c>
       <c r="B754" t="s">
-        <v>680</v>
+        <v>673</v>
       </c>
       <c r="C754" t="s">
         <v>660</v>
       </c>
       <c r="D754" t="s">
-        <v>681</v>
+        <v>674</v>
       </c>
       <c r="E754" t="s">
         <v>25</v>
@@ -68409,16 +68639,16 @@
     </row>
     <row r="755" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A755" t="s">
-        <v>682</v>
+        <v>675</v>
       </c>
       <c r="B755" t="s">
-        <v>683</v>
+        <v>676</v>
       </c>
       <c r="C755" t="s">
         <v>660</v>
       </c>
       <c r="D755" t="s">
-        <v>681</v>
+        <v>674</v>
       </c>
       <c r="E755" t="s">
         <v>25</v>
@@ -68447,16 +68677,16 @@
     </row>
     <row r="756" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A756" t="s">
-        <v>684</v>
+        <v>677</v>
       </c>
       <c r="B756" t="s">
-        <v>685</v>
+        <v>678</v>
       </c>
       <c r="C756" t="s">
         <v>660</v>
       </c>
       <c r="D756" t="s">
-        <v>681</v>
+        <v>674</v>
       </c>
       <c r="E756" t="s">
         <v>25</v>
@@ -68485,10 +68715,10 @@
     </row>
     <row r="757" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A757" t="s">
-        <v>686</v>
+        <v>679</v>
       </c>
       <c r="B757" t="s">
-        <v>687</v>
+        <v>680</v>
       </c>
       <c r="C757" t="s">
         <v>660</v>
@@ -68523,16 +68753,16 @@
     </row>
     <row r="758" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A758" t="s">
-        <v>688</v>
+        <v>682</v>
       </c>
       <c r="B758" t="s">
-        <v>689</v>
+        <v>683</v>
       </c>
       <c r="C758" t="s">
         <v>660</v>
       </c>
       <c r="D758" t="s">
-        <v>690</v>
+        <v>681</v>
       </c>
       <c r="E758" t="s">
         <v>25</v>
@@ -68561,16 +68791,16 @@
     </row>
     <row r="759" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A759" t="s">
-        <v>691</v>
+        <v>684</v>
       </c>
       <c r="B759" t="s">
-        <v>689</v>
+        <v>685</v>
       </c>
       <c r="C759" t="s">
         <v>660</v>
       </c>
       <c r="D759" t="s">
-        <v>690</v>
+        <v>681</v>
       </c>
       <c r="E759" t="s">
         <v>25</v>
@@ -68599,16 +68829,16 @@
     </row>
     <row r="760" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A760" t="s">
-        <v>692</v>
+        <v>686</v>
       </c>
       <c r="B760" t="s">
-        <v>693</v>
+        <v>687</v>
       </c>
       <c r="C760" t="s">
         <v>660</v>
       </c>
       <c r="D760" t="s">
-        <v>690</v>
+        <v>681</v>
       </c>
       <c r="E760" t="s">
         <v>25</v>
@@ -68637,16 +68867,16 @@
     </row>
     <row r="761" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A761" t="s">
-        <v>694</v>
+        <v>688</v>
       </c>
       <c r="B761" t="s">
-        <v>695</v>
+        <v>689</v>
       </c>
       <c r="C761" t="s">
         <v>660</v>
       </c>
       <c r="D761" t="s">
-        <v>696</v>
+        <v>690</v>
       </c>
       <c r="E761" t="s">
         <v>25</v>
@@ -68675,16 +68905,16 @@
     </row>
     <row r="762" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A762" t="s">
-        <v>697</v>
+        <v>691</v>
       </c>
       <c r="B762" t="s">
-        <v>698</v>
+        <v>689</v>
       </c>
       <c r="C762" t="s">
         <v>660</v>
       </c>
       <c r="D762" t="s">
-        <v>696</v>
+        <v>690</v>
       </c>
       <c r="E762" t="s">
         <v>25</v>
@@ -68713,16 +68943,16 @@
     </row>
     <row r="763" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A763" t="s">
-        <v>699</v>
+        <v>692</v>
       </c>
       <c r="B763" t="s">
-        <v>700</v>
+        <v>693</v>
       </c>
       <c r="C763" t="s">
         <v>660</v>
       </c>
       <c r="D763" t="s">
-        <v>696</v>
+        <v>690</v>
       </c>
       <c r="E763" t="s">
         <v>25</v>
@@ -68751,10 +68981,10 @@
     </row>
     <row r="764" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A764" t="s">
-        <v>701</v>
+        <v>694</v>
       </c>
       <c r="B764" t="s">
-        <v>702</v>
+        <v>695</v>
       </c>
       <c r="C764" t="s">
         <v>660</v>
@@ -68789,10 +69019,10 @@
     </row>
     <row r="765" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A765" t="s">
-        <v>703</v>
+        <v>697</v>
       </c>
       <c r="B765" t="s">
-        <v>704</v>
+        <v>698</v>
       </c>
       <c r="C765" t="s">
         <v>660</v>
@@ -68827,16 +69057,16 @@
     </row>
     <row r="766" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A766" t="s">
-        <v>705</v>
+        <v>699</v>
       </c>
       <c r="B766" t="s">
-        <v>706</v>
+        <v>700</v>
       </c>
       <c r="C766" t="s">
         <v>660</v>
       </c>
       <c r="D766" t="s">
-        <v>707</v>
+        <v>696</v>
       </c>
       <c r="E766" t="s">
         <v>25</v>
@@ -68865,16 +69095,16 @@
     </row>
     <row r="767" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A767" t="s">
-        <v>708</v>
+        <v>701</v>
       </c>
       <c r="B767" t="s">
-        <v>709</v>
+        <v>702</v>
       </c>
       <c r="C767" t="s">
         <v>660</v>
       </c>
       <c r="D767" t="s">
-        <v>707</v>
+        <v>696</v>
       </c>
       <c r="E767" t="s">
         <v>25</v>
@@ -68903,16 +69133,16 @@
     </row>
     <row r="768" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A768" t="s">
-        <v>710</v>
+        <v>703</v>
       </c>
       <c r="B768" t="s">
-        <v>711</v>
+        <v>704</v>
       </c>
       <c r="C768" t="s">
         <v>660</v>
       </c>
       <c r="D768" t="s">
-        <v>707</v>
+        <v>696</v>
       </c>
       <c r="E768" t="s">
         <v>25</v>
@@ -68941,10 +69171,10 @@
     </row>
     <row r="769" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A769" t="s">
-        <v>712</v>
+        <v>705</v>
       </c>
       <c r="B769" t="s">
-        <v>713</v>
+        <v>706</v>
       </c>
       <c r="C769" t="s">
         <v>660</v>
@@ -68979,10 +69209,10 @@
     </row>
     <row r="770" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A770" t="s">
-        <v>714</v>
+        <v>708</v>
       </c>
       <c r="B770" t="s">
-        <v>715</v>
+        <v>709</v>
       </c>
       <c r="C770" t="s">
         <v>660</v>
@@ -69017,10 +69247,10 @@
     </row>
     <row r="771" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A771" t="s">
-        <v>716</v>
+        <v>710</v>
       </c>
       <c r="B771" t="s">
-        <v>717</v>
+        <v>711</v>
       </c>
       <c r="C771" t="s">
         <v>660</v>
@@ -69055,16 +69285,16 @@
     </row>
     <row r="772" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A772" t="s">
-        <v>718</v>
+        <v>712</v>
       </c>
       <c r="B772" t="s">
-        <v>719</v>
+        <v>713</v>
       </c>
       <c r="C772" t="s">
         <v>660</v>
       </c>
       <c r="D772" t="s">
-        <v>720</v>
+        <v>707</v>
       </c>
       <c r="E772" t="s">
         <v>25</v>
@@ -69093,16 +69323,16 @@
     </row>
     <row r="773" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A773" t="s">
-        <v>721</v>
+        <v>714</v>
       </c>
       <c r="B773" t="s">
-        <v>722</v>
+        <v>715</v>
       </c>
       <c r="C773" t="s">
         <v>660</v>
       </c>
       <c r="D773" t="s">
-        <v>720</v>
+        <v>707</v>
       </c>
       <c r="E773" t="s">
         <v>25</v>
@@ -69131,16 +69361,16 @@
     </row>
     <row r="774" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A774" t="s">
-        <v>723</v>
+        <v>716</v>
       </c>
       <c r="B774" t="s">
-        <v>724</v>
+        <v>717</v>
       </c>
       <c r="C774" t="s">
-        <v>725</v>
+        <v>660</v>
       </c>
       <c r="D774" t="s">
-        <v>726</v>
+        <v>707</v>
       </c>
       <c r="E774" t="s">
         <v>25</v>
@@ -69169,16 +69399,16 @@
     </row>
     <row r="775" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A775" t="s">
-        <v>727</v>
+        <v>718</v>
       </c>
       <c r="B775" t="s">
-        <v>728</v>
+        <v>719</v>
       </c>
       <c r="C775" t="s">
-        <v>725</v>
+        <v>660</v>
       </c>
       <c r="D775" t="s">
-        <v>726</v>
+        <v>720</v>
       </c>
       <c r="E775" t="s">
         <v>25</v>
@@ -69207,16 +69437,16 @@
     </row>
     <row r="776" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A776" t="s">
-        <v>729</v>
+        <v>721</v>
       </c>
       <c r="B776" t="s">
-        <v>730</v>
+        <v>722</v>
       </c>
       <c r="C776" t="s">
-        <v>725</v>
+        <v>660</v>
       </c>
       <c r="D776" t="s">
-        <v>726</v>
+        <v>720</v>
       </c>
       <c r="E776" t="s">
         <v>25</v>
@@ -69245,10 +69475,10 @@
     </row>
     <row r="777" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A777" t="s">
-        <v>731</v>
+        <v>723</v>
       </c>
       <c r="B777" t="s">
-        <v>732</v>
+        <v>724</v>
       </c>
       <c r="C777" t="s">
         <v>725</v>
@@ -69283,10 +69513,10 @@
     </row>
     <row r="778" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A778" t="s">
-        <v>733</v>
+        <v>727</v>
       </c>
       <c r="B778" t="s">
-        <v>734</v>
+        <v>728</v>
       </c>
       <c r="C778" t="s">
         <v>725</v>
@@ -69321,10 +69551,10 @@
     </row>
     <row r="779" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A779" t="s">
-        <v>735</v>
+        <v>729</v>
       </c>
       <c r="B779" t="s">
-        <v>736</v>
+        <v>730</v>
       </c>
       <c r="C779" t="s">
         <v>725</v>
@@ -69359,10 +69589,10 @@
     </row>
     <row r="780" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A780" t="s">
-        <v>737</v>
+        <v>731</v>
       </c>
       <c r="B780" t="s">
-        <v>738</v>
+        <v>732</v>
       </c>
       <c r="C780" t="s">
         <v>725</v>
@@ -69397,10 +69627,10 @@
     </row>
     <row r="781" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A781" t="s">
-        <v>739</v>
+        <v>733</v>
       </c>
       <c r="B781" t="s">
-        <v>740</v>
+        <v>734</v>
       </c>
       <c r="C781" t="s">
         <v>725</v>
@@ -69435,10 +69665,10 @@
     </row>
     <row r="782" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A782" t="s">
-        <v>741</v>
+        <v>735</v>
       </c>
       <c r="B782" t="s">
-        <v>742</v>
+        <v>736</v>
       </c>
       <c r="C782" t="s">
         <v>725</v>
@@ -69473,10 +69703,10 @@
     </row>
     <row r="783" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A783" t="s">
-        <v>743</v>
+        <v>737</v>
       </c>
       <c r="B783" t="s">
-        <v>744</v>
+        <v>738</v>
       </c>
       <c r="C783" t="s">
         <v>725</v>
@@ -69511,10 +69741,10 @@
     </row>
     <row r="784" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A784" t="s">
-        <v>745</v>
+        <v>739</v>
       </c>
       <c r="B784" t="s">
-        <v>746</v>
+        <v>740</v>
       </c>
       <c r="C784" t="s">
         <v>725</v>
@@ -69549,10 +69779,10 @@
     </row>
     <row r="785" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A785" t="s">
-        <v>747</v>
+        <v>741</v>
       </c>
       <c r="B785" t="s">
-        <v>748</v>
+        <v>742</v>
       </c>
       <c r="C785" t="s">
         <v>725</v>
@@ -69587,10 +69817,10 @@
     </row>
     <row r="786" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A786" t="s">
-        <v>749</v>
+        <v>743</v>
       </c>
       <c r="B786" t="s">
-        <v>750</v>
+        <v>744</v>
       </c>
       <c r="C786" t="s">
         <v>725</v>
@@ -69625,16 +69855,16 @@
     </row>
     <row r="787" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A787" t="s">
-        <v>751</v>
+        <v>745</v>
       </c>
       <c r="B787" t="s">
-        <v>752</v>
+        <v>746</v>
       </c>
       <c r="C787" t="s">
         <v>725</v>
       </c>
       <c r="D787" t="s">
-        <v>753</v>
+        <v>726</v>
       </c>
       <c r="E787" t="s">
         <v>25</v>
@@ -69663,16 +69893,16 @@
     </row>
     <row r="788" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A788" t="s">
-        <v>754</v>
+        <v>747</v>
       </c>
       <c r="B788" t="s">
-        <v>755</v>
+        <v>748</v>
       </c>
       <c r="C788" t="s">
         <v>725</v>
       </c>
       <c r="D788" t="s">
-        <v>753</v>
+        <v>726</v>
       </c>
       <c r="E788" t="s">
         <v>25</v>
@@ -69701,16 +69931,16 @@
     </row>
     <row r="789" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A789" t="s">
-        <v>756</v>
+        <v>749</v>
       </c>
       <c r="B789" t="s">
-        <v>757</v>
+        <v>750</v>
       </c>
       <c r="C789" t="s">
         <v>725</v>
       </c>
       <c r="D789" t="s">
-        <v>753</v>
+        <v>726</v>
       </c>
       <c r="E789" t="s">
         <v>25</v>
@@ -69739,10 +69969,10 @@
     </row>
     <row r="790" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A790" t="s">
-        <v>758</v>
+        <v>751</v>
       </c>
       <c r="B790" t="s">
-        <v>759</v>
+        <v>752</v>
       </c>
       <c r="C790" t="s">
         <v>725</v>
@@ -69777,10 +70007,10 @@
     </row>
     <row r="791" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A791" t="s">
-        <v>760</v>
+        <v>754</v>
       </c>
       <c r="B791" t="s">
-        <v>761</v>
+        <v>755</v>
       </c>
       <c r="C791" t="s">
         <v>725</v>
@@ -69815,16 +70045,16 @@
     </row>
     <row r="792" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A792" t="s">
-        <v>762</v>
+        <v>756</v>
       </c>
       <c r="B792" t="s">
-        <v>763</v>
+        <v>757</v>
       </c>
       <c r="C792" t="s">
         <v>725</v>
       </c>
       <c r="D792" t="s">
-        <v>196</v>
+        <v>753</v>
       </c>
       <c r="E792" t="s">
         <v>25</v>
@@ -69853,16 +70083,16 @@
     </row>
     <row r="793" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A793" t="s">
-        <v>764</v>
+        <v>758</v>
       </c>
       <c r="B793" t="s">
-        <v>765</v>
+        <v>759</v>
       </c>
       <c r="C793" t="s">
         <v>725</v>
       </c>
       <c r="D793" t="s">
-        <v>196</v>
+        <v>753</v>
       </c>
       <c r="E793" t="s">
         <v>25</v>
@@ -69891,16 +70121,16 @@
     </row>
     <row r="794" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A794" t="s">
-        <v>766</v>
+        <v>760</v>
       </c>
       <c r="B794" t="s">
-        <v>767</v>
+        <v>761</v>
       </c>
       <c r="C794" t="s">
         <v>725</v>
       </c>
       <c r="D794" t="s">
-        <v>196</v>
+        <v>753</v>
       </c>
       <c r="E794" t="s">
         <v>25</v>
@@ -69929,16 +70159,16 @@
     </row>
     <row r="795" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A795" t="s">
-        <v>768</v>
+        <v>762</v>
       </c>
       <c r="B795" t="s">
-        <v>769</v>
+        <v>763</v>
       </c>
       <c r="C795" t="s">
         <v>725</v>
       </c>
       <c r="D795" t="s">
-        <v>770</v>
+        <v>196</v>
       </c>
       <c r="E795" t="s">
         <v>25</v>
@@ -69967,16 +70197,16 @@
     </row>
     <row r="796" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A796" t="s">
-        <v>771</v>
+        <v>764</v>
       </c>
       <c r="B796" t="s">
-        <v>772</v>
+        <v>765</v>
       </c>
       <c r="C796" t="s">
         <v>725</v>
       </c>
       <c r="D796" t="s">
-        <v>770</v>
+        <v>196</v>
       </c>
       <c r="E796" t="s">
         <v>25</v>
@@ -70005,16 +70235,16 @@
     </row>
     <row r="797" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A797" t="s">
-        <v>773</v>
+        <v>766</v>
       </c>
       <c r="B797" t="s">
-        <v>774</v>
+        <v>767</v>
       </c>
       <c r="C797" t="s">
         <v>725</v>
       </c>
       <c r="D797" t="s">
-        <v>775</v>
+        <v>196</v>
       </c>
       <c r="E797" t="s">
         <v>25</v>
@@ -70043,16 +70273,16 @@
     </row>
     <row r="798" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A798" t="s">
-        <v>776</v>
+        <v>768</v>
       </c>
       <c r="B798" t="s">
-        <v>777</v>
+        <v>769</v>
       </c>
       <c r="C798" t="s">
         <v>725</v>
       </c>
       <c r="D798" t="s">
-        <v>775</v>
+        <v>770</v>
       </c>
       <c r="E798" t="s">
         <v>25</v>
@@ -70081,16 +70311,16 @@
     </row>
     <row r="799" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A799" t="s">
-        <v>778</v>
+        <v>771</v>
       </c>
       <c r="B799" t="s">
-        <v>779</v>
+        <v>772</v>
       </c>
       <c r="C799" t="s">
         <v>725</v>
       </c>
       <c r="D799" t="s">
-        <v>775</v>
+        <v>770</v>
       </c>
       <c r="E799" t="s">
         <v>25</v>
@@ -70119,16 +70349,16 @@
     </row>
     <row r="800" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A800" t="s">
-        <v>780</v>
+        <v>773</v>
       </c>
       <c r="B800" t="s">
-        <v>781</v>
+        <v>774</v>
       </c>
       <c r="C800" t="s">
         <v>725</v>
       </c>
       <c r="D800" t="s">
-        <v>782</v>
+        <v>775</v>
       </c>
       <c r="E800" t="s">
         <v>25</v>
@@ -70157,16 +70387,16 @@
     </row>
     <row r="801" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A801" t="s">
-        <v>783</v>
+        <v>776</v>
       </c>
       <c r="B801" t="s">
-        <v>784</v>
+        <v>777</v>
       </c>
       <c r="C801" t="s">
         <v>725</v>
       </c>
       <c r="D801" t="s">
-        <v>782</v>
+        <v>775</v>
       </c>
       <c r="E801" t="s">
         <v>25</v>
@@ -70195,16 +70425,16 @@
     </row>
     <row r="802" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A802" t="s">
-        <v>785</v>
+        <v>778</v>
       </c>
       <c r="B802" t="s">
-        <v>786</v>
+        <v>779</v>
       </c>
       <c r="C802" t="s">
         <v>725</v>
       </c>
       <c r="D802" t="s">
-        <v>782</v>
+        <v>775</v>
       </c>
       <c r="E802" t="s">
         <v>25</v>
@@ -70233,10 +70463,10 @@
     </row>
     <row r="803" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A803" t="s">
-        <v>787</v>
+        <v>780</v>
       </c>
       <c r="B803" t="s">
-        <v>788</v>
+        <v>781</v>
       </c>
       <c r="C803" t="s">
         <v>725</v>
@@ -70271,10 +70501,10 @@
     </row>
     <row r="804" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A804" t="s">
-        <v>789</v>
+        <v>783</v>
       </c>
       <c r="B804" t="s">
-        <v>790</v>
+        <v>784</v>
       </c>
       <c r="C804" t="s">
         <v>725</v>
@@ -70309,10 +70539,10 @@
     </row>
     <row r="805" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A805" t="s">
-        <v>791</v>
+        <v>785</v>
       </c>
       <c r="B805" t="s">
-        <v>792</v>
+        <v>786</v>
       </c>
       <c r="C805" t="s">
         <v>725</v>
@@ -70347,10 +70577,10 @@
     </row>
     <row r="806" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A806" t="s">
-        <v>793</v>
+        <v>787</v>
       </c>
       <c r="B806" t="s">
-        <v>794</v>
+        <v>788</v>
       </c>
       <c r="C806" t="s">
         <v>725</v>
@@ -70385,10 +70615,10 @@
     </row>
     <row r="807" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A807" t="s">
-        <v>795</v>
+        <v>789</v>
       </c>
       <c r="B807" t="s">
-        <v>796</v>
+        <v>790</v>
       </c>
       <c r="C807" t="s">
         <v>725</v>
@@ -70423,10 +70653,10 @@
     </row>
     <row r="808" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A808" t="s">
-        <v>797</v>
+        <v>791</v>
       </c>
       <c r="B808" t="s">
-        <v>798</v>
+        <v>792</v>
       </c>
       <c r="C808" t="s">
         <v>725</v>
@@ -70461,10 +70691,10 @@
     </row>
     <row r="809" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A809" t="s">
-        <v>799</v>
+        <v>793</v>
       </c>
       <c r="B809" t="s">
-        <v>800</v>
+        <v>794</v>
       </c>
       <c r="C809" t="s">
         <v>725</v>
@@ -70499,10 +70729,10 @@
     </row>
     <row r="810" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A810" t="s">
-        <v>801</v>
+        <v>795</v>
       </c>
       <c r="B810" t="s">
-        <v>802</v>
+        <v>796</v>
       </c>
       <c r="C810" t="s">
         <v>725</v>
@@ -70537,10 +70767,10 @@
     </row>
     <row r="811" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A811" t="s">
-        <v>803</v>
+        <v>797</v>
       </c>
       <c r="B811" t="s">
-        <v>804</v>
+        <v>798</v>
       </c>
       <c r="C811" t="s">
         <v>725</v>
@@ -70575,16 +70805,16 @@
     </row>
     <row r="812" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A812" t="s">
-        <v>805</v>
+        <v>799</v>
       </c>
       <c r="B812" t="s">
-        <v>806</v>
+        <v>800</v>
       </c>
       <c r="C812" t="s">
         <v>725</v>
       </c>
       <c r="D812" t="s">
-        <v>807</v>
+        <v>782</v>
       </c>
       <c r="E812" t="s">
         <v>25</v>
@@ -70613,16 +70843,16 @@
     </row>
     <row r="813" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A813" t="s">
-        <v>808</v>
+        <v>801</v>
       </c>
       <c r="B813" t="s">
-        <v>809</v>
+        <v>802</v>
       </c>
       <c r="C813" t="s">
         <v>725</v>
       </c>
       <c r="D813" t="s">
-        <v>807</v>
+        <v>782</v>
       </c>
       <c r="E813" t="s">
         <v>25</v>
@@ -70651,16 +70881,16 @@
     </row>
     <row r="814" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A814" t="s">
-        <v>810</v>
+        <v>803</v>
       </c>
       <c r="B814" t="s">
-        <v>811</v>
+        <v>804</v>
       </c>
       <c r="C814" t="s">
         <v>725</v>
       </c>
       <c r="D814" t="s">
-        <v>807</v>
+        <v>782</v>
       </c>
       <c r="E814" t="s">
         <v>25</v>
@@ -70689,10 +70919,10 @@
     </row>
     <row r="815" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A815" t="s">
-        <v>812</v>
+        <v>805</v>
       </c>
       <c r="B815" t="s">
-        <v>813</v>
+        <v>806</v>
       </c>
       <c r="C815" t="s">
         <v>725</v>
@@ -70727,10 +70957,10 @@
     </row>
     <row r="816" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A816" t="s">
-        <v>814</v>
+        <v>808</v>
       </c>
       <c r="B816" t="s">
-        <v>815</v>
+        <v>809</v>
       </c>
       <c r="C816" t="s">
         <v>725</v>
@@ -70765,16 +70995,16 @@
     </row>
     <row r="817" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A817" t="s">
-        <v>816</v>
+        <v>810</v>
       </c>
       <c r="B817" t="s">
-        <v>817</v>
+        <v>811</v>
       </c>
       <c r="C817" t="s">
         <v>725</v>
       </c>
       <c r="D817" t="s">
-        <v>818</v>
+        <v>807</v>
       </c>
       <c r="E817" t="s">
         <v>25</v>
@@ -70803,16 +71033,16 @@
     </row>
     <row r="818" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A818" t="s">
-        <v>819</v>
+        <v>812</v>
       </c>
       <c r="B818" t="s">
-        <v>820</v>
+        <v>813</v>
       </c>
       <c r="C818" t="s">
         <v>725</v>
       </c>
       <c r="D818" t="s">
-        <v>818</v>
+        <v>807</v>
       </c>
       <c r="E818" t="s">
         <v>25</v>
@@ -70841,16 +71071,16 @@
     </row>
     <row r="819" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A819" t="s">
-        <v>821</v>
+        <v>814</v>
       </c>
       <c r="B819" t="s">
-        <v>822</v>
+        <v>815</v>
       </c>
       <c r="C819" t="s">
-        <v>823</v>
+        <v>725</v>
       </c>
       <c r="D819" t="s">
-        <v>824</v>
+        <v>807</v>
       </c>
       <c r="E819" t="s">
         <v>25</v>
@@ -70879,16 +71109,16 @@
     </row>
     <row r="820" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A820" t="s">
-        <v>825</v>
+        <v>816</v>
       </c>
       <c r="B820" t="s">
-        <v>826</v>
+        <v>817</v>
       </c>
       <c r="C820" t="s">
-        <v>823</v>
+        <v>725</v>
       </c>
       <c r="D820" t="s">
-        <v>824</v>
+        <v>818</v>
       </c>
       <c r="E820" t="s">
         <v>25</v>
@@ -70917,16 +71147,16 @@
     </row>
     <row r="821" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A821" t="s">
-        <v>827</v>
+        <v>819</v>
       </c>
       <c r="B821" t="s">
-        <v>828</v>
+        <v>820</v>
       </c>
       <c r="C821" t="s">
-        <v>823</v>
+        <v>725</v>
       </c>
       <c r="D821" t="s">
-        <v>824</v>
+        <v>818</v>
       </c>
       <c r="E821" t="s">
         <v>25</v>
@@ -70955,10 +71185,10 @@
     </row>
     <row r="822" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A822" t="s">
-        <v>829</v>
+        <v>821</v>
       </c>
       <c r="B822" t="s">
-        <v>830</v>
+        <v>822</v>
       </c>
       <c r="C822" t="s">
         <v>823</v>
@@ -70993,10 +71223,10 @@
     </row>
     <row r="823" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A823" t="s">
-        <v>831</v>
+        <v>825</v>
       </c>
       <c r="B823" t="s">
-        <v>832</v>
+        <v>826</v>
       </c>
       <c r="C823" t="s">
         <v>823</v>
@@ -71031,10 +71261,10 @@
     </row>
     <row r="824" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A824" t="s">
-        <v>833</v>
+        <v>827</v>
       </c>
       <c r="B824" t="s">
-        <v>834</v>
+        <v>828</v>
       </c>
       <c r="C824" t="s">
         <v>823</v>
@@ -71069,16 +71299,16 @@
     </row>
     <row r="825" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A825" t="s">
-        <v>835</v>
+        <v>829</v>
       </c>
       <c r="B825" t="s">
-        <v>836</v>
+        <v>830</v>
       </c>
       <c r="C825" t="s">
         <v>823</v>
       </c>
       <c r="D825" t="s">
-        <v>837</v>
+        <v>824</v>
       </c>
       <c r="E825" t="s">
         <v>25</v>
@@ -71107,16 +71337,16 @@
     </row>
     <row r="826" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A826" t="s">
-        <v>838</v>
+        <v>831</v>
       </c>
       <c r="B826" t="s">
-        <v>839</v>
+        <v>832</v>
       </c>
       <c r="C826" t="s">
         <v>823</v>
       </c>
       <c r="D826" t="s">
-        <v>837</v>
+        <v>824</v>
       </c>
       <c r="E826" t="s">
         <v>25</v>
@@ -71145,16 +71375,16 @@
     </row>
     <row r="827" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A827" t="s">
-        <v>840</v>
+        <v>833</v>
       </c>
       <c r="B827" t="s">
-        <v>841</v>
+        <v>834</v>
       </c>
       <c r="C827" t="s">
         <v>823</v>
       </c>
       <c r="D827" t="s">
-        <v>837</v>
+        <v>824</v>
       </c>
       <c r="E827" t="s">
         <v>25</v>
@@ -71183,10 +71413,10 @@
     </row>
     <row r="828" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A828" t="s">
-        <v>842</v>
+        <v>835</v>
       </c>
       <c r="B828" t="s">
-        <v>843</v>
+        <v>836</v>
       </c>
       <c r="C828" t="s">
         <v>823</v>
@@ -71221,10 +71451,10 @@
     </row>
     <row r="829" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A829" t="s">
-        <v>844</v>
+        <v>838</v>
       </c>
       <c r="B829" t="s">
-        <v>845</v>
+        <v>839</v>
       </c>
       <c r="C829" t="s">
         <v>823</v>
@@ -71259,16 +71489,16 @@
     </row>
     <row r="830" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A830" t="s">
-        <v>846</v>
+        <v>840</v>
       </c>
       <c r="B830" t="s">
-        <v>847</v>
+        <v>841</v>
       </c>
       <c r="C830" t="s">
         <v>823</v>
       </c>
       <c r="D830" t="s">
-        <v>848</v>
+        <v>837</v>
       </c>
       <c r="E830" t="s">
         <v>25</v>
@@ -71297,16 +71527,16 @@
     </row>
     <row r="831" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A831" t="s">
-        <v>849</v>
+        <v>842</v>
       </c>
       <c r="B831" t="s">
-        <v>850</v>
+        <v>843</v>
       </c>
       <c r="C831" t="s">
         <v>823</v>
       </c>
       <c r="D831" t="s">
-        <v>848</v>
+        <v>837</v>
       </c>
       <c r="E831" t="s">
         <v>25</v>
@@ -71335,16 +71565,16 @@
     </row>
     <row r="832" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A832" t="s">
-        <v>851</v>
+        <v>844</v>
       </c>
       <c r="B832" t="s">
-        <v>852</v>
+        <v>845</v>
       </c>
       <c r="C832" t="s">
         <v>823</v>
       </c>
       <c r="D832" t="s">
-        <v>848</v>
+        <v>837</v>
       </c>
       <c r="E832" t="s">
         <v>25</v>
@@ -71373,16 +71603,16 @@
     </row>
     <row r="833" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A833" t="s">
-        <v>853</v>
+        <v>846</v>
       </c>
       <c r="B833" t="s">
-        <v>854</v>
+        <v>847</v>
       </c>
       <c r="C833" t="s">
         <v>823</v>
       </c>
       <c r="D833" t="s">
-        <v>855</v>
+        <v>848</v>
       </c>
       <c r="E833" t="s">
         <v>25</v>
@@ -71411,16 +71641,16 @@
     </row>
     <row r="834" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A834" t="s">
-        <v>856</v>
+        <v>849</v>
       </c>
       <c r="B834" t="s">
-        <v>857</v>
+        <v>850</v>
       </c>
       <c r="C834" t="s">
         <v>823</v>
       </c>
       <c r="D834" t="s">
-        <v>855</v>
+        <v>848</v>
       </c>
       <c r="E834" t="s">
         <v>25</v>
@@ -71449,16 +71679,16 @@
     </row>
     <row r="835" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A835" t="s">
-        <v>858</v>
+        <v>851</v>
       </c>
       <c r="B835" t="s">
-        <v>859</v>
+        <v>852</v>
       </c>
       <c r="C835" t="s">
         <v>823</v>
       </c>
       <c r="D835" t="s">
-        <v>860</v>
+        <v>848</v>
       </c>
       <c r="E835" t="s">
         <v>25</v>
@@ -71487,16 +71717,16 @@
     </row>
     <row r="836" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A836" t="s">
-        <v>861</v>
+        <v>853</v>
       </c>
       <c r="B836" t="s">
-        <v>862</v>
+        <v>854</v>
       </c>
       <c r="C836" t="s">
         <v>823</v>
       </c>
       <c r="D836" t="s">
-        <v>860</v>
+        <v>855</v>
       </c>
       <c r="E836" t="s">
         <v>25</v>
@@ -71525,16 +71755,16 @@
     </row>
     <row r="837" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A837" t="s">
-        <v>863</v>
+        <v>856</v>
       </c>
       <c r="B837" t="s">
-        <v>864</v>
+        <v>857</v>
       </c>
       <c r="C837" t="s">
         <v>823</v>
       </c>
       <c r="D837" t="s">
-        <v>860</v>
+        <v>855</v>
       </c>
       <c r="E837" t="s">
         <v>25</v>
@@ -71563,10 +71793,10 @@
     </row>
     <row r="838" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A838" t="s">
-        <v>865</v>
+        <v>858</v>
       </c>
       <c r="B838" t="s">
-        <v>866</v>
+        <v>859</v>
       </c>
       <c r="C838" t="s">
         <v>823</v>
@@ -71601,16 +71831,16 @@
     </row>
     <row r="839" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A839" t="s">
-        <v>867</v>
+        <v>861</v>
       </c>
       <c r="B839" t="s">
-        <v>868</v>
+        <v>862</v>
       </c>
       <c r="C839" t="s">
         <v>823</v>
       </c>
       <c r="D839" t="s">
-        <v>869</v>
+        <v>860</v>
       </c>
       <c r="E839" t="s">
         <v>25</v>
@@ -71639,16 +71869,16 @@
     </row>
     <row r="840" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A840" t="s">
-        <v>870</v>
+        <v>863</v>
       </c>
       <c r="B840" t="s">
-        <v>871</v>
+        <v>864</v>
       </c>
       <c r="C840" t="s">
         <v>823</v>
       </c>
       <c r="D840" t="s">
-        <v>869</v>
+        <v>860</v>
       </c>
       <c r="E840" t="s">
         <v>25</v>
@@ -71677,16 +71907,16 @@
     </row>
     <row r="841" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A841" t="s">
-        <v>872</v>
+        <v>865</v>
       </c>
       <c r="B841" t="s">
-        <v>873</v>
+        <v>866</v>
       </c>
       <c r="C841" t="s">
         <v>823</v>
       </c>
       <c r="D841" t="s">
-        <v>869</v>
+        <v>860</v>
       </c>
       <c r="E841" t="s">
         <v>25</v>
@@ -71715,10 +71945,10 @@
     </row>
     <row r="842" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A842" t="s">
-        <v>874</v>
+        <v>867</v>
       </c>
       <c r="B842" t="s">
-        <v>875</v>
+        <v>868</v>
       </c>
       <c r="C842" t="s">
         <v>823</v>
@@ -71753,10 +71983,10 @@
     </row>
     <row r="843" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A843" t="s">
-        <v>876</v>
+        <v>870</v>
       </c>
       <c r="B843" t="s">
-        <v>877</v>
+        <v>871</v>
       </c>
       <c r="C843" t="s">
         <v>823</v>
@@ -71791,16 +72021,16 @@
     </row>
     <row r="844" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A844" t="s">
-        <v>878</v>
+        <v>872</v>
       </c>
       <c r="B844" t="s">
-        <v>879</v>
+        <v>873</v>
       </c>
       <c r="C844" t="s">
-        <v>880</v>
+        <v>823</v>
       </c>
       <c r="D844" t="s">
-        <v>25</v>
+        <v>869</v>
       </c>
       <c r="E844" t="s">
         <v>25</v>
@@ -71829,16 +72059,16 @@
     </row>
     <row r="845" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A845" t="s">
-        <v>881</v>
+        <v>874</v>
       </c>
       <c r="B845" t="s">
-        <v>882</v>
+        <v>875</v>
       </c>
       <c r="C845" t="s">
-        <v>880</v>
+        <v>823</v>
       </c>
       <c r="D845" t="s">
-        <v>25</v>
+        <v>869</v>
       </c>
       <c r="E845" t="s">
         <v>25</v>
@@ -71867,16 +72097,16 @@
     </row>
     <row r="846" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A846" t="s">
-        <v>883</v>
+        <v>876</v>
       </c>
       <c r="B846" t="s">
-        <v>884</v>
+        <v>877</v>
       </c>
       <c r="C846" t="s">
-        <v>880</v>
+        <v>823</v>
       </c>
       <c r="D846" t="s">
-        <v>25</v>
+        <v>869</v>
       </c>
       <c r="E846" t="s">
         <v>25</v>
@@ -71905,10 +72135,10 @@
     </row>
     <row r="847" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A847" t="s">
-        <v>885</v>
+        <v>878</v>
       </c>
       <c r="B847" t="s">
-        <v>886</v>
+        <v>879</v>
       </c>
       <c r="C847" t="s">
         <v>880</v>
@@ -71943,10 +72173,10 @@
     </row>
     <row r="848" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A848" t="s">
-        <v>887</v>
+        <v>881</v>
       </c>
       <c r="B848" t="s">
-        <v>888</v>
+        <v>882</v>
       </c>
       <c r="C848" t="s">
         <v>880</v>
@@ -71981,10 +72211,10 @@
     </row>
     <row r="849" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A849" t="s">
-        <v>889</v>
+        <v>883</v>
       </c>
       <c r="B849" t="s">
-        <v>890</v>
+        <v>884</v>
       </c>
       <c r="C849" t="s">
         <v>880</v>
@@ -72019,10 +72249,10 @@
     </row>
     <row r="850" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A850" t="s">
-        <v>891</v>
+        <v>885</v>
       </c>
       <c r="B850" t="s">
-        <v>892</v>
+        <v>886</v>
       </c>
       <c r="C850" t="s">
         <v>880</v>
@@ -72057,10 +72287,10 @@
     </row>
     <row r="851" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A851" t="s">
-        <v>893</v>
+        <v>887</v>
       </c>
       <c r="B851" t="s">
-        <v>894</v>
+        <v>888</v>
       </c>
       <c r="C851" t="s">
         <v>880</v>
@@ -72095,10 +72325,10 @@
     </row>
     <row r="852" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A852" t="s">
-        <v>895</v>
+        <v>889</v>
       </c>
       <c r="B852" t="s">
-        <v>896</v>
+        <v>890</v>
       </c>
       <c r="C852" t="s">
         <v>880</v>
@@ -72133,10 +72363,10 @@
     </row>
     <row r="853" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A853" t="s">
-        <v>897</v>
+        <v>891</v>
       </c>
       <c r="B853" t="s">
-        <v>898</v>
+        <v>892</v>
       </c>
       <c r="C853" t="s">
         <v>880</v>
@@ -72171,10 +72401,10 @@
     </row>
     <row r="854" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A854" t="s">
-        <v>899</v>
+        <v>893</v>
       </c>
       <c r="B854" t="s">
-        <v>900</v>
+        <v>894</v>
       </c>
       <c r="C854" t="s">
         <v>880</v>
@@ -72209,10 +72439,10 @@
     </row>
     <row r="855" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A855" t="s">
-        <v>901</v>
+        <v>895</v>
       </c>
       <c r="B855" t="s">
-        <v>902</v>
+        <v>896</v>
       </c>
       <c r="C855" t="s">
         <v>880</v>
@@ -72247,10 +72477,10 @@
     </row>
     <row r="856" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A856" t="s">
-        <v>903</v>
+        <v>897</v>
       </c>
       <c r="B856" t="s">
-        <v>904</v>
+        <v>898</v>
       </c>
       <c r="C856" t="s">
         <v>880</v>
@@ -72285,10 +72515,10 @@
     </row>
     <row r="857" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A857" t="s">
-        <v>905</v>
+        <v>899</v>
       </c>
       <c r="B857" t="s">
-        <v>906</v>
+        <v>900</v>
       </c>
       <c r="C857" t="s">
         <v>880</v>
@@ -72323,10 +72553,10 @@
     </row>
     <row r="858" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A858" t="s">
-        <v>907</v>
+        <v>901</v>
       </c>
       <c r="B858" t="s">
-        <v>908</v>
+        <v>902</v>
       </c>
       <c r="C858" t="s">
         <v>880</v>
@@ -72361,16 +72591,16 @@
     </row>
     <row r="859" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A859" t="s">
-        <v>909</v>
+        <v>903</v>
       </c>
       <c r="B859" t="s">
-        <v>910</v>
+        <v>904</v>
       </c>
       <c r="C859" t="s">
-        <v>911</v>
+        <v>880</v>
       </c>
       <c r="D859" t="s">
-        <v>912</v>
+        <v>25</v>
       </c>
       <c r="E859" t="s">
         <v>25</v>
@@ -72399,16 +72629,16 @@
     </row>
     <row r="860" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A860" t="s">
-        <v>913</v>
+        <v>905</v>
       </c>
       <c r="B860" t="s">
-        <v>914</v>
+        <v>906</v>
       </c>
       <c r="C860" t="s">
-        <v>911</v>
+        <v>880</v>
       </c>
       <c r="D860" t="s">
-        <v>912</v>
+        <v>25</v>
       </c>
       <c r="E860" t="s">
         <v>25</v>
@@ -72437,16 +72667,16 @@
     </row>
     <row r="861" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A861" t="s">
-        <v>915</v>
+        <v>907</v>
       </c>
       <c r="B861" t="s">
-        <v>916</v>
+        <v>908</v>
       </c>
       <c r="C861" t="s">
-        <v>911</v>
+        <v>880</v>
       </c>
       <c r="D861" t="s">
-        <v>912</v>
+        <v>25</v>
       </c>
       <c r="E861" t="s">
         <v>25</v>
@@ -72475,10 +72705,10 @@
     </row>
     <row r="862" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A862" t="s">
-        <v>917</v>
+        <v>909</v>
       </c>
       <c r="B862" t="s">
-        <v>918</v>
+        <v>910</v>
       </c>
       <c r="C862" t="s">
         <v>911</v>
@@ -72513,16 +72743,16 @@
     </row>
     <row r="863" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A863" t="s">
-        <v>919</v>
+        <v>913</v>
       </c>
       <c r="B863" t="s">
-        <v>920</v>
+        <v>914</v>
       </c>
       <c r="C863" t="s">
         <v>911</v>
       </c>
       <c r="D863" t="s">
-        <v>921</v>
+        <v>912</v>
       </c>
       <c r="E863" t="s">
         <v>25</v>
@@ -72551,16 +72781,16 @@
     </row>
     <row r="864" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A864" t="s">
-        <v>922</v>
+        <v>915</v>
       </c>
       <c r="B864" t="s">
-        <v>923</v>
+        <v>916</v>
       </c>
       <c r="C864" t="s">
         <v>911</v>
       </c>
       <c r="D864" t="s">
-        <v>921</v>
+        <v>912</v>
       </c>
       <c r="E864" t="s">
         <v>25</v>
@@ -72589,16 +72819,16 @@
     </row>
     <row r="865" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A865" t="s">
-        <v>924</v>
+        <v>917</v>
       </c>
       <c r="B865" t="s">
-        <v>925</v>
+        <v>918</v>
       </c>
       <c r="C865" t="s">
         <v>911</v>
       </c>
       <c r="D865" t="s">
-        <v>921</v>
+        <v>912</v>
       </c>
       <c r="E865" t="s">
         <v>25</v>
@@ -72627,10 +72857,10 @@
     </row>
     <row r="866" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A866" t="s">
-        <v>926</v>
+        <v>919</v>
       </c>
       <c r="B866" t="s">
-        <v>927</v>
+        <v>920</v>
       </c>
       <c r="C866" t="s">
         <v>911</v>
@@ -72665,10 +72895,10 @@
     </row>
     <row r="867" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A867" t="s">
-        <v>928</v>
+        <v>922</v>
       </c>
       <c r="B867" t="s">
-        <v>929</v>
+        <v>923</v>
       </c>
       <c r="C867" t="s">
         <v>911</v>
@@ -72703,10 +72933,10 @@
     </row>
     <row r="868" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A868" t="s">
-        <v>930</v>
+        <v>924</v>
       </c>
       <c r="B868" t="s">
-        <v>931</v>
+        <v>925</v>
       </c>
       <c r="C868" t="s">
         <v>911</v>
@@ -72741,10 +72971,10 @@
     </row>
     <row r="869" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A869" t="s">
-        <v>932</v>
+        <v>926</v>
       </c>
       <c r="B869" t="s">
-        <v>933</v>
+        <v>927</v>
       </c>
       <c r="C869" t="s">
         <v>911</v>
@@ -72779,16 +73009,16 @@
     </row>
     <row r="870" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A870" t="s">
-        <v>934</v>
+        <v>928</v>
       </c>
       <c r="B870" t="s">
-        <v>935</v>
+        <v>929</v>
       </c>
       <c r="C870" t="s">
-        <v>936</v>
+        <v>911</v>
       </c>
       <c r="D870" t="s">
-        <v>937</v>
+        <v>921</v>
       </c>
       <c r="E870" t="s">
         <v>25</v>
@@ -72817,16 +73047,16 @@
     </row>
     <row r="871" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A871" t="s">
-        <v>938</v>
+        <v>930</v>
       </c>
       <c r="B871" t="s">
-        <v>939</v>
+        <v>931</v>
       </c>
       <c r="C871" t="s">
-        <v>936</v>
+        <v>911</v>
       </c>
       <c r="D871" t="s">
-        <v>937</v>
+        <v>921</v>
       </c>
       <c r="E871" t="s">
         <v>25</v>
@@ -72855,16 +73085,16 @@
     </row>
     <row r="872" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A872" t="s">
-        <v>940</v>
+        <v>932</v>
       </c>
       <c r="B872" t="s">
-        <v>941</v>
+        <v>933</v>
       </c>
       <c r="C872" t="s">
-        <v>936</v>
+        <v>911</v>
       </c>
       <c r="D872" t="s">
-        <v>937</v>
+        <v>921</v>
       </c>
       <c r="E872" t="s">
         <v>25</v>
@@ -72893,10 +73123,10 @@
     </row>
     <row r="873" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A873" t="s">
-        <v>942</v>
+        <v>934</v>
       </c>
       <c r="B873" t="s">
-        <v>943</v>
+        <v>935</v>
       </c>
       <c r="C873" t="s">
         <v>936</v>
@@ -72931,10 +73161,10 @@
     </row>
     <row r="874" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A874" t="s">
-        <v>944</v>
+        <v>938</v>
       </c>
       <c r="B874" t="s">
-        <v>945</v>
+        <v>939</v>
       </c>
       <c r="C874" t="s">
         <v>936</v>
@@ -72969,10 +73199,10 @@
     </row>
     <row r="875" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A875" t="s">
-        <v>946</v>
+        <v>940</v>
       </c>
       <c r="B875" t="s">
-        <v>947</v>
+        <v>941</v>
       </c>
       <c r="C875" t="s">
         <v>936</v>
@@ -73007,10 +73237,10 @@
     </row>
     <row r="876" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A876" t="s">
-        <v>948</v>
+        <v>942</v>
       </c>
       <c r="B876" t="s">
-        <v>949</v>
+        <v>943</v>
       </c>
       <c r="C876" t="s">
         <v>936</v>
@@ -73045,10 +73275,10 @@
     </row>
     <row r="877" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A877" t="s">
-        <v>950</v>
+        <v>944</v>
       </c>
       <c r="B877" t="s">
-        <v>951</v>
+        <v>945</v>
       </c>
       <c r="C877" t="s">
         <v>936</v>
@@ -73083,16 +73313,16 @@
     </row>
     <row r="878" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A878" t="s">
-        <v>952</v>
+        <v>946</v>
       </c>
       <c r="B878" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
       <c r="C878" t="s">
         <v>936</v>
       </c>
       <c r="D878" t="s">
-        <v>954</v>
+        <v>937</v>
       </c>
       <c r="E878" t="s">
         <v>25</v>
@@ -73121,16 +73351,16 @@
     </row>
     <row r="879" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A879" t="s">
-        <v>955</v>
+        <v>948</v>
       </c>
       <c r="B879" t="s">
-        <v>956</v>
+        <v>949</v>
       </c>
       <c r="C879" t="s">
         <v>936</v>
       </c>
       <c r="D879" t="s">
-        <v>954</v>
+        <v>937</v>
       </c>
       <c r="E879" t="s">
         <v>25</v>
@@ -73159,16 +73389,16 @@
     </row>
     <row r="880" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A880" t="s">
-        <v>957</v>
+        <v>950</v>
       </c>
       <c r="B880" t="s">
-        <v>958</v>
+        <v>951</v>
       </c>
       <c r="C880" t="s">
         <v>936</v>
       </c>
       <c r="D880" t="s">
-        <v>954</v>
+        <v>937</v>
       </c>
       <c r="E880" t="s">
         <v>25</v>
@@ -73197,10 +73427,10 @@
     </row>
     <row r="881" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A881" t="s">
-        <v>959</v>
+        <v>952</v>
       </c>
       <c r="B881" t="s">
-        <v>960</v>
+        <v>953</v>
       </c>
       <c r="C881" t="s">
         <v>936</v>
@@ -73235,10 +73465,10 @@
     </row>
     <row r="882" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A882" t="s">
-        <v>961</v>
+        <v>955</v>
       </c>
       <c r="B882" t="s">
-        <v>962</v>
+        <v>956</v>
       </c>
       <c r="C882" t="s">
         <v>936</v>
@@ -73273,16 +73503,16 @@
     </row>
     <row r="883" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A883" t="s">
-        <v>963</v>
+        <v>957</v>
       </c>
       <c r="B883" t="s">
-        <v>964</v>
+        <v>958</v>
       </c>
       <c r="C883" t="s">
         <v>936</v>
       </c>
       <c r="D883" t="s">
-        <v>965</v>
+        <v>954</v>
       </c>
       <c r="E883" t="s">
         <v>25</v>
@@ -73311,16 +73541,16 @@
     </row>
     <row r="884" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A884" t="s">
-        <v>966</v>
+        <v>959</v>
       </c>
       <c r="B884" t="s">
-        <v>967</v>
+        <v>960</v>
       </c>
       <c r="C884" t="s">
         <v>936</v>
       </c>
       <c r="D884" t="s">
-        <v>965</v>
+        <v>954</v>
       </c>
       <c r="E884" t="s">
         <v>25</v>
@@ -73349,16 +73579,16 @@
     </row>
     <row r="885" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A885" t="s">
-        <v>968</v>
+        <v>961</v>
       </c>
       <c r="B885" t="s">
-        <v>969</v>
+        <v>962</v>
       </c>
       <c r="C885" t="s">
         <v>936</v>
       </c>
       <c r="D885" t="s">
-        <v>970</v>
+        <v>954</v>
       </c>
       <c r="E885" t="s">
         <v>25</v>
@@ -73387,16 +73617,16 @@
     </row>
     <row r="886" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A886" t="s">
-        <v>971</v>
+        <v>963</v>
       </c>
       <c r="B886" t="s">
-        <v>972</v>
+        <v>964</v>
       </c>
       <c r="C886" t="s">
         <v>936</v>
       </c>
       <c r="D886" t="s">
-        <v>970</v>
+        <v>965</v>
       </c>
       <c r="E886" t="s">
         <v>25</v>
@@ -73425,16 +73655,16 @@
     </row>
     <row r="887" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A887" t="s">
-        <v>973</v>
+        <v>966</v>
       </c>
       <c r="B887" t="s">
-        <v>974</v>
+        <v>967</v>
       </c>
       <c r="C887" t="s">
         <v>936</v>
       </c>
       <c r="D887" t="s">
-        <v>970</v>
+        <v>965</v>
       </c>
       <c r="E887" t="s">
         <v>25</v>
@@ -73463,10 +73693,10 @@
     </row>
     <row r="888" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A888" t="s">
-        <v>975</v>
+        <v>968</v>
       </c>
       <c r="B888" t="s">
-        <v>976</v>
+        <v>969</v>
       </c>
       <c r="C888" t="s">
         <v>936</v>
@@ -73501,10 +73731,10 @@
     </row>
     <row r="889" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A889" t="s">
-        <v>977</v>
+        <v>971</v>
       </c>
       <c r="B889" t="s">
-        <v>978</v>
+        <v>972</v>
       </c>
       <c r="C889" t="s">
         <v>936</v>
@@ -73539,10 +73769,10 @@
     </row>
     <row r="890" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A890" t="s">
-        <v>979</v>
+        <v>973</v>
       </c>
       <c r="B890" t="s">
-        <v>980</v>
+        <v>974</v>
       </c>
       <c r="C890" t="s">
         <v>936</v>
@@ -73577,16 +73807,16 @@
     </row>
     <row r="891" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A891" t="s">
-        <v>981</v>
+        <v>975</v>
       </c>
       <c r="B891" t="s">
-        <v>982</v>
+        <v>976</v>
       </c>
       <c r="C891" t="s">
         <v>936</v>
       </c>
       <c r="D891" t="s">
-        <v>983</v>
+        <v>970</v>
       </c>
       <c r="E891" t="s">
         <v>25</v>
@@ -73615,16 +73845,16 @@
     </row>
     <row r="892" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A892" t="s">
-        <v>984</v>
+        <v>977</v>
       </c>
       <c r="B892" t="s">
-        <v>985</v>
+        <v>978</v>
       </c>
       <c r="C892" t="s">
         <v>936</v>
       </c>
       <c r="D892" t="s">
-        <v>983</v>
+        <v>970</v>
       </c>
       <c r="E892" t="s">
         <v>25</v>
@@ -73653,16 +73883,16 @@
     </row>
     <row r="893" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A893" t="s">
-        <v>986</v>
+        <v>979</v>
       </c>
       <c r="B893" t="s">
-        <v>987</v>
+        <v>980</v>
       </c>
       <c r="C893" t="s">
         <v>936</v>
       </c>
       <c r="D893" t="s">
-        <v>983</v>
+        <v>970</v>
       </c>
       <c r="E893" t="s">
         <v>25</v>
@@ -73691,10 +73921,10 @@
     </row>
     <row r="894" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A894" t="s">
-        <v>988</v>
+        <v>981</v>
       </c>
       <c r="B894" t="s">
-        <v>989</v>
+        <v>982</v>
       </c>
       <c r="C894" t="s">
         <v>936</v>
@@ -73729,16 +73959,16 @@
     </row>
     <row r="895" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A895" t="s">
-        <v>990</v>
+        <v>984</v>
       </c>
       <c r="B895" t="s">
-        <v>991</v>
+        <v>985</v>
       </c>
       <c r="C895" t="s">
         <v>936</v>
       </c>
       <c r="D895" t="s">
-        <v>992</v>
+        <v>983</v>
       </c>
       <c r="E895" t="s">
         <v>25</v>
@@ -73767,16 +73997,16 @@
     </row>
     <row r="896" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A896" t="s">
-        <v>993</v>
+        <v>986</v>
       </c>
       <c r="B896" t="s">
-        <v>994</v>
+        <v>987</v>
       </c>
       <c r="C896" t="s">
         <v>936</v>
       </c>
       <c r="D896" t="s">
-        <v>992</v>
+        <v>983</v>
       </c>
       <c r="E896" t="s">
         <v>25</v>
@@ -73805,16 +74035,16 @@
     </row>
     <row r="897" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A897" t="s">
-        <v>995</v>
+        <v>988</v>
       </c>
       <c r="B897" t="s">
-        <v>996</v>
+        <v>989</v>
       </c>
       <c r="C897" t="s">
         <v>936</v>
       </c>
       <c r="D897" t="s">
-        <v>992</v>
+        <v>983</v>
       </c>
       <c r="E897" t="s">
         <v>25</v>
@@ -73843,10 +74073,10 @@
     </row>
     <row r="898" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A898" t="s">
-        <v>997</v>
+        <v>990</v>
       </c>
       <c r="B898" t="s">
-        <v>998</v>
+        <v>991</v>
       </c>
       <c r="C898" t="s">
         <v>936</v>
@@ -73881,16 +74111,16 @@
     </row>
     <row r="899" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A899" t="s">
-        <v>999</v>
+        <v>993</v>
       </c>
       <c r="B899" t="s">
-        <v>1000</v>
+        <v>994</v>
       </c>
       <c r="C899" t="s">
         <v>936</v>
       </c>
       <c r="D899" t="s">
-        <v>1001</v>
+        <v>992</v>
       </c>
       <c r="E899" t="s">
         <v>25</v>
@@ -73919,16 +74149,16 @@
     </row>
     <row r="900" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A900" t="s">
-        <v>1002</v>
+        <v>995</v>
       </c>
       <c r="B900" t="s">
-        <v>1003</v>
+        <v>996</v>
       </c>
       <c r="C900" t="s">
         <v>936</v>
       </c>
       <c r="D900" t="s">
-        <v>1001</v>
+        <v>992</v>
       </c>
       <c r="E900" t="s">
         <v>25</v>
@@ -73957,16 +74187,16 @@
     </row>
     <row r="901" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A901" t="s">
-        <v>1004</v>
+        <v>997</v>
       </c>
       <c r="B901" t="s">
-        <v>1005</v>
+        <v>998</v>
       </c>
       <c r="C901" t="s">
         <v>936</v>
       </c>
       <c r="D901" t="s">
-        <v>1001</v>
+        <v>992</v>
       </c>
       <c r="E901" t="s">
         <v>25</v>
@@ -73995,10 +74225,10 @@
     </row>
     <row r="902" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A902" t="s">
-        <v>1006</v>
+        <v>999</v>
       </c>
       <c r="B902" t="s">
-        <v>1007</v>
+        <v>1000</v>
       </c>
       <c r="C902" t="s">
         <v>936</v>
@@ -74033,16 +74263,16 @@
     </row>
     <row r="903" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A903" t="s">
-        <v>1008</v>
+        <v>1002</v>
       </c>
       <c r="B903" t="s">
-        <v>1009</v>
+        <v>1003</v>
       </c>
       <c r="C903" t="s">
         <v>936</v>
       </c>
       <c r="D903" t="s">
-        <v>1010</v>
+        <v>1001</v>
       </c>
       <c r="E903" t="s">
         <v>25</v>
@@ -74071,16 +74301,16 @@
     </row>
     <row r="904" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A904" t="s">
-        <v>1011</v>
+        <v>1004</v>
       </c>
       <c r="B904" t="s">
-        <v>1012</v>
+        <v>1005</v>
       </c>
       <c r="C904" t="s">
         <v>936</v>
       </c>
       <c r="D904" t="s">
-        <v>1010</v>
+        <v>1001</v>
       </c>
       <c r="E904" t="s">
         <v>25</v>
@@ -74109,16 +74339,16 @@
     </row>
     <row r="905" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A905" t="s">
-        <v>1013</v>
+        <v>1006</v>
       </c>
       <c r="B905" t="s">
-        <v>1014</v>
+        <v>1007</v>
       </c>
       <c r="C905" t="s">
         <v>936</v>
       </c>
       <c r="D905" t="s">
-        <v>1010</v>
+        <v>1001</v>
       </c>
       <c r="E905" t="s">
         <v>25</v>
@@ -74147,10 +74377,10 @@
     </row>
     <row r="906" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A906" t="s">
-        <v>1015</v>
+        <v>1008</v>
       </c>
       <c r="B906" t="s">
-        <v>1016</v>
+        <v>1009</v>
       </c>
       <c r="C906" t="s">
         <v>936</v>
@@ -74185,16 +74415,16 @@
     </row>
     <row r="907" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A907" t="s">
-        <v>1017</v>
+        <v>1011</v>
       </c>
       <c r="B907" t="s">
-        <v>1018</v>
+        <v>1012</v>
       </c>
       <c r="C907" t="s">
         <v>936</v>
       </c>
       <c r="D907" t="s">
-        <v>1019</v>
+        <v>1010</v>
       </c>
       <c r="E907" t="s">
         <v>25</v>
@@ -74223,16 +74453,16 @@
     </row>
     <row r="908" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A908" t="s">
-        <v>1020</v>
+        <v>1013</v>
       </c>
       <c r="B908" t="s">
-        <v>1021</v>
+        <v>1014</v>
       </c>
       <c r="C908" t="s">
         <v>936</v>
       </c>
       <c r="D908" t="s">
-        <v>1019</v>
+        <v>1010</v>
       </c>
       <c r="E908" t="s">
         <v>25</v>
@@ -74261,16 +74491,16 @@
     </row>
     <row r="909" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A909" t="s">
-        <v>1022</v>
+        <v>1015</v>
       </c>
       <c r="B909" t="s">
-        <v>1023</v>
+        <v>1016</v>
       </c>
       <c r="C909" t="s">
         <v>936</v>
       </c>
       <c r="D909" t="s">
-        <v>1019</v>
+        <v>1010</v>
       </c>
       <c r="E909" t="s">
         <v>25</v>
@@ -74299,10 +74529,10 @@
     </row>
     <row r="910" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A910" t="s">
-        <v>1024</v>
+        <v>1017</v>
       </c>
       <c r="B910" t="s">
-        <v>1025</v>
+        <v>1018</v>
       </c>
       <c r="C910" t="s">
         <v>936</v>
@@ -74337,10 +74567,10 @@
     </row>
     <row r="911" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A911" t="s">
-        <v>1026</v>
+        <v>1020</v>
       </c>
       <c r="B911" t="s">
-        <v>1027</v>
+        <v>1021</v>
       </c>
       <c r="C911" t="s">
         <v>936</v>
@@ -74375,10 +74605,10 @@
     </row>
     <row r="912" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A912" t="s">
-        <v>1028</v>
+        <v>1022</v>
       </c>
       <c r="B912" t="s">
-        <v>1029</v>
+        <v>1023</v>
       </c>
       <c r="C912" t="s">
         <v>936</v>
@@ -74408,6 +74638,120 @@
         <v>25</v>
       </c>
       <c r="L912" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="913" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A913" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B913" t="s">
+        <v>1025</v>
+      </c>
+      <c r="C913" t="s">
+        <v>936</v>
+      </c>
+      <c r="D913" t="s">
+        <v>1019</v>
+      </c>
+      <c r="E913" t="s">
+        <v>25</v>
+      </c>
+      <c r="F913" t="s">
+        <v>25</v>
+      </c>
+      <c r="G913" t="s">
+        <v>25</v>
+      </c>
+      <c r="H913" t="s">
+        <v>19</v>
+      </c>
+      <c r="I913" t="s">
+        <v>25</v>
+      </c>
+      <c r="J913" t="s">
+        <v>25</v>
+      </c>
+      <c r="K913" t="s">
+        <v>25</v>
+      </c>
+      <c r="L913" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="914" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A914" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B914" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C914" t="s">
+        <v>936</v>
+      </c>
+      <c r="D914" t="s">
+        <v>1019</v>
+      </c>
+      <c r="E914" t="s">
+        <v>25</v>
+      </c>
+      <c r="F914" t="s">
+        <v>25</v>
+      </c>
+      <c r="G914" t="s">
+        <v>25</v>
+      </c>
+      <c r="H914" t="s">
+        <v>19</v>
+      </c>
+      <c r="I914" t="s">
+        <v>25</v>
+      </c>
+      <c r="J914" t="s">
+        <v>25</v>
+      </c>
+      <c r="K914" t="s">
+        <v>25</v>
+      </c>
+      <c r="L914" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="915" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A915" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B915" t="s">
+        <v>1029</v>
+      </c>
+      <c r="C915" t="s">
+        <v>936</v>
+      </c>
+      <c r="D915" t="s">
+        <v>1019</v>
+      </c>
+      <c r="E915" t="s">
+        <v>25</v>
+      </c>
+      <c r="F915" t="s">
+        <v>25</v>
+      </c>
+      <c r="G915" t="s">
+        <v>25</v>
+      </c>
+      <c r="H915" t="s">
+        <v>19</v>
+      </c>
+      <c r="I915" t="s">
+        <v>25</v>
+      </c>
+      <c r="J915" t="s">
+        <v>25</v>
+      </c>
+      <c r="K915" t="s">
+        <v>25</v>
+      </c>
+      <c r="L915" t="s">
         <v>25</v>
       </c>
     </row>
@@ -74416,7 +74760,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L3 A50:D50 L37 G37:I37 G38:L38 B39:L39 B37:E38 A81 A56:D56 L56 A59:D59 J59:L59 A62:D62 J62:L62 H56 F59 F62 H59 H62 A53:D53 H53:I53 A5:L7 A4:E4 G4:L4 L53 F50 H50:L50 A19:L20 B10:D10 A11:D12 F10:F12 J10:L12 H10:H12 B17:D18 F17:F18 H17:H18 J17:L17 K18:L18 A28:G28 L21 F22:F24 J22:L24 A33:D36 L33 A21:D25 H21:H25 L25 A29:D29 H29:I29 L29 K28:L28 I28 F34:F36 J34:L36 H33:H36 A63:G63 I63:L63 A66:D66 F66 H66:L66 A67:A68 J67:L68 J72:L73 F72 F73:G73 F67:G68 C67:D68 H72 A72:A74 A84 I84:L84 C72:D74 A77 C77:D77 C81:D81 L74 J77:L77 J81:L81 F84:G84 F77 F81 H74 H77 H81 C84:D84 A85:D85 L85 A87 J87:L87 H85 F87 H87 C87:D87 A91:D91 F91 H91:L91 A97:G99 L98 A96:D96 F96 H96:L96 A122:D122 I97:L97 I98:J98 I99:L99 A101:D101 F101 A104:D104 H104:I104 J101:L101 H101 L104 A109:D109 H109:I109 L109 A113:G113 I113:L113 A117 F117 C117:D117 A121 C121:D121 F121 J117:L117 J121:L121 A138:D138 K126:L126 H117 H121 H122:I122 L122 A126:D127 H126:I127 L127 A128:G128 I128:L128 A130:D130 F130 H130:L130 A131:G132 I131:L132 A134:D134 F134 H134:L134 A142:D142 F142 H138 J138:L138 H142:L142 A143:G143 I143:L143 A144:D144 H144:I144 L144 A151:D151 F151 H151:L151 A155:F156 A152:G154 A157:G157 I152:L157 A159:D159 F159 H159:L159 A167:D167 A162:A163 C163:G163 C162:D162 J163:L163 L162 H162 A165:D165 F165 H165:L165 A181:L181 A172:D172 I172:L172 A168:G168 I168:L168 F167 H167:L167 F172 A176:D176 F176 H176:L176 A177:G179 I177:L179 A180:E180 G180:I180 L180 A206:D206 A182:G182 I182:L182 A188:D188 F188 H188:L188 A189:G189 I189:L189 F191 H191:L191 A191:D192 H192:I192 L192 F196 H196:L196 A196:D197 H197:I197 L197 A198:G198 I198:L198 A200:D200 F200 H200:L200 F202 H202:L202 A210:G210 A209:D209 H209:L209 A202:D203 H203:I203 L203 K227:L228 F206 H206:L206 F209 A213:F213 A212:G212 A211:F211 A214:G214 I210:L214 A217:D217 F217 H217 A220:D220 F220 H220 J217:L217 J220:L220 I226:L226 I227:I228 A227:G231 I229:L231 A233:D233 F233 H233:L233 A262:G262 A255:G258 K258:L258 A240:D240 F240 H240:L240 A241:A242 H241:I242 L241:L242 C241:D242 A245:D245 F245 H245:L245 A343:G343 A265:D265 L265 A246:G247 I246:L247 A251:D251 I251 A254:D254 I254 L251 L254 I255:L257 I258 A261:D261 F261 H261:L261 I262:L262 F265 H265:I265 A269:D269 F269 H269:L269 A272:D272 F272 H272:L272 A276:D276 F276 H276:L276 A279:D279 H279:L279 A283:D283 F283 H283:L283 C287:D287 F287 H287:L287 A291:D291 F291 H291:L291 A295:D295 F295 H295:L295 A298:D298 F298 H298:L298 A299:G299 I299:L299 A303:D303 F303 H303:L303 A305:D305 F305 H305:L305 A308:D308 F308 H308:L308 A311:D311 F311 H311:L311 A312:G312 I312:L312 A315:D315 F315 H315:L315 A319:D319 F319 H319:L319 A323:D323 F323 H323:L323 A331:D331 F331 H331:L331 A332:G332 I332:L332 A335:D335 F335 H335:L335 A336:G337 I336:L337 A359:D359 A346:D346 I346:L346 I343:L343 F346 A385:D385 A363:D363 L363 A350:D350 F350 H350:L350 A352:D352 F352 H352:L352 A354:D354 F354 H354:I354 K354:L354 A355:G355 I355:L355 F359 H359:L359 F363 H363:J363 A367:D367 F367 H367:L367 A368:G368 I368:L368 A371:D371 F371 H371:L371 A375:D375 F375 H375:L375 A378:D378 F378 H378:L378 A379:G379 I379:L379 A382:D382 F382 H382:L382 A393:D393 A387:D387 H387 F385 H385:L385 J387:L387 A389:D389 J389:L389 F387 H389 F389 A390:G392 I390:L391 A408:D408 A394:G394 I394:L394 J392:L392 L393 H393 C397:D397 F397 H397 J397:L397 A401:D401 F401 H401 J401:L401 A438 C409:F409 I409:L409 A405:D405 F405 H405 J405:L405 F408 H408 J408:L408 A413 F413 A417 F417 A420 F420 J413:L413 J417:L417 J420:L420 C417:D417 C420:D420 C413:D413 H413 H417 H420 A425:D425 F425 H425 J425:L425 A426:G426 I426:L426 A427:D427 H427 L427 A469 A440 L440 A428:G428 I428:L428 A431:D431 F431 H431:L431 A432:G434 I432:L434 F438 F440 H438 H440 J438:L438 J440 C438:D438 C440:D440 A445:D445 F445 H445:L445 A446:G449 I446:L449 A452:D452 F452 H452:L452 A454:D454 F454 H454:L454 A460:D460 F460 H460:L460 A462 F462 A464 F464 H462 H464 J464:L464 J462:L462 C462:D462 C464:D464 A466 J466:L466 F466 C466:D466 A467:G467 I467:L467 A470:G470 I470:L470 F469 H469 J469:L469 A562:D562 A482:D482 L482 C469:D469 H475:L475 A475:D476 H476:I476 H477 A477:A479 F478:F479 C477:D479 L476:L477 H478:L479 F482 H482 J482 A485:D485 F485 H485:L485 A488:D488 F488 H488:L488 A491:D491 F491 H491:L491 A494:D494 F494 H494:L494 A498:D498 F498 H498:L498 A502:D502 F502 H502:L502 A505:D505 F505 H505:L505 A508:D508 F508 H508:L508 A509:G511 I509:L511 A516:D516 F516 H516:L516 A520 F520 H520:L520 A525:D525 F525 H525:L525 A528:D528 F528 H528:L528 A532:D532 F532 H532:L532 A540 I540:L540 A542:D542 F542 H542:L542 A544:D544 F544 H544:L544 A546:D546 F546 H546:L546 A548:D548 F548 H548:L548 A551:D551 H551:L551 A553:D553 F553 H553:L553 A576:D576 A563 C563:G563 A559:D559 F559 H559:L559 F562 H562:L562 F540 C540:D540 I563:L563 C520:D520 A565:D565 F565 H565:L565 A567:D567 F567 H567:L567 A586:D586 A584 C584:D584 A714:L912 A590:D590 L590 A570:D570 F570 H570:L570 A572:D572 F572 H572:L572 A575 F575 H575:L575 C575:D575 H576:I576 L576 F584 H584:L584 F586 H586:L586 F590 H590:J590 A617:D617 A622:B622 D622 A226:D226 F226 A591:G591 I591:L591 A592:D592 H592:I592 L592 A596:D596 A600:D600 F600 H600:L600 F596 H596:L596 A604:D604 F604 H604:L604 A607:D607 F607 H607:L607 A608:G608 A612:D612 F612 H612:L612 I617:L617 I608:L608 F617 F622 H622:L622 A626:D626 F626 H626:L626 A627:G627 I627:L627 A629:D629 F629 H629:L629 A633:D633 F633 H633:L633 A634:G634 I634:L634 A635:G635 I635:L635 A640:D640 F640 H640:L640 A644:D644 F644 H644:L644 A647:D647 F647 H647:L647 A651:D651 F651 H651:L651 A654 C654:D654 F654 H654:L654 A657:D657 F657 H657:L657 A659:D659 F659 H659:L659 A662:D662 F662 H662:L662 A666:D666 F666 H666:L666 A670:D670 F670 H670:L670 A674:D674 F674 H674:L674 A678:D678 F678 H678:L678 A681:D681 F681 H681:L681 A684:D684 F684 H684:L684 A689:D689 F689 H689:L689 A692:D692 F692 H692:L692 A693:G693 I693:L693 A697:D697 F697 H697:L697 C702:D702 F702 H702:L702 C703:G703 I703:L703 A707:D707 F707 H707:L707 A708:G708 I708:L708 A713:D713 F713 H713:L713" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L3 A50:D50 L37 G37:I37 G38:L38 B39:L39 B37:E38 A81 A56:D56 L56 A59:D59 J59:L59 A62:D62 J62:L62 H56 F59 F62 H59 H62 A53:D53 H53:I53 A5:L7 A4:E4 G4:L4 L53 F50 H50:L50 A19:L20 B10:D10 A11:D12 F10:F12 J10:L12 H10:H12 B17:D18 F17:F18 H17:H18 J17:L17 K18:L18 A28:G28 L21 F22:F24 J22:L24 A33:D36 L33 A21:D25 H21:H25 L25 A29:D29 H29:I29 L29 K28:L28 I28 F34:F36 J34:L36 H33:H36 A63:G63 I63:L63 A66:D66 F66 H66:L66 A67:A68 J67:L68 J72:L73 F72 F73:G73 F67:G68 C67:D68 H72 A72:A74 A84 I84:L84 C72:D74 A77 C77:D77 C81:D81 L74 J77:L77 J81:L81 F84:G84 F77 F81 H74 H77 H81 C84:D84 A85:D85 L85 A87 J87:L87 H85 F87 H87 C87:D87 A91:D91 F91 H91:L91 A97:G99 L98 A96:D96 F96 H96:L96 A122:D122 I97:L97 I98:J98 I99:L99 A101:D101 F101 A104:D104 H104:I104 J101:L101 H101 L104 A109:D109 H109:I109 L109 A113:G113 I113:L113 A117 F117 C117:D117 A121 C121:D121 F121 J117:L117 J121:L121 A138:D138 K126:L126 H117 H121 H122:I122 L122 A126:D127 H126:I127 L127 A128:G128 I128:L128 A130:D130 F130 H130:L130 A131:G132 I131:L132 A134:D134 F134 H134:L134 A142:D142 F142 H138 J138:L138 H142:L142 A143:G143 I143:L143 A144:D144 H144:I144 L144 A151:D151 F151 H151:L151 A155:F156 A152:G154 A157:G157 I152:L157 A159:D159 F159 H159:L159 A167:D167 A162:A163 C163:G163 C162:D162 J163:L163 L162 H162 A165:D165 F165 H165:L165 A181:L181 A172:D172 I172:L172 A168:G168 I168:L168 F167 H167:L167 F172 A176:D176 F176 H176:L176 A177:G179 I177:L179 A180:E180 G180:I180 L180 A206:D206 A182:G182 I182:L182 A188:D188 F188 H188:L188 A189:G189 I189:L189 F191 H191:L191 A191:D192 H192:I192 L192 F196 H196:L196 A196:D197 H197:I197 L197 A198:G198 I198:L198 A200:D200 F200 H200:L200 F202 H202:L202 A210:G210 A209:D209 H209:L209 A202:D203 H203:I203 L203 K227:L228 F206 H206:L206 F209 A213:F213 A212:G212 A211:F211 A214:G214 I210:L214 A217:D217 F217 H217 A220:D220 F220 H220 J217:L217 J220:L220 I226:L226 I227:I228 A227:G231 I229:L231 A233:D233 F233 H233:L233 A262:G262 A255:G258 K258:L258 A240:D240 F240 H240:L240 A241:A242 H241:I242 L241:L242 C241:D242 A245:D245 F245 H245:L245 A343:G343 A265:D265 L265 A246:G247 I246:L247 A251:D251 I251 A254:D254 I254 L251 L254 I255:L257 I258 A261:D261 F261 H261:L261 I262:L262 F265 H265:I265 A269:D269 F269 H269:L269 A272:D272 F272 H272:L272 A276:D276 F276 H276:L276 A279:D279 H279:L279 A283:D283 F283 H283:L283 C287:D287 F287 H287:L287 A291:D291 F291 H291:L291 A295:D295 F295 H295:L295 A298:D298 F298 H298:L298 A299:G299 I299:L299 A303:D303 F303 H303:L303 A305:D305 F305 H305:L305 A308:D308 F308 H308:L308 A311:D311 F311 H311:L311 A312:G312 I312:L312 A315:D315 F315 H315:L315 A319:D319 F319 H319:L319 A323:D323 F323 H323:L323 A331:D331 F331 H331:L331 A332:G332 I332:L332 A335:D335 F335 H335:L335 A336:G337 I336:L337 A359:D359 A346:D346 I346:L346 I343:L343 F346 A385:D385 A363:D363 L363 A350:D350 F350 H350:L350 A352:D352 F352 H352:L352 A354:D354 F354 H354:I354 K354:L354 A355:G355 I355:L355 F359 H359:L359 F363 H363:J363 A367:D367 F367 H367:L367 A368:G368 I368:L368 A371:D371 F371 H371:L371 A375:D375 F375 H375:L375 A378:D378 F378 H378:L378 A379:G379 I379:L379 A382:D382 F382 H382:L382 A393:D393 A387:D387 H387 F385 H385:L385 J387:L387 A389:D389 J389:L389 F387 H389 F389 A390:G392 I390:L391 A408:D408 A394:G394 I394:L394 J392:L392 L393 H393 C397:D397 F397 H397 J397:L397 A401:D401 F401 H401 J401:L401 A438 C409:F409 I409:L409 A405:D405 F405 H405 J405:L405 F408 H408 J408:L408 A413 F413 A417 F417 A420 F420 J413:L413 J417:L417 J420:L420 C417:D417 C420:D420 C413:D413 H413 H417 H420 A425:D425 F425 H425 J425:L425 A426:G426 I426:L426 A427:D427 H427 L427 A469 A440 L440 A428:G428 I428:L428 A431:D431 F431 H431:L431 A432:G434 I432:L434 F438 F440 H438 H440 J438:L438 J440 C438:D438 C440:D440 A445:D445 F445 H445:L445 A446:G449 I446:L449 A452:D452 F452 H452:L452 A454:D454 F454 H454:L454 A460:D460 F460 H460:L460 A462 F462 A464 F464 H462 H464 J464:L464 J462:L462 C462:D462 C464:D464 A466 J466:L466 F466 C466:D466 A467:G467 I467:L467 A470:G470 I470:L470 F469 H469 J469:L469 A562:D562 A482:D482 L482 C469:D469 H475:L475 A475:D476 H476:I476 H477 A477:A479 F478:F479 C477:D479 L476:L477 H478:L479 F482 H482 J482 A485:D485 F485 H485:L485 A488:D488 F488 H488:L488 A491:D491 F491 H491:L491 A494:D494 F494 H494:L494 A498:D498 F498 H498:L498 A502:D502 F502 H502:L502 A505:D505 F505 H505:L505 A508:D508 F508 H508:L508 A509:G511 I509:L511 A516:D516 F516 H516:L516 A520 F520 H520:L520 A525:D525 F525 H525:L525 A528:D528 F528 H528:L528 A532:D532 F532 H532:L532 A540 I540:L540 A542:D542 F542 H542:L542 A544:D544 F544 H544:L544 A546:D546 F546 H546:L546 A548:D548 F548 H548:L548 A551:D551 H551:L551 A553:D553 F553 H553:L553 A576:D576 A563 C563:G563 A559:D559 F559 H559:L559 F562 H562:L562 F540 C540:D540 I563:L563 C520:D520 A565:D565 F565 H565:L565 A567:D567 F567 H567:L567 A586:D586 A584 C584:D584 A721:L915 A590:D590 L590 A570:D570 F570 H570:L570 A572:D572 F572 H572:L572 A575 F575 H575:L575 C575:D575 H576:I576 L576 F584 H584:L584 F586 H586:L586 F590 H590:J590 A617:D617 A622:B622 D622 A226:D226 F226 A591:G591 I591:L591 A592:D592 H592:I592 L592 A596:D596 A600:D600 F600 H600:L600 F596 H596:L596 A604:D604 F604 H604:L604 A607:D607 F607 H607:L607 A608:G608 A612:D612 F612 H612:L612 I617:L617 I608:L608 F617 F622 H622:L622 A626:D626 F626 H626:L626 A627:G627 I627:L627 A629:D629 F629 H629:L629 A633:D633 F633 H633:L633 A634:G635 I634:L635 A640:D640 F640 H640:L640 A644:D644 F644 H644:L644 A647:D647 F647 H647:L647 A651:D651 F651 H651:L651 A654 C654:D654 F654 H654:L654 A657:D657 F657 H657:L657 A659:D659 F659 H659:L659 A662:D662 F662 H662:L662 A666:D666 F666 H666:L666 A670:D670 F670 H670:L670 A674:D674 F674 H674:L674 A678:D678 F678 H678:L678 A681:D681 F681 H681:L681 A684:D684 F684 H684:L684 A689:D689 F689 H689:L689 A692:D692 F692 H692:L692 A693:G693 I693:L693 A697:D697 F697 H697:L697 C702:D702 F702 H702:L702 C703:G703 I703:L703 A707:D707 F707 H707:L707 A708:G708 I708:L708 A713:D713 F713 H713:L713 A714:G715 I714:L715 A716:G716 A720:D720 F720 H720:L720 I716:L716" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
se agrega categoria solar
</commit_message>
<xml_diff>
--- a/BD/Catalogo_Bloopia_Estructurado.xlsx
+++ b/BD/Catalogo_Bloopia_Estructurado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimilitareduco-my.sharepoint.com/personal/est_tatiana_castillo_unimilitar_edu_co/Documents/Backup/Descargas/copiaBloopia (2)/copiaBloopia/Bloopia/BD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3617" documentId="11_39DF2C4B9F61F837F4C1046A4016A4F540A1B085" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD541ABF-9024-4BC2-AFD7-D0C6957BFA47}"/>
+  <xr:revisionPtr revIDLastSave="3655" documentId="11_39DF2C4B9F61F837F4C1046A4016A4F540A1B085" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40F13211-BC71-47D7-9E2C-DD4D9D049469}"/>
   <bookViews>
     <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10327" uniqueCount="2199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10438" uniqueCount="2215">
   <si>
     <t>Codigo</t>
   </si>
@@ -39946,6 +39946,425 @@
 Verifica que las válvulas estén limpias antes de cada uso.
 Lava y seca completamente la olla después de utilizarla para prolongar su vida útil.
 Sigue siempre las indicaciones del manual para una cocción segura.</t>
+    </r>
+  </si>
+  <si>
+    <t>BLO-SOL-001</t>
+  </si>
+  <si>
+    <t>Reflector T02-COB-3M</t>
+  </si>
+  <si>
+    <t>assets/productos/solar/reflectort02/reflectorT02.webp</t>
+  </si>
+  <si>
+    <t>assets/productos/solar/reflectort02/reflectorT022.webp</t>
+  </si>
+  <si>
+    <t>assets/productos/solar/reflectort02/reflectorT023.webp</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Ilumina tus espacios exteriores de forma inteligente con el </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Reflector Solar LED T02 COB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Gracias a sus 216 LEDs tipo COB, proporciona una luz intensa y uniforme que mejora la visibilidad durante la noche, ideal para hogares, negocios y zonas de acceso.
+Su sensor de movimiento activa automáticamente la iluminación al detectar presencia y permanece encendido durante aproximadamente 30 segundos, ofreciendo mayor seguridad y ahorro energético.
+Al funcionar completamente con energía solar, elimina el consumo eléctrico y evita instalaciones complejas, ya que no requiere cableado. Además, incorpora un control remoto para configurar fácilmente su funcionamiento según tus necesidades.
+Su diseño resistente al agua y a las condiciones climáticas lo convierte en una excelente opción para uso permanente en exteriores.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>El Reflector Solar LED T02 COB</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> ofrece una iluminación potente, eficiente y 100% alimentada por energía solar. Equipado con 216 LEDs de alta intensidad, sensor de movimiento, control remoto y protección para exteriores, es la solución ideal para mejorar la seguridad e iluminar patios, jardines, entradas, terrazas y fachadas sin consumir electricidad.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Características principales</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+216 LEDs tipo COB de alta potencia.
+Funciona con energía solar.
+Sensor de movimiento automático.
+Incluye control remoto.
+Resistente al agua y al clima exterior.
+Ángulo de detección de 120°.
+Instalación rápida y sin cables.
+Ideal para patios, jardines, entradas, terrazas, fachadas y garajes.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Especificaciones técnicas</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Modelo: T02 COB.
+Tipo de luz: LED de alta intensidad.
+Sensor: Movimiento automático.
+Tiempo de encendido: Aproximadamente 30 segundos.
+Alimentación: Energía solar.
+Uso: Exterior.
+Ángulo de detección: 120°.
+Cobertura
+Amplio ángulo de detección de 120°.
+Ideal para múltiples posiciones y espacios exteriores.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Contenido del paquete</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1 Reflector Solar LED.
+1 Panel solar.
+1 Control remoto.
+Tornillos y tarugos para instalación.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Beneficios</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+No consume energía eléctrica.
+Iluminación automática al detectar movimiento.
+Mayor seguridad para el hogar o negocio.
+Instalación sencilla sin necesidad de cableado.
+Resistente a la lluvia y a las condiciones del exterior.
+Bajo mantenimiento y larga vida útil.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Recomendaciones de uso</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Instálalo en un lugar donde el panel reciba luz solar directa durante el día.
+Ideal para entradas, patios, jardines, terrazas, garajes y fachadas.
+Utiliza el control remoto para ajustar el funcionamiento según tus necesidades.
+Limpia periódicamente el panel solar para mantener un rendimiento óptimo.
+Evita instalar el panel en zonas con sombra permanente para asegurar una carga eficiente.</t>
+    </r>
+  </si>
+  <si>
+    <t>assets/productos/solar/reflectorsolar/reflectorsolar.webp</t>
+  </si>
+  <si>
+    <t>assets/productos/solar/reflectorsolar/reflectorsolar2.webp</t>
+  </si>
+  <si>
+    <t>assets/productos/solar/reflectorsolar/reflectorsolar3.webp</t>
+  </si>
+  <si>
+    <t>assets/productos/solar/reflectorsolar/reflectorsolar4.webp</t>
+  </si>
+  <si>
+    <t>assets/productos/solar/reflectorsolar/reflectorsolar5.webp</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Ilumina y protege tus espacios exteriores con el </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Reflector Solar LED X3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, una solución eficiente que combina potencia, ahorro energético y facilidad de instalación. Su innovador diseño de tres paneles LED ajustables proporciona una cobertura mucho más amplia, permitiendo orientar la iluminación hacia diferentes direcciones según tus necesidades.
+Gracias a su sensor de movimiento inteligente, la luz se activa automáticamente al detectar presencia, ofreciendo mayor seguridad y comodidad durante la noche.
+Al funcionar completamente con energía solar, elimina el consumo eléctrico y no requiere instalaciones complicadas ni cableado. Además, su protección IP65 lo hace resistente a la lluvia, humedad y condiciones climáticas exteriores, garantizando un excelente rendimiento durante todo el año.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">El Reflector Solar LED X3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ofrece una iluminación exterior más amplia gracias a su diseño de tres paneles ajustables, que permiten dirigir la luz en diferentes ángulos. Funciona con energía solar, incorpora sensor de movimiento y cuenta con protección IP65, siendo ideal para patios, jardines, entradas, terrazas, fachadas y garajes.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Características principales</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Triple panel LED ajustable para una mayor cobertura.
+Funciona con energía solar.
+Sensor de movimiento automático.
+Protección IP65 contra agua y humedad.
+Amplio ángulo de iluminación.
+Instalación sencilla y sin cables.
+Ideal para uso en exteriores.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Especificaciones técnicas</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Tipo: Reflector solar LED.
+Diseño: Triple panel ajustable.
+Sensor: Movimiento automático.
+Alimentación: Energía solar.
+Protección: IP65 (resistente a lluvia y humedad).
+Uso: Exterior.
+Cobertura y detección
+Amplio ángulo de iluminación gracias a sus tres paneles.
+Sensor de movimiento de alta precisión.
+Activación automática al detectar presencia.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Contenido del paquete</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+1 Reflector Solar LED X3.
+Panel solar integrado.
+Kit de instalación (tornillos y tarugos).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Beneficios</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Iluminación amplia y uniforme.
+Ahorro total en consumo eléctrico.
+Mayor seguridad para el hogar o negocio.
+Resistente a las condiciones climáticas.
+Instalación rápida y sin necesidad de cables.
+Bajo mantenimiento y larga vida útil.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Recomendaciones de uso</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Instálalo en un lugar donde reciba luz solar directa durante el día.
+Ajusta los tres paneles para iluminar las áreas que necesites.
+Ideal para entradas, patios, jardines, terrazas, fachadas y garajes.
+Mantén limpio el panel solar para garantizar una carga eficiente.
+Evita instalarlo en zonas con sombra permanente para obtener el máximo rendimiento.</t>
     </r>
   </si>
 </sst>
@@ -40348,7 +40767,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M915"/>
+  <dimension ref="A1:M922"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -67347,10 +67766,10 @@
     </row>
     <row r="721" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A721" t="s">
-        <v>600</v>
+        <v>2199</v>
       </c>
       <c r="B721" t="s">
-        <v>601</v>
+        <v>2200</v>
       </c>
       <c r="C721" t="s">
         <v>602</v>
@@ -67358,14 +67777,14 @@
       <c r="D721" t="s">
         <v>25</v>
       </c>
-      <c r="E721" t="s">
-        <v>25</v>
-      </c>
-      <c r="F721" t="s">
-        <v>25</v>
+      <c r="E721">
+        <v>54578</v>
+      </c>
+      <c r="F721" s="2" t="s">
+        <v>2204</v>
       </c>
       <c r="G721" t="s">
-        <v>25</v>
+        <v>2201</v>
       </c>
       <c r="H721" t="s">
         <v>19</v>
@@ -67374,10 +67793,10 @@
         <v>25</v>
       </c>
       <c r="J721" t="s">
-        <v>25</v>
-      </c>
-      <c r="K721" t="s">
-        <v>25</v>
+        <v>2205</v>
+      </c>
+      <c r="K721" s="2" t="s">
+        <v>2206</v>
       </c>
       <c r="L721" t="s">
         <v>25</v>
@@ -67385,10 +67804,10 @@
     </row>
     <row r="722" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A722" t="s">
-        <v>603</v>
+        <v>2199</v>
       </c>
       <c r="B722" t="s">
-        <v>604</v>
+        <v>2200</v>
       </c>
       <c r="C722" t="s">
         <v>602</v>
@@ -67396,14 +67815,14 @@
       <c r="D722" t="s">
         <v>25</v>
       </c>
-      <c r="E722" t="s">
-        <v>25</v>
+      <c r="E722">
+        <v>54578</v>
       </c>
       <c r="F722" t="s">
         <v>25</v>
       </c>
       <c r="G722" t="s">
-        <v>25</v>
+        <v>2202</v>
       </c>
       <c r="H722" t="s">
         <v>19</v>
@@ -67423,10 +67842,10 @@
     </row>
     <row r="723" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A723" t="s">
-        <v>605</v>
+        <v>2199</v>
       </c>
       <c r="B723" t="s">
-        <v>606</v>
+        <v>2200</v>
       </c>
       <c r="C723" t="s">
         <v>602</v>
@@ -67434,14 +67853,14 @@
       <c r="D723" t="s">
         <v>25</v>
       </c>
-      <c r="E723" t="s">
-        <v>25</v>
+      <c r="E723">
+        <v>54578</v>
       </c>
       <c r="F723" t="s">
         <v>25</v>
       </c>
       <c r="G723" t="s">
-        <v>25</v>
+        <v>2203</v>
       </c>
       <c r="H723" t="s">
         <v>19</v>
@@ -67461,10 +67880,10 @@
     </row>
     <row r="724" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A724" t="s">
-        <v>607</v>
+        <v>600</v>
       </c>
       <c r="B724" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="C724" t="s">
         <v>602</v>
@@ -67472,14 +67891,14 @@
       <c r="D724" t="s">
         <v>25</v>
       </c>
-      <c r="E724" t="s">
-        <v>25</v>
-      </c>
-      <c r="F724" t="s">
-        <v>25</v>
+      <c r="E724">
+        <v>51467</v>
+      </c>
+      <c r="F724" s="2" t="s">
+        <v>2212</v>
       </c>
       <c r="G724" t="s">
-        <v>25</v>
+        <v>2207</v>
       </c>
       <c r="H724" t="s">
         <v>19</v>
@@ -67488,10 +67907,10 @@
         <v>25</v>
       </c>
       <c r="J724" t="s">
-        <v>25</v>
-      </c>
-      <c r="K724" t="s">
-        <v>25</v>
+        <v>2213</v>
+      </c>
+      <c r="K724" s="2" t="s">
+        <v>2214</v>
       </c>
       <c r="L724" t="s">
         <v>25</v>
@@ -67499,10 +67918,10 @@
     </row>
     <row r="725" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A725" t="s">
-        <v>609</v>
+        <v>600</v>
       </c>
       <c r="B725" t="s">
-        <v>610</v>
+        <v>601</v>
       </c>
       <c r="C725" t="s">
         <v>602</v>
@@ -67510,14 +67929,14 @@
       <c r="D725" t="s">
         <v>25</v>
       </c>
-      <c r="E725" t="s">
-        <v>25</v>
+      <c r="E725">
+        <v>51467</v>
       </c>
       <c r="F725" t="s">
         <v>25</v>
       </c>
       <c r="G725" t="s">
-        <v>25</v>
+        <v>2208</v>
       </c>
       <c r="H725" t="s">
         <v>19</v>
@@ -67537,10 +67956,10 @@
     </row>
     <row r="726" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A726" t="s">
-        <v>611</v>
+        <v>600</v>
       </c>
       <c r="B726" t="s">
-        <v>612</v>
+        <v>601</v>
       </c>
       <c r="C726" t="s">
         <v>602</v>
@@ -67548,14 +67967,14 @@
       <c r="D726" t="s">
         <v>25</v>
       </c>
-      <c r="E726" t="s">
-        <v>25</v>
+      <c r="E726">
+        <v>51467</v>
       </c>
       <c r="F726" t="s">
         <v>25</v>
       </c>
       <c r="G726" t="s">
-        <v>25</v>
+        <v>2209</v>
       </c>
       <c r="H726" t="s">
         <v>19</v>
@@ -67575,10 +67994,10 @@
     </row>
     <row r="727" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A727" t="s">
-        <v>613</v>
+        <v>600</v>
       </c>
       <c r="B727" t="s">
-        <v>614</v>
+        <v>601</v>
       </c>
       <c r="C727" t="s">
         <v>602</v>
@@ -67586,14 +68005,14 @@
       <c r="D727" t="s">
         <v>25</v>
       </c>
-      <c r="E727" t="s">
-        <v>25</v>
+      <c r="E727">
+        <v>51467</v>
       </c>
       <c r="F727" t="s">
         <v>25</v>
       </c>
       <c r="G727" t="s">
-        <v>25</v>
+        <v>2210</v>
       </c>
       <c r="H727" t="s">
         <v>19</v>
@@ -67613,10 +68032,10 @@
     </row>
     <row r="728" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A728" t="s">
-        <v>615</v>
+        <v>600</v>
       </c>
       <c r="B728" t="s">
-        <v>616</v>
+        <v>601</v>
       </c>
       <c r="C728" t="s">
         <v>602</v>
@@ -67624,14 +68043,14 @@
       <c r="D728" t="s">
         <v>25</v>
       </c>
-      <c r="E728" t="s">
-        <v>25</v>
+      <c r="E728">
+        <v>51467</v>
       </c>
       <c r="F728" t="s">
         <v>25</v>
       </c>
       <c r="G728" t="s">
-        <v>25</v>
+        <v>2211</v>
       </c>
       <c r="H728" t="s">
         <v>19</v>
@@ -67651,16 +68070,16 @@
     </row>
     <row r="729" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A729" t="s">
-        <v>617</v>
+        <v>603</v>
       </c>
       <c r="B729" t="s">
-        <v>618</v>
+        <v>604</v>
       </c>
       <c r="C729" t="s">
-        <v>619</v>
+        <v>602</v>
       </c>
       <c r="D729" t="s">
-        <v>620</v>
+        <v>25</v>
       </c>
       <c r="E729" t="s">
         <v>25</v>
@@ -67689,16 +68108,16 @@
     </row>
     <row r="730" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A730" t="s">
-        <v>621</v>
+        <v>605</v>
       </c>
       <c r="B730" t="s">
-        <v>622</v>
+        <v>606</v>
       </c>
       <c r="C730" t="s">
-        <v>619</v>
+        <v>602</v>
       </c>
       <c r="D730" t="s">
-        <v>620</v>
+        <v>25</v>
       </c>
       <c r="E730" t="s">
         <v>25</v>
@@ -67727,16 +68146,16 @@
     </row>
     <row r="731" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A731" t="s">
-        <v>623</v>
+        <v>607</v>
       </c>
       <c r="B731" t="s">
-        <v>624</v>
+        <v>608</v>
       </c>
       <c r="C731" t="s">
-        <v>619</v>
+        <v>602</v>
       </c>
       <c r="D731" t="s">
-        <v>620</v>
+        <v>25</v>
       </c>
       <c r="E731" t="s">
         <v>25</v>
@@ -67765,16 +68184,16 @@
     </row>
     <row r="732" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A732" t="s">
-        <v>625</v>
+        <v>609</v>
       </c>
       <c r="B732" t="s">
-        <v>626</v>
+        <v>610</v>
       </c>
       <c r="C732" t="s">
-        <v>619</v>
+        <v>602</v>
       </c>
       <c r="D732" t="s">
-        <v>620</v>
+        <v>25</v>
       </c>
       <c r="E732" t="s">
         <v>25</v>
@@ -67803,16 +68222,16 @@
     </row>
     <row r="733" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A733" t="s">
-        <v>627</v>
+        <v>611</v>
       </c>
       <c r="B733" t="s">
-        <v>628</v>
+        <v>612</v>
       </c>
       <c r="C733" t="s">
-        <v>619</v>
+        <v>602</v>
       </c>
       <c r="D733" t="s">
-        <v>138</v>
+        <v>25</v>
       </c>
       <c r="E733" t="s">
         <v>25</v>
@@ -67841,16 +68260,16 @@
     </row>
     <row r="734" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A734" t="s">
-        <v>629</v>
+        <v>613</v>
       </c>
       <c r="B734" t="s">
-        <v>630</v>
+        <v>614</v>
       </c>
       <c r="C734" t="s">
-        <v>619</v>
+        <v>602</v>
       </c>
       <c r="D734" t="s">
-        <v>138</v>
+        <v>25</v>
       </c>
       <c r="E734" t="s">
         <v>25</v>
@@ -67879,16 +68298,16 @@
     </row>
     <row r="735" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A735" t="s">
-        <v>631</v>
+        <v>615</v>
       </c>
       <c r="B735" t="s">
-        <v>632</v>
+        <v>616</v>
       </c>
       <c r="C735" t="s">
-        <v>619</v>
+        <v>602</v>
       </c>
       <c r="D735" t="s">
-        <v>138</v>
+        <v>25</v>
       </c>
       <c r="E735" t="s">
         <v>25</v>
@@ -67917,16 +68336,16 @@
     </row>
     <row r="736" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A736" t="s">
-        <v>633</v>
+        <v>617</v>
       </c>
       <c r="B736" t="s">
-        <v>634</v>
+        <v>618</v>
       </c>
       <c r="C736" t="s">
         <v>619</v>
       </c>
       <c r="D736" t="s">
-        <v>138</v>
+        <v>620</v>
       </c>
       <c r="E736" t="s">
         <v>25</v>
@@ -67955,16 +68374,16 @@
     </row>
     <row r="737" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A737" t="s">
-        <v>635</v>
+        <v>621</v>
       </c>
       <c r="B737" t="s">
-        <v>636</v>
+        <v>622</v>
       </c>
       <c r="C737" t="s">
         <v>619</v>
       </c>
       <c r="D737" t="s">
-        <v>637</v>
+        <v>620</v>
       </c>
       <c r="E737" t="s">
         <v>25</v>
@@ -67993,16 +68412,16 @@
     </row>
     <row r="738" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A738" t="s">
-        <v>638</v>
+        <v>623</v>
       </c>
       <c r="B738" t="s">
-        <v>639</v>
+        <v>624</v>
       </c>
       <c r="C738" t="s">
         <v>619</v>
       </c>
       <c r="D738" t="s">
-        <v>637</v>
+        <v>620</v>
       </c>
       <c r="E738" t="s">
         <v>25</v>
@@ -68031,16 +68450,16 @@
     </row>
     <row r="739" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A739" t="s">
-        <v>640</v>
+        <v>625</v>
       </c>
       <c r="B739" t="s">
-        <v>641</v>
+        <v>626</v>
       </c>
       <c r="C739" t="s">
         <v>619</v>
       </c>
       <c r="D739" t="s">
-        <v>637</v>
+        <v>620</v>
       </c>
       <c r="E739" t="s">
         <v>25</v>
@@ -68069,16 +68488,16 @@
     </row>
     <row r="740" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A740" t="s">
-        <v>642</v>
+        <v>627</v>
       </c>
       <c r="B740" t="s">
-        <v>643</v>
+        <v>628</v>
       </c>
       <c r="C740" t="s">
         <v>619</v>
       </c>
       <c r="D740" t="s">
-        <v>637</v>
+        <v>138</v>
       </c>
       <c r="E740" t="s">
         <v>25</v>
@@ -68107,16 +68526,16 @@
     </row>
     <row r="741" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A741" t="s">
-        <v>644</v>
+        <v>629</v>
       </c>
       <c r="B741" t="s">
-        <v>645</v>
+        <v>630</v>
       </c>
       <c r="C741" t="s">
         <v>619</v>
       </c>
       <c r="D741" t="s">
-        <v>637</v>
+        <v>138</v>
       </c>
       <c r="E741" t="s">
         <v>25</v>
@@ -68145,16 +68564,16 @@
     </row>
     <row r="742" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A742" t="s">
-        <v>646</v>
+        <v>631</v>
       </c>
       <c r="B742" t="s">
-        <v>647</v>
+        <v>632</v>
       </c>
       <c r="C742" t="s">
         <v>619</v>
       </c>
       <c r="D742" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="E742" t="s">
         <v>25</v>
@@ -68183,16 +68602,16 @@
     </row>
     <row r="743" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A743" t="s">
-        <v>648</v>
+        <v>633</v>
       </c>
       <c r="B743" t="s">
-        <v>649</v>
+        <v>634</v>
       </c>
       <c r="C743" t="s">
         <v>619</v>
       </c>
       <c r="D743" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="E743" t="s">
         <v>25</v>
@@ -68221,16 +68640,16 @@
     </row>
     <row r="744" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A744" t="s">
-        <v>650</v>
+        <v>635</v>
       </c>
       <c r="B744" t="s">
-        <v>651</v>
+        <v>636</v>
       </c>
       <c r="C744" t="s">
         <v>619</v>
       </c>
       <c r="D744" t="s">
-        <v>652</v>
+        <v>637</v>
       </c>
       <c r="E744" t="s">
         <v>25</v>
@@ -68259,16 +68678,16 @@
     </row>
     <row r="745" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A745" t="s">
-        <v>653</v>
+        <v>638</v>
       </c>
       <c r="B745" t="s">
-        <v>654</v>
+        <v>639</v>
       </c>
       <c r="C745" t="s">
         <v>619</v>
       </c>
       <c r="D745" t="s">
-        <v>652</v>
+        <v>637</v>
       </c>
       <c r="E745" t="s">
         <v>25</v>
@@ -68297,16 +68716,16 @@
     </row>
     <row r="746" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A746" t="s">
-        <v>655</v>
+        <v>640</v>
       </c>
       <c r="B746" t="s">
-        <v>656</v>
+        <v>641</v>
       </c>
       <c r="C746" t="s">
         <v>619</v>
       </c>
       <c r="D746" t="s">
-        <v>652</v>
+        <v>637</v>
       </c>
       <c r="E746" t="s">
         <v>25</v>
@@ -68335,16 +68754,16 @@
     </row>
     <row r="747" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A747" t="s">
-        <v>655</v>
+        <v>642</v>
       </c>
       <c r="B747" t="s">
-        <v>657</v>
+        <v>643</v>
       </c>
       <c r="C747" t="s">
         <v>619</v>
       </c>
       <c r="D747" t="s">
-        <v>652</v>
+        <v>637</v>
       </c>
       <c r="E747" t="s">
         <v>25</v>
@@ -68373,16 +68792,16 @@
     </row>
     <row r="748" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A748" t="s">
-        <v>658</v>
+        <v>644</v>
       </c>
       <c r="B748" t="s">
-        <v>659</v>
+        <v>645</v>
       </c>
       <c r="C748" t="s">
-        <v>660</v>
+        <v>619</v>
       </c>
       <c r="D748" t="s">
-        <v>661</v>
+        <v>637</v>
       </c>
       <c r="E748" t="s">
         <v>25</v>
@@ -68411,16 +68830,16 @@
     </row>
     <row r="749" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A749" t="s">
-        <v>662</v>
+        <v>646</v>
       </c>
       <c r="B749" t="s">
-        <v>663</v>
+        <v>647</v>
       </c>
       <c r="C749" t="s">
-        <v>660</v>
+        <v>619</v>
       </c>
       <c r="D749" t="s">
-        <v>661</v>
+        <v>128</v>
       </c>
       <c r="E749" t="s">
         <v>25</v>
@@ -68449,16 +68868,16 @@
     </row>
     <row r="750" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A750" t="s">
-        <v>664</v>
+        <v>648</v>
       </c>
       <c r="B750" t="s">
-        <v>665</v>
+        <v>649</v>
       </c>
       <c r="C750" t="s">
-        <v>660</v>
+        <v>619</v>
       </c>
       <c r="D750" t="s">
-        <v>661</v>
+        <v>128</v>
       </c>
       <c r="E750" t="s">
         <v>25</v>
@@ -68487,16 +68906,16 @@
     </row>
     <row r="751" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A751" t="s">
-        <v>666</v>
+        <v>650</v>
       </c>
       <c r="B751" t="s">
-        <v>667</v>
+        <v>651</v>
       </c>
       <c r="C751" t="s">
-        <v>660</v>
+        <v>619</v>
       </c>
       <c r="D751" t="s">
-        <v>661</v>
+        <v>652</v>
       </c>
       <c r="E751" t="s">
         <v>25</v>
@@ -68525,16 +68944,16 @@
     </row>
     <row r="752" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A752" t="s">
-        <v>668</v>
+        <v>653</v>
       </c>
       <c r="B752" t="s">
-        <v>669</v>
+        <v>654</v>
       </c>
       <c r="C752" t="s">
-        <v>660</v>
+        <v>619</v>
       </c>
       <c r="D752" t="s">
-        <v>661</v>
+        <v>652</v>
       </c>
       <c r="E752" t="s">
         <v>25</v>
@@ -68563,16 +68982,16 @@
     </row>
     <row r="753" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A753" t="s">
-        <v>670</v>
+        <v>655</v>
       </c>
       <c r="B753" t="s">
-        <v>671</v>
+        <v>656</v>
       </c>
       <c r="C753" t="s">
-        <v>660</v>
+        <v>619</v>
       </c>
       <c r="D753" t="s">
-        <v>661</v>
+        <v>652</v>
       </c>
       <c r="E753" t="s">
         <v>25</v>
@@ -68601,16 +69020,16 @@
     </row>
     <row r="754" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A754" t="s">
-        <v>672</v>
+        <v>655</v>
       </c>
       <c r="B754" t="s">
-        <v>673</v>
+        <v>657</v>
       </c>
       <c r="C754" t="s">
-        <v>660</v>
+        <v>619</v>
       </c>
       <c r="D754" t="s">
-        <v>674</v>
+        <v>652</v>
       </c>
       <c r="E754" t="s">
         <v>25</v>
@@ -68639,16 +69058,16 @@
     </row>
     <row r="755" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A755" t="s">
-        <v>675</v>
+        <v>658</v>
       </c>
       <c r="B755" t="s">
-        <v>676</v>
+        <v>659</v>
       </c>
       <c r="C755" t="s">
         <v>660</v>
       </c>
       <c r="D755" t="s">
-        <v>674</v>
+        <v>661</v>
       </c>
       <c r="E755" t="s">
         <v>25</v>
@@ -68677,16 +69096,16 @@
     </row>
     <row r="756" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A756" t="s">
-        <v>677</v>
+        <v>662</v>
       </c>
       <c r="B756" t="s">
-        <v>678</v>
+        <v>663</v>
       </c>
       <c r="C756" t="s">
         <v>660</v>
       </c>
       <c r="D756" t="s">
-        <v>674</v>
+        <v>661</v>
       </c>
       <c r="E756" t="s">
         <v>25</v>
@@ -68715,16 +69134,16 @@
     </row>
     <row r="757" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A757" t="s">
-        <v>679</v>
+        <v>664</v>
       </c>
       <c r="B757" t="s">
-        <v>680</v>
+        <v>665</v>
       </c>
       <c r="C757" t="s">
         <v>660</v>
       </c>
       <c r="D757" t="s">
-        <v>681</v>
+        <v>661</v>
       </c>
       <c r="E757" t="s">
         <v>25</v>
@@ -68753,16 +69172,16 @@
     </row>
     <row r="758" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A758" t="s">
-        <v>682</v>
+        <v>666</v>
       </c>
       <c r="B758" t="s">
-        <v>683</v>
+        <v>667</v>
       </c>
       <c r="C758" t="s">
         <v>660</v>
       </c>
       <c r="D758" t="s">
-        <v>681</v>
+        <v>661</v>
       </c>
       <c r="E758" t="s">
         <v>25</v>
@@ -68791,16 +69210,16 @@
     </row>
     <row r="759" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A759" t="s">
-        <v>684</v>
+        <v>668</v>
       </c>
       <c r="B759" t="s">
-        <v>685</v>
+        <v>669</v>
       </c>
       <c r="C759" t="s">
         <v>660</v>
       </c>
       <c r="D759" t="s">
-        <v>681</v>
+        <v>661</v>
       </c>
       <c r="E759" t="s">
         <v>25</v>
@@ -68829,16 +69248,16 @@
     </row>
     <row r="760" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A760" t="s">
-        <v>686</v>
+        <v>670</v>
       </c>
       <c r="B760" t="s">
-        <v>687</v>
+        <v>671</v>
       </c>
       <c r="C760" t="s">
         <v>660</v>
       </c>
       <c r="D760" t="s">
-        <v>681</v>
+        <v>661</v>
       </c>
       <c r="E760" t="s">
         <v>25</v>
@@ -68867,16 +69286,16 @@
     </row>
     <row r="761" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A761" t="s">
-        <v>688</v>
+        <v>672</v>
       </c>
       <c r="B761" t="s">
-        <v>689</v>
+        <v>673</v>
       </c>
       <c r="C761" t="s">
         <v>660</v>
       </c>
       <c r="D761" t="s">
-        <v>690</v>
+        <v>674</v>
       </c>
       <c r="E761" t="s">
         <v>25</v>
@@ -68905,16 +69324,16 @@
     </row>
     <row r="762" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A762" t="s">
-        <v>691</v>
+        <v>675</v>
       </c>
       <c r="B762" t="s">
-        <v>689</v>
+        <v>676</v>
       </c>
       <c r="C762" t="s">
         <v>660</v>
       </c>
       <c r="D762" t="s">
-        <v>690</v>
+        <v>674</v>
       </c>
       <c r="E762" t="s">
         <v>25</v>
@@ -68943,16 +69362,16 @@
     </row>
     <row r="763" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A763" t="s">
-        <v>692</v>
+        <v>677</v>
       </c>
       <c r="B763" t="s">
-        <v>693</v>
+        <v>678</v>
       </c>
       <c r="C763" t="s">
         <v>660</v>
       </c>
       <c r="D763" t="s">
-        <v>690</v>
+        <v>674</v>
       </c>
       <c r="E763" t="s">
         <v>25</v>
@@ -68981,16 +69400,16 @@
     </row>
     <row r="764" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A764" t="s">
-        <v>694</v>
+        <v>679</v>
       </c>
       <c r="B764" t="s">
-        <v>695</v>
+        <v>680</v>
       </c>
       <c r="C764" t="s">
         <v>660</v>
       </c>
       <c r="D764" t="s">
-        <v>696</v>
+        <v>681</v>
       </c>
       <c r="E764" t="s">
         <v>25</v>
@@ -69019,16 +69438,16 @@
     </row>
     <row r="765" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A765" t="s">
-        <v>697</v>
+        <v>682</v>
       </c>
       <c r="B765" t="s">
-        <v>698</v>
+        <v>683</v>
       </c>
       <c r="C765" t="s">
         <v>660</v>
       </c>
       <c r="D765" t="s">
-        <v>696</v>
+        <v>681</v>
       </c>
       <c r="E765" t="s">
         <v>25</v>
@@ -69057,16 +69476,16 @@
     </row>
     <row r="766" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A766" t="s">
-        <v>699</v>
+        <v>684</v>
       </c>
       <c r="B766" t="s">
-        <v>700</v>
+        <v>685</v>
       </c>
       <c r="C766" t="s">
         <v>660</v>
       </c>
       <c r="D766" t="s">
-        <v>696</v>
+        <v>681</v>
       </c>
       <c r="E766" t="s">
         <v>25</v>
@@ -69095,16 +69514,16 @@
     </row>
     <row r="767" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A767" t="s">
-        <v>701</v>
+        <v>686</v>
       </c>
       <c r="B767" t="s">
-        <v>702</v>
+        <v>687</v>
       </c>
       <c r="C767" t="s">
         <v>660</v>
       </c>
       <c r="D767" t="s">
-        <v>696</v>
+        <v>681</v>
       </c>
       <c r="E767" t="s">
         <v>25</v>
@@ -69133,16 +69552,16 @@
     </row>
     <row r="768" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A768" t="s">
-        <v>703</v>
+        <v>688</v>
       </c>
       <c r="B768" t="s">
-        <v>704</v>
+        <v>689</v>
       </c>
       <c r="C768" t="s">
         <v>660</v>
       </c>
       <c r="D768" t="s">
-        <v>696</v>
+        <v>690</v>
       </c>
       <c r="E768" t="s">
         <v>25</v>
@@ -69171,16 +69590,16 @@
     </row>
     <row r="769" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A769" t="s">
-        <v>705</v>
+        <v>691</v>
       </c>
       <c r="B769" t="s">
-        <v>706</v>
+        <v>689</v>
       </c>
       <c r="C769" t="s">
         <v>660</v>
       </c>
       <c r="D769" t="s">
-        <v>707</v>
+        <v>690</v>
       </c>
       <c r="E769" t="s">
         <v>25</v>
@@ -69209,16 +69628,16 @@
     </row>
     <row r="770" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A770" t="s">
-        <v>708</v>
+        <v>692</v>
       </c>
       <c r="B770" t="s">
-        <v>709</v>
+        <v>693</v>
       </c>
       <c r="C770" t="s">
         <v>660</v>
       </c>
       <c r="D770" t="s">
-        <v>707</v>
+        <v>690</v>
       </c>
       <c r="E770" t="s">
         <v>25</v>
@@ -69247,16 +69666,16 @@
     </row>
     <row r="771" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A771" t="s">
-        <v>710</v>
+        <v>694</v>
       </c>
       <c r="B771" t="s">
-        <v>711</v>
+        <v>695</v>
       </c>
       <c r="C771" t="s">
         <v>660</v>
       </c>
       <c r="D771" t="s">
-        <v>707</v>
+        <v>696</v>
       </c>
       <c r="E771" t="s">
         <v>25</v>
@@ -69285,16 +69704,16 @@
     </row>
     <row r="772" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A772" t="s">
-        <v>712</v>
+        <v>697</v>
       </c>
       <c r="B772" t="s">
-        <v>713</v>
+        <v>698</v>
       </c>
       <c r="C772" t="s">
         <v>660</v>
       </c>
       <c r="D772" t="s">
-        <v>707</v>
+        <v>696</v>
       </c>
       <c r="E772" t="s">
         <v>25</v>
@@ -69323,16 +69742,16 @@
     </row>
     <row r="773" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A773" t="s">
-        <v>714</v>
+        <v>699</v>
       </c>
       <c r="B773" t="s">
-        <v>715</v>
+        <v>700</v>
       </c>
       <c r="C773" t="s">
         <v>660</v>
       </c>
       <c r="D773" t="s">
-        <v>707</v>
+        <v>696</v>
       </c>
       <c r="E773" t="s">
         <v>25</v>
@@ -69361,16 +69780,16 @@
     </row>
     <row r="774" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A774" t="s">
-        <v>716</v>
+        <v>701</v>
       </c>
       <c r="B774" t="s">
-        <v>717</v>
+        <v>702</v>
       </c>
       <c r="C774" t="s">
         <v>660</v>
       </c>
       <c r="D774" t="s">
-        <v>707</v>
+        <v>696</v>
       </c>
       <c r="E774" t="s">
         <v>25</v>
@@ -69399,16 +69818,16 @@
     </row>
     <row r="775" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A775" t="s">
-        <v>718</v>
+        <v>703</v>
       </c>
       <c r="B775" t="s">
-        <v>719</v>
+        <v>704</v>
       </c>
       <c r="C775" t="s">
         <v>660</v>
       </c>
       <c r="D775" t="s">
-        <v>720</v>
+        <v>696</v>
       </c>
       <c r="E775" t="s">
         <v>25</v>
@@ -69437,16 +69856,16 @@
     </row>
     <row r="776" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A776" t="s">
-        <v>721</v>
+        <v>705</v>
       </c>
       <c r="B776" t="s">
-        <v>722</v>
+        <v>706</v>
       </c>
       <c r="C776" t="s">
         <v>660</v>
       </c>
       <c r="D776" t="s">
-        <v>720</v>
+        <v>707</v>
       </c>
       <c r="E776" t="s">
         <v>25</v>
@@ -69475,16 +69894,16 @@
     </row>
     <row r="777" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A777" t="s">
-        <v>723</v>
+        <v>708</v>
       </c>
       <c r="B777" t="s">
-        <v>724</v>
+        <v>709</v>
       </c>
       <c r="C777" t="s">
-        <v>725</v>
+        <v>660</v>
       </c>
       <c r="D777" t="s">
-        <v>726</v>
+        <v>707</v>
       </c>
       <c r="E777" t="s">
         <v>25</v>
@@ -69513,16 +69932,16 @@
     </row>
     <row r="778" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A778" t="s">
-        <v>727</v>
+        <v>710</v>
       </c>
       <c r="B778" t="s">
-        <v>728</v>
+        <v>711</v>
       </c>
       <c r="C778" t="s">
-        <v>725</v>
+        <v>660</v>
       </c>
       <c r="D778" t="s">
-        <v>726</v>
+        <v>707</v>
       </c>
       <c r="E778" t="s">
         <v>25</v>
@@ -69551,16 +69970,16 @@
     </row>
     <row r="779" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A779" t="s">
-        <v>729</v>
+        <v>712</v>
       </c>
       <c r="B779" t="s">
-        <v>730</v>
+        <v>713</v>
       </c>
       <c r="C779" t="s">
-        <v>725</v>
+        <v>660</v>
       </c>
       <c r="D779" t="s">
-        <v>726</v>
+        <v>707</v>
       </c>
       <c r="E779" t="s">
         <v>25</v>
@@ -69589,16 +70008,16 @@
     </row>
     <row r="780" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A780" t="s">
-        <v>731</v>
+        <v>714</v>
       </c>
       <c r="B780" t="s">
-        <v>732</v>
+        <v>715</v>
       </c>
       <c r="C780" t="s">
-        <v>725</v>
+        <v>660</v>
       </c>
       <c r="D780" t="s">
-        <v>726</v>
+        <v>707</v>
       </c>
       <c r="E780" t="s">
         <v>25</v>
@@ -69627,16 +70046,16 @@
     </row>
     <row r="781" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A781" t="s">
-        <v>733</v>
+        <v>716</v>
       </c>
       <c r="B781" t="s">
-        <v>734</v>
+        <v>717</v>
       </c>
       <c r="C781" t="s">
-        <v>725</v>
+        <v>660</v>
       </c>
       <c r="D781" t="s">
-        <v>726</v>
+        <v>707</v>
       </c>
       <c r="E781" t="s">
         <v>25</v>
@@ -69665,16 +70084,16 @@
     </row>
     <row r="782" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A782" t="s">
-        <v>735</v>
+        <v>718</v>
       </c>
       <c r="B782" t="s">
-        <v>736</v>
+        <v>719</v>
       </c>
       <c r="C782" t="s">
-        <v>725</v>
+        <v>660</v>
       </c>
       <c r="D782" t="s">
-        <v>726</v>
+        <v>720</v>
       </c>
       <c r="E782" t="s">
         <v>25</v>
@@ -69703,16 +70122,16 @@
     </row>
     <row r="783" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A783" t="s">
-        <v>737</v>
+        <v>721</v>
       </c>
       <c r="B783" t="s">
-        <v>738</v>
+        <v>722</v>
       </c>
       <c r="C783" t="s">
-        <v>725</v>
+        <v>660</v>
       </c>
       <c r="D783" t="s">
-        <v>726</v>
+        <v>720</v>
       </c>
       <c r="E783" t="s">
         <v>25</v>
@@ -69741,10 +70160,10 @@
     </row>
     <row r="784" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A784" t="s">
-        <v>739</v>
+        <v>723</v>
       </c>
       <c r="B784" t="s">
-        <v>740</v>
+        <v>724</v>
       </c>
       <c r="C784" t="s">
         <v>725</v>
@@ -69779,10 +70198,10 @@
     </row>
     <row r="785" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A785" t="s">
-        <v>741</v>
+        <v>727</v>
       </c>
       <c r="B785" t="s">
-        <v>742</v>
+        <v>728</v>
       </c>
       <c r="C785" t="s">
         <v>725</v>
@@ -69817,10 +70236,10 @@
     </row>
     <row r="786" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A786" t="s">
-        <v>743</v>
+        <v>729</v>
       </c>
       <c r="B786" t="s">
-        <v>744</v>
+        <v>730</v>
       </c>
       <c r="C786" t="s">
         <v>725</v>
@@ -69855,10 +70274,10 @@
     </row>
     <row r="787" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A787" t="s">
-        <v>745</v>
+        <v>731</v>
       </c>
       <c r="B787" t="s">
-        <v>746</v>
+        <v>732</v>
       </c>
       <c r="C787" t="s">
         <v>725</v>
@@ -69893,10 +70312,10 @@
     </row>
     <row r="788" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A788" t="s">
-        <v>747</v>
+        <v>733</v>
       </c>
       <c r="B788" t="s">
-        <v>748</v>
+        <v>734</v>
       </c>
       <c r="C788" t="s">
         <v>725</v>
@@ -69931,10 +70350,10 @@
     </row>
     <row r="789" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A789" t="s">
-        <v>749</v>
+        <v>735</v>
       </c>
       <c r="B789" t="s">
-        <v>750</v>
+        <v>736</v>
       </c>
       <c r="C789" t="s">
         <v>725</v>
@@ -69969,16 +70388,16 @@
     </row>
     <row r="790" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A790" t="s">
-        <v>751</v>
+        <v>737</v>
       </c>
       <c r="B790" t="s">
-        <v>752</v>
+        <v>738</v>
       </c>
       <c r="C790" t="s">
         <v>725</v>
       </c>
       <c r="D790" t="s">
-        <v>753</v>
+        <v>726</v>
       </c>
       <c r="E790" t="s">
         <v>25</v>
@@ -70007,16 +70426,16 @@
     </row>
     <row r="791" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A791" t="s">
-        <v>754</v>
+        <v>739</v>
       </c>
       <c r="B791" t="s">
-        <v>755</v>
+        <v>740</v>
       </c>
       <c r="C791" t="s">
         <v>725</v>
       </c>
       <c r="D791" t="s">
-        <v>753</v>
+        <v>726</v>
       </c>
       <c r="E791" t="s">
         <v>25</v>
@@ -70045,16 +70464,16 @@
     </row>
     <row r="792" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A792" t="s">
-        <v>756</v>
+        <v>741</v>
       </c>
       <c r="B792" t="s">
-        <v>757</v>
+        <v>742</v>
       </c>
       <c r="C792" t="s">
         <v>725</v>
       </c>
       <c r="D792" t="s">
-        <v>753</v>
+        <v>726</v>
       </c>
       <c r="E792" t="s">
         <v>25</v>
@@ -70083,16 +70502,16 @@
     </row>
     <row r="793" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A793" t="s">
-        <v>758</v>
+        <v>743</v>
       </c>
       <c r="B793" t="s">
-        <v>759</v>
+        <v>744</v>
       </c>
       <c r="C793" t="s">
         <v>725</v>
       </c>
       <c r="D793" t="s">
-        <v>753</v>
+        <v>726</v>
       </c>
       <c r="E793" t="s">
         <v>25</v>
@@ -70121,16 +70540,16 @@
     </row>
     <row r="794" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A794" t="s">
-        <v>760</v>
+        <v>745</v>
       </c>
       <c r="B794" t="s">
-        <v>761</v>
+        <v>746</v>
       </c>
       <c r="C794" t="s">
         <v>725</v>
       </c>
       <c r="D794" t="s">
-        <v>753</v>
+        <v>726</v>
       </c>
       <c r="E794" t="s">
         <v>25</v>
@@ -70159,16 +70578,16 @@
     </row>
     <row r="795" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A795" t="s">
-        <v>762</v>
+        <v>747</v>
       </c>
       <c r="B795" t="s">
-        <v>763</v>
+        <v>748</v>
       </c>
       <c r="C795" t="s">
         <v>725</v>
       </c>
       <c r="D795" t="s">
-        <v>196</v>
+        <v>726</v>
       </c>
       <c r="E795" t="s">
         <v>25</v>
@@ -70197,16 +70616,16 @@
     </row>
     <row r="796" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A796" t="s">
-        <v>764</v>
+        <v>749</v>
       </c>
       <c r="B796" t="s">
-        <v>765</v>
+        <v>750</v>
       </c>
       <c r="C796" t="s">
         <v>725</v>
       </c>
       <c r="D796" t="s">
-        <v>196</v>
+        <v>726</v>
       </c>
       <c r="E796" t="s">
         <v>25</v>
@@ -70235,16 +70654,16 @@
     </row>
     <row r="797" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A797" t="s">
-        <v>766</v>
+        <v>751</v>
       </c>
       <c r="B797" t="s">
-        <v>767</v>
+        <v>752</v>
       </c>
       <c r="C797" t="s">
         <v>725</v>
       </c>
       <c r="D797" t="s">
-        <v>196</v>
+        <v>753</v>
       </c>
       <c r="E797" t="s">
         <v>25</v>
@@ -70273,16 +70692,16 @@
     </row>
     <row r="798" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A798" t="s">
-        <v>768</v>
+        <v>754</v>
       </c>
       <c r="B798" t="s">
-        <v>769</v>
+        <v>755</v>
       </c>
       <c r="C798" t="s">
         <v>725</v>
       </c>
       <c r="D798" t="s">
-        <v>770</v>
+        <v>753</v>
       </c>
       <c r="E798" t="s">
         <v>25</v>
@@ -70311,16 +70730,16 @@
     </row>
     <row r="799" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A799" t="s">
-        <v>771</v>
+        <v>756</v>
       </c>
       <c r="B799" t="s">
-        <v>772</v>
+        <v>757</v>
       </c>
       <c r="C799" t="s">
         <v>725</v>
       </c>
       <c r="D799" t="s">
-        <v>770</v>
+        <v>753</v>
       </c>
       <c r="E799" t="s">
         <v>25</v>
@@ -70349,16 +70768,16 @@
     </row>
     <row r="800" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A800" t="s">
-        <v>773</v>
+        <v>758</v>
       </c>
       <c r="B800" t="s">
-        <v>774</v>
+        <v>759</v>
       </c>
       <c r="C800" t="s">
         <v>725</v>
       </c>
       <c r="D800" t="s">
-        <v>775</v>
+        <v>753</v>
       </c>
       <c r="E800" t="s">
         <v>25</v>
@@ -70387,16 +70806,16 @@
     </row>
     <row r="801" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A801" t="s">
-        <v>776</v>
+        <v>760</v>
       </c>
       <c r="B801" t="s">
-        <v>777</v>
+        <v>761</v>
       </c>
       <c r="C801" t="s">
         <v>725</v>
       </c>
       <c r="D801" t="s">
-        <v>775</v>
+        <v>753</v>
       </c>
       <c r="E801" t="s">
         <v>25</v>
@@ -70425,16 +70844,16 @@
     </row>
     <row r="802" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A802" t="s">
-        <v>778</v>
+        <v>762</v>
       </c>
       <c r="B802" t="s">
-        <v>779</v>
+        <v>763</v>
       </c>
       <c r="C802" t="s">
         <v>725</v>
       </c>
       <c r="D802" t="s">
-        <v>775</v>
+        <v>196</v>
       </c>
       <c r="E802" t="s">
         <v>25</v>
@@ -70463,16 +70882,16 @@
     </row>
     <row r="803" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A803" t="s">
-        <v>780</v>
+        <v>764</v>
       </c>
       <c r="B803" t="s">
-        <v>781</v>
+        <v>765</v>
       </c>
       <c r="C803" t="s">
         <v>725</v>
       </c>
       <c r="D803" t="s">
-        <v>782</v>
+        <v>196</v>
       </c>
       <c r="E803" t="s">
         <v>25</v>
@@ -70501,16 +70920,16 @@
     </row>
     <row r="804" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A804" t="s">
-        <v>783</v>
+        <v>766</v>
       </c>
       <c r="B804" t="s">
-        <v>784</v>
+        <v>767</v>
       </c>
       <c r="C804" t="s">
         <v>725</v>
       </c>
       <c r="D804" t="s">
-        <v>782</v>
+        <v>196</v>
       </c>
       <c r="E804" t="s">
         <v>25</v>
@@ -70539,16 +70958,16 @@
     </row>
     <row r="805" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A805" t="s">
-        <v>785</v>
+        <v>768</v>
       </c>
       <c r="B805" t="s">
-        <v>786</v>
+        <v>769</v>
       </c>
       <c r="C805" t="s">
         <v>725</v>
       </c>
       <c r="D805" t="s">
-        <v>782</v>
+        <v>770</v>
       </c>
       <c r="E805" t="s">
         <v>25</v>
@@ -70577,16 +70996,16 @@
     </row>
     <row r="806" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A806" t="s">
-        <v>787</v>
+        <v>771</v>
       </c>
       <c r="B806" t="s">
-        <v>788</v>
+        <v>772</v>
       </c>
       <c r="C806" t="s">
         <v>725</v>
       </c>
       <c r="D806" t="s">
-        <v>782</v>
+        <v>770</v>
       </c>
       <c r="E806" t="s">
         <v>25</v>
@@ -70615,16 +71034,16 @@
     </row>
     <row r="807" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A807" t="s">
-        <v>789</v>
+        <v>773</v>
       </c>
       <c r="B807" t="s">
-        <v>790</v>
+        <v>774</v>
       </c>
       <c r="C807" t="s">
         <v>725</v>
       </c>
       <c r="D807" t="s">
-        <v>782</v>
+        <v>775</v>
       </c>
       <c r="E807" t="s">
         <v>25</v>
@@ -70653,16 +71072,16 @@
     </row>
     <row r="808" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A808" t="s">
-        <v>791</v>
+        <v>776</v>
       </c>
       <c r="B808" t="s">
-        <v>792</v>
+        <v>777</v>
       </c>
       <c r="C808" t="s">
         <v>725</v>
       </c>
       <c r="D808" t="s">
-        <v>782</v>
+        <v>775</v>
       </c>
       <c r="E808" t="s">
         <v>25</v>
@@ -70691,16 +71110,16 @@
     </row>
     <row r="809" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A809" t="s">
-        <v>793</v>
+        <v>778</v>
       </c>
       <c r="B809" t="s">
-        <v>794</v>
+        <v>779</v>
       </c>
       <c r="C809" t="s">
         <v>725</v>
       </c>
       <c r="D809" t="s">
-        <v>782</v>
+        <v>775</v>
       </c>
       <c r="E809" t="s">
         <v>25</v>
@@ -70729,10 +71148,10 @@
     </row>
     <row r="810" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A810" t="s">
-        <v>795</v>
+        <v>780</v>
       </c>
       <c r="B810" t="s">
-        <v>796</v>
+        <v>781</v>
       </c>
       <c r="C810" t="s">
         <v>725</v>
@@ -70767,10 +71186,10 @@
     </row>
     <row r="811" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A811" t="s">
-        <v>797</v>
+        <v>783</v>
       </c>
       <c r="B811" t="s">
-        <v>798</v>
+        <v>784</v>
       </c>
       <c r="C811" t="s">
         <v>725</v>
@@ -70805,10 +71224,10 @@
     </row>
     <row r="812" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A812" t="s">
-        <v>799</v>
+        <v>785</v>
       </c>
       <c r="B812" t="s">
-        <v>800</v>
+        <v>786</v>
       </c>
       <c r="C812" t="s">
         <v>725</v>
@@ -70843,10 +71262,10 @@
     </row>
     <row r="813" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A813" t="s">
-        <v>801</v>
+        <v>787</v>
       </c>
       <c r="B813" t="s">
-        <v>802</v>
+        <v>788</v>
       </c>
       <c r="C813" t="s">
         <v>725</v>
@@ -70881,10 +71300,10 @@
     </row>
     <row r="814" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A814" t="s">
-        <v>803</v>
+        <v>789</v>
       </c>
       <c r="B814" t="s">
-        <v>804</v>
+        <v>790</v>
       </c>
       <c r="C814" t="s">
         <v>725</v>
@@ -70919,16 +71338,16 @@
     </row>
     <row r="815" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A815" t="s">
-        <v>805</v>
+        <v>791</v>
       </c>
       <c r="B815" t="s">
-        <v>806</v>
+        <v>792</v>
       </c>
       <c r="C815" t="s">
         <v>725</v>
       </c>
       <c r="D815" t="s">
-        <v>807</v>
+        <v>782</v>
       </c>
       <c r="E815" t="s">
         <v>25</v>
@@ -70957,16 +71376,16 @@
     </row>
     <row r="816" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A816" t="s">
-        <v>808</v>
+        <v>793</v>
       </c>
       <c r="B816" t="s">
-        <v>809</v>
+        <v>794</v>
       </c>
       <c r="C816" t="s">
         <v>725</v>
       </c>
       <c r="D816" t="s">
-        <v>807</v>
+        <v>782</v>
       </c>
       <c r="E816" t="s">
         <v>25</v>
@@ -70995,16 +71414,16 @@
     </row>
     <row r="817" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A817" t="s">
-        <v>810</v>
+        <v>795</v>
       </c>
       <c r="B817" t="s">
-        <v>811</v>
+        <v>796</v>
       </c>
       <c r="C817" t="s">
         <v>725</v>
       </c>
       <c r="D817" t="s">
-        <v>807</v>
+        <v>782</v>
       </c>
       <c r="E817" t="s">
         <v>25</v>
@@ -71033,16 +71452,16 @@
     </row>
     <row r="818" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A818" t="s">
-        <v>812</v>
+        <v>797</v>
       </c>
       <c r="B818" t="s">
-        <v>813</v>
+        <v>798</v>
       </c>
       <c r="C818" t="s">
         <v>725</v>
       </c>
       <c r="D818" t="s">
-        <v>807</v>
+        <v>782</v>
       </c>
       <c r="E818" t="s">
         <v>25</v>
@@ -71071,16 +71490,16 @@
     </row>
     <row r="819" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A819" t="s">
-        <v>814</v>
+        <v>799</v>
       </c>
       <c r="B819" t="s">
-        <v>815</v>
+        <v>800</v>
       </c>
       <c r="C819" t="s">
         <v>725</v>
       </c>
       <c r="D819" t="s">
-        <v>807</v>
+        <v>782</v>
       </c>
       <c r="E819" t="s">
         <v>25</v>
@@ -71109,16 +71528,16 @@
     </row>
     <row r="820" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A820" t="s">
-        <v>816</v>
+        <v>801</v>
       </c>
       <c r="B820" t="s">
-        <v>817</v>
+        <v>802</v>
       </c>
       <c r="C820" t="s">
         <v>725</v>
       </c>
       <c r="D820" t="s">
-        <v>818</v>
+        <v>782</v>
       </c>
       <c r="E820" t="s">
         <v>25</v>
@@ -71147,16 +71566,16 @@
     </row>
     <row r="821" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A821" t="s">
-        <v>819</v>
+        <v>803</v>
       </c>
       <c r="B821" t="s">
-        <v>820</v>
+        <v>804</v>
       </c>
       <c r="C821" t="s">
         <v>725</v>
       </c>
       <c r="D821" t="s">
-        <v>818</v>
+        <v>782</v>
       </c>
       <c r="E821" t="s">
         <v>25</v>
@@ -71185,16 +71604,16 @@
     </row>
     <row r="822" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A822" t="s">
-        <v>821</v>
+        <v>805</v>
       </c>
       <c r="B822" t="s">
-        <v>822</v>
+        <v>806</v>
       </c>
       <c r="C822" t="s">
-        <v>823</v>
+        <v>725</v>
       </c>
       <c r="D822" t="s">
-        <v>824</v>
+        <v>807</v>
       </c>
       <c r="E822" t="s">
         <v>25</v>
@@ -71223,16 +71642,16 @@
     </row>
     <row r="823" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A823" t="s">
-        <v>825</v>
+        <v>808</v>
       </c>
       <c r="B823" t="s">
-        <v>826</v>
+        <v>809</v>
       </c>
       <c r="C823" t="s">
-        <v>823</v>
+        <v>725</v>
       </c>
       <c r="D823" t="s">
-        <v>824</v>
+        <v>807</v>
       </c>
       <c r="E823" t="s">
         <v>25</v>
@@ -71261,16 +71680,16 @@
     </row>
     <row r="824" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A824" t="s">
-        <v>827</v>
+        <v>810</v>
       </c>
       <c r="B824" t="s">
-        <v>828</v>
+        <v>811</v>
       </c>
       <c r="C824" t="s">
-        <v>823</v>
+        <v>725</v>
       </c>
       <c r="D824" t="s">
-        <v>824</v>
+        <v>807</v>
       </c>
       <c r="E824" t="s">
         <v>25</v>
@@ -71299,16 +71718,16 @@
     </row>
     <row r="825" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A825" t="s">
-        <v>829</v>
+        <v>812</v>
       </c>
       <c r="B825" t="s">
-        <v>830</v>
+        <v>813</v>
       </c>
       <c r="C825" t="s">
-        <v>823</v>
+        <v>725</v>
       </c>
       <c r="D825" t="s">
-        <v>824</v>
+        <v>807</v>
       </c>
       <c r="E825" t="s">
         <v>25</v>
@@ -71337,16 +71756,16 @@
     </row>
     <row r="826" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A826" t="s">
-        <v>831</v>
+        <v>814</v>
       </c>
       <c r="B826" t="s">
-        <v>832</v>
+        <v>815</v>
       </c>
       <c r="C826" t="s">
-        <v>823</v>
+        <v>725</v>
       </c>
       <c r="D826" t="s">
-        <v>824</v>
+        <v>807</v>
       </c>
       <c r="E826" t="s">
         <v>25</v>
@@ -71375,16 +71794,16 @@
     </row>
     <row r="827" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A827" t="s">
-        <v>833</v>
+        <v>816</v>
       </c>
       <c r="B827" t="s">
-        <v>834</v>
+        <v>817</v>
       </c>
       <c r="C827" t="s">
-        <v>823</v>
+        <v>725</v>
       </c>
       <c r="D827" t="s">
-        <v>824</v>
+        <v>818</v>
       </c>
       <c r="E827" t="s">
         <v>25</v>
@@ -71413,16 +71832,16 @@
     </row>
     <row r="828" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A828" t="s">
-        <v>835</v>
+        <v>819</v>
       </c>
       <c r="B828" t="s">
-        <v>836</v>
+        <v>820</v>
       </c>
       <c r="C828" t="s">
-        <v>823</v>
+        <v>725</v>
       </c>
       <c r="D828" t="s">
-        <v>837</v>
+        <v>818</v>
       </c>
       <c r="E828" t="s">
         <v>25</v>
@@ -71451,16 +71870,16 @@
     </row>
     <row r="829" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A829" t="s">
-        <v>838</v>
+        <v>821</v>
       </c>
       <c r="B829" t="s">
-        <v>839</v>
+        <v>822</v>
       </c>
       <c r="C829" t="s">
         <v>823</v>
       </c>
       <c r="D829" t="s">
-        <v>837</v>
+        <v>824</v>
       </c>
       <c r="E829" t="s">
         <v>25</v>
@@ -71489,16 +71908,16 @@
     </row>
     <row r="830" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A830" t="s">
-        <v>840</v>
+        <v>825</v>
       </c>
       <c r="B830" t="s">
-        <v>841</v>
+        <v>826</v>
       </c>
       <c r="C830" t="s">
         <v>823</v>
       </c>
       <c r="D830" t="s">
-        <v>837</v>
+        <v>824</v>
       </c>
       <c r="E830" t="s">
         <v>25</v>
@@ -71527,16 +71946,16 @@
     </row>
     <row r="831" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A831" t="s">
-        <v>842</v>
+        <v>827</v>
       </c>
       <c r="B831" t="s">
-        <v>843</v>
+        <v>828</v>
       </c>
       <c r="C831" t="s">
         <v>823</v>
       </c>
       <c r="D831" t="s">
-        <v>837</v>
+        <v>824</v>
       </c>
       <c r="E831" t="s">
         <v>25</v>
@@ -71565,16 +71984,16 @@
     </row>
     <row r="832" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A832" t="s">
-        <v>844</v>
+        <v>829</v>
       </c>
       <c r="B832" t="s">
-        <v>845</v>
+        <v>830</v>
       </c>
       <c r="C832" t="s">
         <v>823</v>
       </c>
       <c r="D832" t="s">
-        <v>837</v>
+        <v>824</v>
       </c>
       <c r="E832" t="s">
         <v>25</v>
@@ -71603,16 +72022,16 @@
     </row>
     <row r="833" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A833" t="s">
-        <v>846</v>
+        <v>831</v>
       </c>
       <c r="B833" t="s">
-        <v>847</v>
+        <v>832</v>
       </c>
       <c r="C833" t="s">
         <v>823</v>
       </c>
       <c r="D833" t="s">
-        <v>848</v>
+        <v>824</v>
       </c>
       <c r="E833" t="s">
         <v>25</v>
@@ -71641,16 +72060,16 @@
     </row>
     <row r="834" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A834" t="s">
-        <v>849</v>
+        <v>833</v>
       </c>
       <c r="B834" t="s">
-        <v>850</v>
+        <v>834</v>
       </c>
       <c r="C834" t="s">
         <v>823</v>
       </c>
       <c r="D834" t="s">
-        <v>848</v>
+        <v>824</v>
       </c>
       <c r="E834" t="s">
         <v>25</v>
@@ -71679,16 +72098,16 @@
     </row>
     <row r="835" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A835" t="s">
-        <v>851</v>
+        <v>835</v>
       </c>
       <c r="B835" t="s">
-        <v>852</v>
+        <v>836</v>
       </c>
       <c r="C835" t="s">
         <v>823</v>
       </c>
       <c r="D835" t="s">
-        <v>848</v>
+        <v>837</v>
       </c>
       <c r="E835" t="s">
         <v>25</v>
@@ -71717,16 +72136,16 @@
     </row>
     <row r="836" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A836" t="s">
-        <v>853</v>
+        <v>838</v>
       </c>
       <c r="B836" t="s">
-        <v>854</v>
+        <v>839</v>
       </c>
       <c r="C836" t="s">
         <v>823</v>
       </c>
       <c r="D836" t="s">
-        <v>855</v>
+        <v>837</v>
       </c>
       <c r="E836" t="s">
         <v>25</v>
@@ -71755,16 +72174,16 @@
     </row>
     <row r="837" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A837" t="s">
-        <v>856</v>
+        <v>840</v>
       </c>
       <c r="B837" t="s">
-        <v>857</v>
+        <v>841</v>
       </c>
       <c r="C837" t="s">
         <v>823</v>
       </c>
       <c r="D837" t="s">
-        <v>855</v>
+        <v>837</v>
       </c>
       <c r="E837" t="s">
         <v>25</v>
@@ -71793,16 +72212,16 @@
     </row>
     <row r="838" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A838" t="s">
-        <v>858</v>
+        <v>842</v>
       </c>
       <c r="B838" t="s">
-        <v>859</v>
+        <v>843</v>
       </c>
       <c r="C838" t="s">
         <v>823</v>
       </c>
       <c r="D838" t="s">
-        <v>860</v>
+        <v>837</v>
       </c>
       <c r="E838" t="s">
         <v>25</v>
@@ -71831,16 +72250,16 @@
     </row>
     <row r="839" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A839" t="s">
-        <v>861</v>
+        <v>844</v>
       </c>
       <c r="B839" t="s">
-        <v>862</v>
+        <v>845</v>
       </c>
       <c r="C839" t="s">
         <v>823</v>
       </c>
       <c r="D839" t="s">
-        <v>860</v>
+        <v>837</v>
       </c>
       <c r="E839" t="s">
         <v>25</v>
@@ -71869,16 +72288,16 @@
     </row>
     <row r="840" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A840" t="s">
-        <v>863</v>
+        <v>846</v>
       </c>
       <c r="B840" t="s">
-        <v>864</v>
+        <v>847</v>
       </c>
       <c r="C840" t="s">
         <v>823</v>
       </c>
       <c r="D840" t="s">
-        <v>860</v>
+        <v>848</v>
       </c>
       <c r="E840" t="s">
         <v>25</v>
@@ -71907,16 +72326,16 @@
     </row>
     <row r="841" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A841" t="s">
-        <v>865</v>
+        <v>849</v>
       </c>
       <c r="B841" t="s">
-        <v>866</v>
+        <v>850</v>
       </c>
       <c r="C841" t="s">
         <v>823</v>
       </c>
       <c r="D841" t="s">
-        <v>860</v>
+        <v>848</v>
       </c>
       <c r="E841" t="s">
         <v>25</v>
@@ -71945,16 +72364,16 @@
     </row>
     <row r="842" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A842" t="s">
-        <v>867</v>
+        <v>851</v>
       </c>
       <c r="B842" t="s">
-        <v>868</v>
+        <v>852</v>
       </c>
       <c r="C842" t="s">
         <v>823</v>
       </c>
       <c r="D842" t="s">
-        <v>869</v>
+        <v>848</v>
       </c>
       <c r="E842" t="s">
         <v>25</v>
@@ -71983,16 +72402,16 @@
     </row>
     <row r="843" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A843" t="s">
-        <v>870</v>
+        <v>853</v>
       </c>
       <c r="B843" t="s">
-        <v>871</v>
+        <v>854</v>
       </c>
       <c r="C843" t="s">
         <v>823</v>
       </c>
       <c r="D843" t="s">
-        <v>869</v>
+        <v>855</v>
       </c>
       <c r="E843" t="s">
         <v>25</v>
@@ -72021,16 +72440,16 @@
     </row>
     <row r="844" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A844" t="s">
-        <v>872</v>
+        <v>856</v>
       </c>
       <c r="B844" t="s">
-        <v>873</v>
+        <v>857</v>
       </c>
       <c r="C844" t="s">
         <v>823</v>
       </c>
       <c r="D844" t="s">
-        <v>869</v>
+        <v>855</v>
       </c>
       <c r="E844" t="s">
         <v>25</v>
@@ -72059,16 +72478,16 @@
     </row>
     <row r="845" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A845" t="s">
-        <v>874</v>
+        <v>858</v>
       </c>
       <c r="B845" t="s">
-        <v>875</v>
+        <v>859</v>
       </c>
       <c r="C845" t="s">
         <v>823</v>
       </c>
       <c r="D845" t="s">
-        <v>869</v>
+        <v>860</v>
       </c>
       <c r="E845" t="s">
         <v>25</v>
@@ -72097,16 +72516,16 @@
     </row>
     <row r="846" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A846" t="s">
-        <v>876</v>
+        <v>861</v>
       </c>
       <c r="B846" t="s">
-        <v>877</v>
+        <v>862</v>
       </c>
       <c r="C846" t="s">
         <v>823</v>
       </c>
       <c r="D846" t="s">
-        <v>869</v>
+        <v>860</v>
       </c>
       <c r="E846" t="s">
         <v>25</v>
@@ -72135,16 +72554,16 @@
     </row>
     <row r="847" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A847" t="s">
-        <v>878</v>
+        <v>863</v>
       </c>
       <c r="B847" t="s">
-        <v>879</v>
+        <v>864</v>
       </c>
       <c r="C847" t="s">
-        <v>880</v>
+        <v>823</v>
       </c>
       <c r="D847" t="s">
-        <v>25</v>
+        <v>860</v>
       </c>
       <c r="E847" t="s">
         <v>25</v>
@@ -72173,16 +72592,16 @@
     </row>
     <row r="848" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A848" t="s">
-        <v>881</v>
+        <v>865</v>
       </c>
       <c r="B848" t="s">
-        <v>882</v>
+        <v>866</v>
       </c>
       <c r="C848" t="s">
-        <v>880</v>
+        <v>823</v>
       </c>
       <c r="D848" t="s">
-        <v>25</v>
+        <v>860</v>
       </c>
       <c r="E848" t="s">
         <v>25</v>
@@ -72211,16 +72630,16 @@
     </row>
     <row r="849" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A849" t="s">
-        <v>883</v>
+        <v>867</v>
       </c>
       <c r="B849" t="s">
-        <v>884</v>
+        <v>868</v>
       </c>
       <c r="C849" t="s">
-        <v>880</v>
+        <v>823</v>
       </c>
       <c r="D849" t="s">
-        <v>25</v>
+        <v>869</v>
       </c>
       <c r="E849" t="s">
         <v>25</v>
@@ -72249,16 +72668,16 @@
     </row>
     <row r="850" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A850" t="s">
-        <v>885</v>
+        <v>870</v>
       </c>
       <c r="B850" t="s">
-        <v>886</v>
+        <v>871</v>
       </c>
       <c r="C850" t="s">
-        <v>880</v>
+        <v>823</v>
       </c>
       <c r="D850" t="s">
-        <v>25</v>
+        <v>869</v>
       </c>
       <c r="E850" t="s">
         <v>25</v>
@@ -72287,16 +72706,16 @@
     </row>
     <row r="851" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A851" t="s">
-        <v>887</v>
+        <v>872</v>
       </c>
       <c r="B851" t="s">
-        <v>888</v>
+        <v>873</v>
       </c>
       <c r="C851" t="s">
-        <v>880</v>
+        <v>823</v>
       </c>
       <c r="D851" t="s">
-        <v>25</v>
+        <v>869</v>
       </c>
       <c r="E851" t="s">
         <v>25</v>
@@ -72325,16 +72744,16 @@
     </row>
     <row r="852" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A852" t="s">
-        <v>889</v>
+        <v>874</v>
       </c>
       <c r="B852" t="s">
-        <v>890</v>
+        <v>875</v>
       </c>
       <c r="C852" t="s">
-        <v>880</v>
+        <v>823</v>
       </c>
       <c r="D852" t="s">
-        <v>25</v>
+        <v>869</v>
       </c>
       <c r="E852" t="s">
         <v>25</v>
@@ -72363,16 +72782,16 @@
     </row>
     <row r="853" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A853" t="s">
-        <v>891</v>
+        <v>876</v>
       </c>
       <c r="B853" t="s">
-        <v>892</v>
+        <v>877</v>
       </c>
       <c r="C853" t="s">
-        <v>880</v>
+        <v>823</v>
       </c>
       <c r="D853" t="s">
-        <v>25</v>
+        <v>869</v>
       </c>
       <c r="E853" t="s">
         <v>25</v>
@@ -72401,10 +72820,10 @@
     </row>
     <row r="854" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A854" t="s">
-        <v>893</v>
+        <v>878</v>
       </c>
       <c r="B854" t="s">
-        <v>894</v>
+        <v>879</v>
       </c>
       <c r="C854" t="s">
         <v>880</v>
@@ -72439,10 +72858,10 @@
     </row>
     <row r="855" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A855" t="s">
-        <v>895</v>
+        <v>881</v>
       </c>
       <c r="B855" t="s">
-        <v>896</v>
+        <v>882</v>
       </c>
       <c r="C855" t="s">
         <v>880</v>
@@ -72477,10 +72896,10 @@
     </row>
     <row r="856" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A856" t="s">
-        <v>897</v>
+        <v>883</v>
       </c>
       <c r="B856" t="s">
-        <v>898</v>
+        <v>884</v>
       </c>
       <c r="C856" t="s">
         <v>880</v>
@@ -72515,10 +72934,10 @@
     </row>
     <row r="857" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A857" t="s">
-        <v>899</v>
+        <v>885</v>
       </c>
       <c r="B857" t="s">
-        <v>900</v>
+        <v>886</v>
       </c>
       <c r="C857" t="s">
         <v>880</v>
@@ -72553,10 +72972,10 @@
     </row>
     <row r="858" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A858" t="s">
-        <v>901</v>
+        <v>887</v>
       </c>
       <c r="B858" t="s">
-        <v>902</v>
+        <v>888</v>
       </c>
       <c r="C858" t="s">
         <v>880</v>
@@ -72591,10 +73010,10 @@
     </row>
     <row r="859" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A859" t="s">
-        <v>903</v>
+        <v>889</v>
       </c>
       <c r="B859" t="s">
-        <v>904</v>
+        <v>890</v>
       </c>
       <c r="C859" t="s">
         <v>880</v>
@@ -72629,10 +73048,10 @@
     </row>
     <row r="860" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A860" t="s">
-        <v>905</v>
+        <v>891</v>
       </c>
       <c r="B860" t="s">
-        <v>906</v>
+        <v>892</v>
       </c>
       <c r="C860" t="s">
         <v>880</v>
@@ -72667,10 +73086,10 @@
     </row>
     <row r="861" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A861" t="s">
-        <v>907</v>
+        <v>893</v>
       </c>
       <c r="B861" t="s">
-        <v>908</v>
+        <v>894</v>
       </c>
       <c r="C861" t="s">
         <v>880</v>
@@ -72705,16 +73124,16 @@
     </row>
     <row r="862" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A862" t="s">
-        <v>909</v>
+        <v>895</v>
       </c>
       <c r="B862" t="s">
-        <v>910</v>
+        <v>896</v>
       </c>
       <c r="C862" t="s">
-        <v>911</v>
+        <v>880</v>
       </c>
       <c r="D862" t="s">
-        <v>912</v>
+        <v>25</v>
       </c>
       <c r="E862" t="s">
         <v>25</v>
@@ -72743,16 +73162,16 @@
     </row>
     <row r="863" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A863" t="s">
-        <v>913</v>
+        <v>897</v>
       </c>
       <c r="B863" t="s">
-        <v>914</v>
+        <v>898</v>
       </c>
       <c r="C863" t="s">
-        <v>911</v>
+        <v>880</v>
       </c>
       <c r="D863" t="s">
-        <v>912</v>
+        <v>25</v>
       </c>
       <c r="E863" t="s">
         <v>25</v>
@@ -72781,16 +73200,16 @@
     </row>
     <row r="864" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A864" t="s">
-        <v>915</v>
+        <v>899</v>
       </c>
       <c r="B864" t="s">
-        <v>916</v>
+        <v>900</v>
       </c>
       <c r="C864" t="s">
-        <v>911</v>
+        <v>880</v>
       </c>
       <c r="D864" t="s">
-        <v>912</v>
+        <v>25</v>
       </c>
       <c r="E864" t="s">
         <v>25</v>
@@ -72819,16 +73238,16 @@
     </row>
     <row r="865" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A865" t="s">
-        <v>917</v>
+        <v>901</v>
       </c>
       <c r="B865" t="s">
-        <v>918</v>
+        <v>902</v>
       </c>
       <c r="C865" t="s">
-        <v>911</v>
+        <v>880</v>
       </c>
       <c r="D865" t="s">
-        <v>912</v>
+        <v>25</v>
       </c>
       <c r="E865" t="s">
         <v>25</v>
@@ -72857,16 +73276,16 @@
     </row>
     <row r="866" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A866" t="s">
-        <v>919</v>
+        <v>903</v>
       </c>
       <c r="B866" t="s">
-        <v>920</v>
+        <v>904</v>
       </c>
       <c r="C866" t="s">
-        <v>911</v>
+        <v>880</v>
       </c>
       <c r="D866" t="s">
-        <v>921</v>
+        <v>25</v>
       </c>
       <c r="E866" t="s">
         <v>25</v>
@@ -72895,16 +73314,16 @@
     </row>
     <row r="867" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A867" t="s">
-        <v>922</v>
+        <v>905</v>
       </c>
       <c r="B867" t="s">
-        <v>923</v>
+        <v>906</v>
       </c>
       <c r="C867" t="s">
-        <v>911</v>
+        <v>880</v>
       </c>
       <c r="D867" t="s">
-        <v>921</v>
+        <v>25</v>
       </c>
       <c r="E867" t="s">
         <v>25</v>
@@ -72933,16 +73352,16 @@
     </row>
     <row r="868" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A868" t="s">
-        <v>924</v>
+        <v>907</v>
       </c>
       <c r="B868" t="s">
-        <v>925</v>
+        <v>908</v>
       </c>
       <c r="C868" t="s">
-        <v>911</v>
+        <v>880</v>
       </c>
       <c r="D868" t="s">
-        <v>921</v>
+        <v>25</v>
       </c>
       <c r="E868" t="s">
         <v>25</v>
@@ -72971,16 +73390,16 @@
     </row>
     <row r="869" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A869" t="s">
-        <v>926</v>
+        <v>909</v>
       </c>
       <c r="B869" t="s">
-        <v>927</v>
+        <v>910</v>
       </c>
       <c r="C869" t="s">
         <v>911</v>
       </c>
       <c r="D869" t="s">
-        <v>921</v>
+        <v>912</v>
       </c>
       <c r="E869" t="s">
         <v>25</v>
@@ -73009,16 +73428,16 @@
     </row>
     <row r="870" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A870" t="s">
-        <v>928</v>
+        <v>913</v>
       </c>
       <c r="B870" t="s">
-        <v>929</v>
+        <v>914</v>
       </c>
       <c r="C870" t="s">
         <v>911</v>
       </c>
       <c r="D870" t="s">
-        <v>921</v>
+        <v>912</v>
       </c>
       <c r="E870" t="s">
         <v>25</v>
@@ -73047,16 +73466,16 @@
     </row>
     <row r="871" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A871" t="s">
-        <v>930</v>
+        <v>915</v>
       </c>
       <c r="B871" t="s">
-        <v>931</v>
+        <v>916</v>
       </c>
       <c r="C871" t="s">
         <v>911</v>
       </c>
       <c r="D871" t="s">
-        <v>921</v>
+        <v>912</v>
       </c>
       <c r="E871" t="s">
         <v>25</v>
@@ -73085,16 +73504,16 @@
     </row>
     <row r="872" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A872" t="s">
-        <v>932</v>
+        <v>917</v>
       </c>
       <c r="B872" t="s">
-        <v>933</v>
+        <v>918</v>
       </c>
       <c r="C872" t="s">
         <v>911</v>
       </c>
       <c r="D872" t="s">
-        <v>921</v>
+        <v>912</v>
       </c>
       <c r="E872" t="s">
         <v>25</v>
@@ -73123,16 +73542,16 @@
     </row>
     <row r="873" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A873" t="s">
-        <v>934</v>
+        <v>919</v>
       </c>
       <c r="B873" t="s">
-        <v>935</v>
+        <v>920</v>
       </c>
       <c r="C873" t="s">
-        <v>936</v>
+        <v>911</v>
       </c>
       <c r="D873" t="s">
-        <v>937</v>
+        <v>921</v>
       </c>
       <c r="E873" t="s">
         <v>25</v>
@@ -73161,16 +73580,16 @@
     </row>
     <row r="874" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A874" t="s">
-        <v>938</v>
+        <v>922</v>
       </c>
       <c r="B874" t="s">
-        <v>939</v>
+        <v>923</v>
       </c>
       <c r="C874" t="s">
-        <v>936</v>
+        <v>911</v>
       </c>
       <c r="D874" t="s">
-        <v>937</v>
+        <v>921</v>
       </c>
       <c r="E874" t="s">
         <v>25</v>
@@ -73199,16 +73618,16 @@
     </row>
     <row r="875" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A875" t="s">
-        <v>940</v>
+        <v>924</v>
       </c>
       <c r="B875" t="s">
-        <v>941</v>
+        <v>925</v>
       </c>
       <c r="C875" t="s">
-        <v>936</v>
+        <v>911</v>
       </c>
       <c r="D875" t="s">
-        <v>937</v>
+        <v>921</v>
       </c>
       <c r="E875" t="s">
         <v>25</v>
@@ -73237,16 +73656,16 @@
     </row>
     <row r="876" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A876" t="s">
-        <v>942</v>
+        <v>926</v>
       </c>
       <c r="B876" t="s">
-        <v>943</v>
+        <v>927</v>
       </c>
       <c r="C876" t="s">
-        <v>936</v>
+        <v>911</v>
       </c>
       <c r="D876" t="s">
-        <v>937</v>
+        <v>921</v>
       </c>
       <c r="E876" t="s">
         <v>25</v>
@@ -73275,16 +73694,16 @@
     </row>
     <row r="877" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A877" t="s">
-        <v>944</v>
+        <v>928</v>
       </c>
       <c r="B877" t="s">
-        <v>945</v>
+        <v>929</v>
       </c>
       <c r="C877" t="s">
-        <v>936</v>
+        <v>911</v>
       </c>
       <c r="D877" t="s">
-        <v>937</v>
+        <v>921</v>
       </c>
       <c r="E877" t="s">
         <v>25</v>
@@ -73313,16 +73732,16 @@
     </row>
     <row r="878" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A878" t="s">
-        <v>946</v>
+        <v>930</v>
       </c>
       <c r="B878" t="s">
-        <v>947</v>
+        <v>931</v>
       </c>
       <c r="C878" t="s">
-        <v>936</v>
+        <v>911</v>
       </c>
       <c r="D878" t="s">
-        <v>937</v>
+        <v>921</v>
       </c>
       <c r="E878" t="s">
         <v>25</v>
@@ -73351,16 +73770,16 @@
     </row>
     <row r="879" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A879" t="s">
-        <v>948</v>
+        <v>932</v>
       </c>
       <c r="B879" t="s">
-        <v>949</v>
+        <v>933</v>
       </c>
       <c r="C879" t="s">
-        <v>936</v>
+        <v>911</v>
       </c>
       <c r="D879" t="s">
-        <v>937</v>
+        <v>921</v>
       </c>
       <c r="E879" t="s">
         <v>25</v>
@@ -73389,10 +73808,10 @@
     </row>
     <row r="880" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A880" t="s">
-        <v>950</v>
+        <v>934</v>
       </c>
       <c r="B880" t="s">
-        <v>951</v>
+        <v>935</v>
       </c>
       <c r="C880" t="s">
         <v>936</v>
@@ -73427,16 +73846,16 @@
     </row>
     <row r="881" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A881" t="s">
-        <v>952</v>
+        <v>938</v>
       </c>
       <c r="B881" t="s">
-        <v>953</v>
+        <v>939</v>
       </c>
       <c r="C881" t="s">
         <v>936</v>
       </c>
       <c r="D881" t="s">
-        <v>954</v>
+        <v>937</v>
       </c>
       <c r="E881" t="s">
         <v>25</v>
@@ -73465,16 +73884,16 @@
     </row>
     <row r="882" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A882" t="s">
-        <v>955</v>
+        <v>940</v>
       </c>
       <c r="B882" t="s">
-        <v>956</v>
+        <v>941</v>
       </c>
       <c r="C882" t="s">
         <v>936</v>
       </c>
       <c r="D882" t="s">
-        <v>954</v>
+        <v>937</v>
       </c>
       <c r="E882" t="s">
         <v>25</v>
@@ -73503,16 +73922,16 @@
     </row>
     <row r="883" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A883" t="s">
-        <v>957</v>
+        <v>942</v>
       </c>
       <c r="B883" t="s">
-        <v>958</v>
+        <v>943</v>
       </c>
       <c r="C883" t="s">
         <v>936</v>
       </c>
       <c r="D883" t="s">
-        <v>954</v>
+        <v>937</v>
       </c>
       <c r="E883" t="s">
         <v>25</v>
@@ -73541,16 +73960,16 @@
     </row>
     <row r="884" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A884" t="s">
-        <v>959</v>
+        <v>944</v>
       </c>
       <c r="B884" t="s">
-        <v>960</v>
+        <v>945</v>
       </c>
       <c r="C884" t="s">
         <v>936</v>
       </c>
       <c r="D884" t="s">
-        <v>954</v>
+        <v>937</v>
       </c>
       <c r="E884" t="s">
         <v>25</v>
@@ -73579,16 +73998,16 @@
     </row>
     <row r="885" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A885" t="s">
-        <v>961</v>
+        <v>946</v>
       </c>
       <c r="B885" t="s">
-        <v>962</v>
+        <v>947</v>
       </c>
       <c r="C885" t="s">
         <v>936</v>
       </c>
       <c r="D885" t="s">
-        <v>954</v>
+        <v>937</v>
       </c>
       <c r="E885" t="s">
         <v>25</v>
@@ -73617,16 +74036,16 @@
     </row>
     <row r="886" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A886" t="s">
-        <v>963</v>
+        <v>948</v>
       </c>
       <c r="B886" t="s">
-        <v>964</v>
+        <v>949</v>
       </c>
       <c r="C886" t="s">
         <v>936</v>
       </c>
       <c r="D886" t="s">
-        <v>965</v>
+        <v>937</v>
       </c>
       <c r="E886" t="s">
         <v>25</v>
@@ -73655,16 +74074,16 @@
     </row>
     <row r="887" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A887" t="s">
-        <v>966</v>
+        <v>950</v>
       </c>
       <c r="B887" t="s">
-        <v>967</v>
+        <v>951</v>
       </c>
       <c r="C887" t="s">
         <v>936</v>
       </c>
       <c r="D887" t="s">
-        <v>965</v>
+        <v>937</v>
       </c>
       <c r="E887" t="s">
         <v>25</v>
@@ -73693,16 +74112,16 @@
     </row>
     <row r="888" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A888" t="s">
-        <v>968</v>
+        <v>952</v>
       </c>
       <c r="B888" t="s">
-        <v>969</v>
+        <v>953</v>
       </c>
       <c r="C888" t="s">
         <v>936</v>
       </c>
       <c r="D888" t="s">
-        <v>970</v>
+        <v>954</v>
       </c>
       <c r="E888" t="s">
         <v>25</v>
@@ -73731,16 +74150,16 @@
     </row>
     <row r="889" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A889" t="s">
-        <v>971</v>
+        <v>955</v>
       </c>
       <c r="B889" t="s">
-        <v>972</v>
+        <v>956</v>
       </c>
       <c r="C889" t="s">
         <v>936</v>
       </c>
       <c r="D889" t="s">
-        <v>970</v>
+        <v>954</v>
       </c>
       <c r="E889" t="s">
         <v>25</v>
@@ -73769,16 +74188,16 @@
     </row>
     <row r="890" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A890" t="s">
-        <v>973</v>
+        <v>957</v>
       </c>
       <c r="B890" t="s">
-        <v>974</v>
+        <v>958</v>
       </c>
       <c r="C890" t="s">
         <v>936</v>
       </c>
       <c r="D890" t="s">
-        <v>970</v>
+        <v>954</v>
       </c>
       <c r="E890" t="s">
         <v>25</v>
@@ -73807,16 +74226,16 @@
     </row>
     <row r="891" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A891" t="s">
-        <v>975</v>
+        <v>959</v>
       </c>
       <c r="B891" t="s">
-        <v>976</v>
+        <v>960</v>
       </c>
       <c r="C891" t="s">
         <v>936</v>
       </c>
       <c r="D891" t="s">
-        <v>970</v>
+        <v>954</v>
       </c>
       <c r="E891" t="s">
         <v>25</v>
@@ -73845,16 +74264,16 @@
     </row>
     <row r="892" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A892" t="s">
-        <v>977</v>
+        <v>961</v>
       </c>
       <c r="B892" t="s">
-        <v>978</v>
+        <v>962</v>
       </c>
       <c r="C892" t="s">
         <v>936</v>
       </c>
       <c r="D892" t="s">
-        <v>970</v>
+        <v>954</v>
       </c>
       <c r="E892" t="s">
         <v>25</v>
@@ -73883,16 +74302,16 @@
     </row>
     <row r="893" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A893" t="s">
-        <v>979</v>
+        <v>963</v>
       </c>
       <c r="B893" t="s">
-        <v>980</v>
+        <v>964</v>
       </c>
       <c r="C893" t="s">
         <v>936</v>
       </c>
       <c r="D893" t="s">
-        <v>970</v>
+        <v>965</v>
       </c>
       <c r="E893" t="s">
         <v>25</v>
@@ -73921,16 +74340,16 @@
     </row>
     <row r="894" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A894" t="s">
-        <v>981</v>
+        <v>966</v>
       </c>
       <c r="B894" t="s">
-        <v>982</v>
+        <v>967</v>
       </c>
       <c r="C894" t="s">
         <v>936</v>
       </c>
       <c r="D894" t="s">
-        <v>983</v>
+        <v>965</v>
       </c>
       <c r="E894" t="s">
         <v>25</v>
@@ -73959,16 +74378,16 @@
     </row>
     <row r="895" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A895" t="s">
-        <v>984</v>
+        <v>968</v>
       </c>
       <c r="B895" t="s">
-        <v>985</v>
+        <v>969</v>
       </c>
       <c r="C895" t="s">
         <v>936</v>
       </c>
       <c r="D895" t="s">
-        <v>983</v>
+        <v>970</v>
       </c>
       <c r="E895" t="s">
         <v>25</v>
@@ -73997,16 +74416,16 @@
     </row>
     <row r="896" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A896" t="s">
-        <v>986</v>
+        <v>971</v>
       </c>
       <c r="B896" t="s">
-        <v>987</v>
+        <v>972</v>
       </c>
       <c r="C896" t="s">
         <v>936</v>
       </c>
       <c r="D896" t="s">
-        <v>983</v>
+        <v>970</v>
       </c>
       <c r="E896" t="s">
         <v>25</v>
@@ -74035,16 +74454,16 @@
     </row>
     <row r="897" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A897" t="s">
-        <v>988</v>
+        <v>973</v>
       </c>
       <c r="B897" t="s">
-        <v>989</v>
+        <v>974</v>
       </c>
       <c r="C897" t="s">
         <v>936</v>
       </c>
       <c r="D897" t="s">
-        <v>983</v>
+        <v>970</v>
       </c>
       <c r="E897" t="s">
         <v>25</v>
@@ -74073,16 +74492,16 @@
     </row>
     <row r="898" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A898" t="s">
-        <v>990</v>
+        <v>975</v>
       </c>
       <c r="B898" t="s">
-        <v>991</v>
+        <v>976</v>
       </c>
       <c r="C898" t="s">
         <v>936</v>
       </c>
       <c r="D898" t="s">
-        <v>992</v>
+        <v>970</v>
       </c>
       <c r="E898" t="s">
         <v>25</v>
@@ -74111,16 +74530,16 @@
     </row>
     <row r="899" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A899" t="s">
-        <v>993</v>
+        <v>977</v>
       </c>
       <c r="B899" t="s">
-        <v>994</v>
+        <v>978</v>
       </c>
       <c r="C899" t="s">
         <v>936</v>
       </c>
       <c r="D899" t="s">
-        <v>992</v>
+        <v>970</v>
       </c>
       <c r="E899" t="s">
         <v>25</v>
@@ -74149,16 +74568,16 @@
     </row>
     <row r="900" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A900" t="s">
-        <v>995</v>
+        <v>979</v>
       </c>
       <c r="B900" t="s">
-        <v>996</v>
+        <v>980</v>
       </c>
       <c r="C900" t="s">
         <v>936</v>
       </c>
       <c r="D900" t="s">
-        <v>992</v>
+        <v>970</v>
       </c>
       <c r="E900" t="s">
         <v>25</v>
@@ -74187,16 +74606,16 @@
     </row>
     <row r="901" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A901" t="s">
-        <v>997</v>
+        <v>981</v>
       </c>
       <c r="B901" t="s">
-        <v>998</v>
+        <v>982</v>
       </c>
       <c r="C901" t="s">
         <v>936</v>
       </c>
       <c r="D901" t="s">
-        <v>992</v>
+        <v>983</v>
       </c>
       <c r="E901" t="s">
         <v>25</v>
@@ -74225,16 +74644,16 @@
     </row>
     <row r="902" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A902" t="s">
-        <v>999</v>
+        <v>984</v>
       </c>
       <c r="B902" t="s">
-        <v>1000</v>
+        <v>985</v>
       </c>
       <c r="C902" t="s">
         <v>936</v>
       </c>
       <c r="D902" t="s">
-        <v>1001</v>
+        <v>983</v>
       </c>
       <c r="E902" t="s">
         <v>25</v>
@@ -74263,16 +74682,16 @@
     </row>
     <row r="903" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A903" t="s">
-        <v>1002</v>
+        <v>986</v>
       </c>
       <c r="B903" t="s">
-        <v>1003</v>
+        <v>987</v>
       </c>
       <c r="C903" t="s">
         <v>936</v>
       </c>
       <c r="D903" t="s">
-        <v>1001</v>
+        <v>983</v>
       </c>
       <c r="E903" t="s">
         <v>25</v>
@@ -74301,16 +74720,16 @@
     </row>
     <row r="904" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A904" t="s">
-        <v>1004</v>
+        <v>988</v>
       </c>
       <c r="B904" t="s">
-        <v>1005</v>
+        <v>989</v>
       </c>
       <c r="C904" t="s">
         <v>936</v>
       </c>
       <c r="D904" t="s">
-        <v>1001</v>
+        <v>983</v>
       </c>
       <c r="E904" t="s">
         <v>25</v>
@@ -74339,16 +74758,16 @@
     </row>
     <row r="905" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A905" t="s">
-        <v>1006</v>
+        <v>990</v>
       </c>
       <c r="B905" t="s">
-        <v>1007</v>
+        <v>991</v>
       </c>
       <c r="C905" t="s">
         <v>936</v>
       </c>
       <c r="D905" t="s">
-        <v>1001</v>
+        <v>992</v>
       </c>
       <c r="E905" t="s">
         <v>25</v>
@@ -74377,16 +74796,16 @@
     </row>
     <row r="906" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A906" t="s">
-        <v>1008</v>
+        <v>993</v>
       </c>
       <c r="B906" t="s">
-        <v>1009</v>
+        <v>994</v>
       </c>
       <c r="C906" t="s">
         <v>936</v>
       </c>
       <c r="D906" t="s">
-        <v>1010</v>
+        <v>992</v>
       </c>
       <c r="E906" t="s">
         <v>25</v>
@@ -74415,16 +74834,16 @@
     </row>
     <row r="907" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A907" t="s">
-        <v>1011</v>
+        <v>995</v>
       </c>
       <c r="B907" t="s">
-        <v>1012</v>
+        <v>996</v>
       </c>
       <c r="C907" t="s">
         <v>936</v>
       </c>
       <c r="D907" t="s">
-        <v>1010</v>
+        <v>992</v>
       </c>
       <c r="E907" t="s">
         <v>25</v>
@@ -74453,16 +74872,16 @@
     </row>
     <row r="908" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A908" t="s">
-        <v>1013</v>
+        <v>997</v>
       </c>
       <c r="B908" t="s">
-        <v>1014</v>
+        <v>998</v>
       </c>
       <c r="C908" t="s">
         <v>936</v>
       </c>
       <c r="D908" t="s">
-        <v>1010</v>
+        <v>992</v>
       </c>
       <c r="E908" t="s">
         <v>25</v>
@@ -74491,16 +74910,16 @@
     </row>
     <row r="909" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A909" t="s">
-        <v>1015</v>
+        <v>999</v>
       </c>
       <c r="B909" t="s">
-        <v>1016</v>
+        <v>1000</v>
       </c>
       <c r="C909" t="s">
         <v>936</v>
       </c>
       <c r="D909" t="s">
-        <v>1010</v>
+        <v>1001</v>
       </c>
       <c r="E909" t="s">
         <v>25</v>
@@ -74529,16 +74948,16 @@
     </row>
     <row r="910" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A910" t="s">
-        <v>1017</v>
+        <v>1002</v>
       </c>
       <c r="B910" t="s">
-        <v>1018</v>
+        <v>1003</v>
       </c>
       <c r="C910" t="s">
         <v>936</v>
       </c>
       <c r="D910" t="s">
-        <v>1019</v>
+        <v>1001</v>
       </c>
       <c r="E910" t="s">
         <v>25</v>
@@ -74567,16 +74986,16 @@
     </row>
     <row r="911" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A911" t="s">
-        <v>1020</v>
+        <v>1004</v>
       </c>
       <c r="B911" t="s">
-        <v>1021</v>
+        <v>1005</v>
       </c>
       <c r="C911" t="s">
         <v>936</v>
       </c>
       <c r="D911" t="s">
-        <v>1019</v>
+        <v>1001</v>
       </c>
       <c r="E911" t="s">
         <v>25</v>
@@ -74605,16 +75024,16 @@
     </row>
     <row r="912" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A912" t="s">
-        <v>1022</v>
+        <v>1006</v>
       </c>
       <c r="B912" t="s">
-        <v>1023</v>
+        <v>1007</v>
       </c>
       <c r="C912" t="s">
         <v>936</v>
       </c>
       <c r="D912" t="s">
-        <v>1019</v>
+        <v>1001</v>
       </c>
       <c r="E912" t="s">
         <v>25</v>
@@ -74643,16 +75062,16 @@
     </row>
     <row r="913" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A913" t="s">
-        <v>1024</v>
+        <v>1008</v>
       </c>
       <c r="B913" t="s">
-        <v>1025</v>
+        <v>1009</v>
       </c>
       <c r="C913" t="s">
         <v>936</v>
       </c>
       <c r="D913" t="s">
-        <v>1019</v>
+        <v>1010</v>
       </c>
       <c r="E913" t="s">
         <v>25</v>
@@ -74681,16 +75100,16 @@
     </row>
     <row r="914" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A914" t="s">
-        <v>1026</v>
+        <v>1011</v>
       </c>
       <c r="B914" t="s">
-        <v>1027</v>
+        <v>1012</v>
       </c>
       <c r="C914" t="s">
         <v>936</v>
       </c>
       <c r="D914" t="s">
-        <v>1019</v>
+        <v>1010</v>
       </c>
       <c r="E914" t="s">
         <v>25</v>
@@ -74719,39 +75138,305 @@
     </row>
     <row r="915" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A915" t="s">
-        <v>1028</v>
+        <v>1013</v>
       </c>
       <c r="B915" t="s">
-        <v>1029</v>
+        <v>1014</v>
       </c>
       <c r="C915" t="s">
         <v>936</v>
       </c>
       <c r="D915" t="s">
+        <v>1010</v>
+      </c>
+      <c r="E915" t="s">
+        <v>25</v>
+      </c>
+      <c r="F915" t="s">
+        <v>25</v>
+      </c>
+      <c r="G915" t="s">
+        <v>25</v>
+      </c>
+      <c r="H915" t="s">
+        <v>19</v>
+      </c>
+      <c r="I915" t="s">
+        <v>25</v>
+      </c>
+      <c r="J915" t="s">
+        <v>25</v>
+      </c>
+      <c r="K915" t="s">
+        <v>25</v>
+      </c>
+      <c r="L915" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="916" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A916" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B916" t="s">
+        <v>1016</v>
+      </c>
+      <c r="C916" t="s">
+        <v>936</v>
+      </c>
+      <c r="D916" t="s">
+        <v>1010</v>
+      </c>
+      <c r="E916" t="s">
+        <v>25</v>
+      </c>
+      <c r="F916" t="s">
+        <v>25</v>
+      </c>
+      <c r="G916" t="s">
+        <v>25</v>
+      </c>
+      <c r="H916" t="s">
+        <v>19</v>
+      </c>
+      <c r="I916" t="s">
+        <v>25</v>
+      </c>
+      <c r="J916" t="s">
+        <v>25</v>
+      </c>
+      <c r="K916" t="s">
+        <v>25</v>
+      </c>
+      <c r="L916" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="917" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A917" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B917" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C917" t="s">
+        <v>936</v>
+      </c>
+      <c r="D917" t="s">
         <v>1019</v>
       </c>
-      <c r="E915" t="s">
-        <v>25</v>
-      </c>
-      <c r="F915" t="s">
-        <v>25</v>
-      </c>
-      <c r="G915" t="s">
-        <v>25</v>
-      </c>
-      <c r="H915" t="s">
-        <v>19</v>
-      </c>
-      <c r="I915" t="s">
-        <v>25</v>
-      </c>
-      <c r="J915" t="s">
-        <v>25</v>
-      </c>
-      <c r="K915" t="s">
-        <v>25</v>
-      </c>
-      <c r="L915" t="s">
+      <c r="E917" t="s">
+        <v>25</v>
+      </c>
+      <c r="F917" t="s">
+        <v>25</v>
+      </c>
+      <c r="G917" t="s">
+        <v>25</v>
+      </c>
+      <c r="H917" t="s">
+        <v>19</v>
+      </c>
+      <c r="I917" t="s">
+        <v>25</v>
+      </c>
+      <c r="J917" t="s">
+        <v>25</v>
+      </c>
+      <c r="K917" t="s">
+        <v>25</v>
+      </c>
+      <c r="L917" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="918" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A918" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B918" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C918" t="s">
+        <v>936</v>
+      </c>
+      <c r="D918" t="s">
+        <v>1019</v>
+      </c>
+      <c r="E918" t="s">
+        <v>25</v>
+      </c>
+      <c r="F918" t="s">
+        <v>25</v>
+      </c>
+      <c r="G918" t="s">
+        <v>25</v>
+      </c>
+      <c r="H918" t="s">
+        <v>19</v>
+      </c>
+      <c r="I918" t="s">
+        <v>25</v>
+      </c>
+      <c r="J918" t="s">
+        <v>25</v>
+      </c>
+      <c r="K918" t="s">
+        <v>25</v>
+      </c>
+      <c r="L918" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="919" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A919" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B919" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C919" t="s">
+        <v>936</v>
+      </c>
+      <c r="D919" t="s">
+        <v>1019</v>
+      </c>
+      <c r="E919" t="s">
+        <v>25</v>
+      </c>
+      <c r="F919" t="s">
+        <v>25</v>
+      </c>
+      <c r="G919" t="s">
+        <v>25</v>
+      </c>
+      <c r="H919" t="s">
+        <v>19</v>
+      </c>
+      <c r="I919" t="s">
+        <v>25</v>
+      </c>
+      <c r="J919" t="s">
+        <v>25</v>
+      </c>
+      <c r="K919" t="s">
+        <v>25</v>
+      </c>
+      <c r="L919" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="920" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A920" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B920" t="s">
+        <v>1025</v>
+      </c>
+      <c r="C920" t="s">
+        <v>936</v>
+      </c>
+      <c r="D920" t="s">
+        <v>1019</v>
+      </c>
+      <c r="E920" t="s">
+        <v>25</v>
+      </c>
+      <c r="F920" t="s">
+        <v>25</v>
+      </c>
+      <c r="G920" t="s">
+        <v>25</v>
+      </c>
+      <c r="H920" t="s">
+        <v>19</v>
+      </c>
+      <c r="I920" t="s">
+        <v>25</v>
+      </c>
+      <c r="J920" t="s">
+        <v>25</v>
+      </c>
+      <c r="K920" t="s">
+        <v>25</v>
+      </c>
+      <c r="L920" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="921" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A921" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B921" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C921" t="s">
+        <v>936</v>
+      </c>
+      <c r="D921" t="s">
+        <v>1019</v>
+      </c>
+      <c r="E921" t="s">
+        <v>25</v>
+      </c>
+      <c r="F921" t="s">
+        <v>25</v>
+      </c>
+      <c r="G921" t="s">
+        <v>25</v>
+      </c>
+      <c r="H921" t="s">
+        <v>19</v>
+      </c>
+      <c r="I921" t="s">
+        <v>25</v>
+      </c>
+      <c r="J921" t="s">
+        <v>25</v>
+      </c>
+      <c r="K921" t="s">
+        <v>25</v>
+      </c>
+      <c r="L921" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="922" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A922" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B922" t="s">
+        <v>1029</v>
+      </c>
+      <c r="C922" t="s">
+        <v>936</v>
+      </c>
+      <c r="D922" t="s">
+        <v>1019</v>
+      </c>
+      <c r="E922" t="s">
+        <v>25</v>
+      </c>
+      <c r="F922" t="s">
+        <v>25</v>
+      </c>
+      <c r="G922" t="s">
+        <v>25</v>
+      </c>
+      <c r="H922" t="s">
+        <v>19</v>
+      </c>
+      <c r="I922" t="s">
+        <v>25</v>
+      </c>
+      <c r="J922" t="s">
+        <v>25</v>
+      </c>
+      <c r="K922" t="s">
+        <v>25</v>
+      </c>
+      <c r="L922" t="s">
         <v>25</v>
       </c>
     </row>
@@ -74760,7 +75445,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L3 A50:D50 L37 G37:I37 G38:L38 B39:L39 B37:E38 A81 A56:D56 L56 A59:D59 J59:L59 A62:D62 J62:L62 H56 F59 F62 H59 H62 A53:D53 H53:I53 A5:L7 A4:E4 G4:L4 L53 F50 H50:L50 A19:L20 B10:D10 A11:D12 F10:F12 J10:L12 H10:H12 B17:D18 F17:F18 H17:H18 J17:L17 K18:L18 A28:G28 L21 F22:F24 J22:L24 A33:D36 L33 A21:D25 H21:H25 L25 A29:D29 H29:I29 L29 K28:L28 I28 F34:F36 J34:L36 H33:H36 A63:G63 I63:L63 A66:D66 F66 H66:L66 A67:A68 J67:L68 J72:L73 F72 F73:G73 F67:G68 C67:D68 H72 A72:A74 A84 I84:L84 C72:D74 A77 C77:D77 C81:D81 L74 J77:L77 J81:L81 F84:G84 F77 F81 H74 H77 H81 C84:D84 A85:D85 L85 A87 J87:L87 H85 F87 H87 C87:D87 A91:D91 F91 H91:L91 A97:G99 L98 A96:D96 F96 H96:L96 A122:D122 I97:L97 I98:J98 I99:L99 A101:D101 F101 A104:D104 H104:I104 J101:L101 H101 L104 A109:D109 H109:I109 L109 A113:G113 I113:L113 A117 F117 C117:D117 A121 C121:D121 F121 J117:L117 J121:L121 A138:D138 K126:L126 H117 H121 H122:I122 L122 A126:D127 H126:I127 L127 A128:G128 I128:L128 A130:D130 F130 H130:L130 A131:G132 I131:L132 A134:D134 F134 H134:L134 A142:D142 F142 H138 J138:L138 H142:L142 A143:G143 I143:L143 A144:D144 H144:I144 L144 A151:D151 F151 H151:L151 A155:F156 A152:G154 A157:G157 I152:L157 A159:D159 F159 H159:L159 A167:D167 A162:A163 C163:G163 C162:D162 J163:L163 L162 H162 A165:D165 F165 H165:L165 A181:L181 A172:D172 I172:L172 A168:G168 I168:L168 F167 H167:L167 F172 A176:D176 F176 H176:L176 A177:G179 I177:L179 A180:E180 G180:I180 L180 A206:D206 A182:G182 I182:L182 A188:D188 F188 H188:L188 A189:G189 I189:L189 F191 H191:L191 A191:D192 H192:I192 L192 F196 H196:L196 A196:D197 H197:I197 L197 A198:G198 I198:L198 A200:D200 F200 H200:L200 F202 H202:L202 A210:G210 A209:D209 H209:L209 A202:D203 H203:I203 L203 K227:L228 F206 H206:L206 F209 A213:F213 A212:G212 A211:F211 A214:G214 I210:L214 A217:D217 F217 H217 A220:D220 F220 H220 J217:L217 J220:L220 I226:L226 I227:I228 A227:G231 I229:L231 A233:D233 F233 H233:L233 A262:G262 A255:G258 K258:L258 A240:D240 F240 H240:L240 A241:A242 H241:I242 L241:L242 C241:D242 A245:D245 F245 H245:L245 A343:G343 A265:D265 L265 A246:G247 I246:L247 A251:D251 I251 A254:D254 I254 L251 L254 I255:L257 I258 A261:D261 F261 H261:L261 I262:L262 F265 H265:I265 A269:D269 F269 H269:L269 A272:D272 F272 H272:L272 A276:D276 F276 H276:L276 A279:D279 H279:L279 A283:D283 F283 H283:L283 C287:D287 F287 H287:L287 A291:D291 F291 H291:L291 A295:D295 F295 H295:L295 A298:D298 F298 H298:L298 A299:G299 I299:L299 A303:D303 F303 H303:L303 A305:D305 F305 H305:L305 A308:D308 F308 H308:L308 A311:D311 F311 H311:L311 A312:G312 I312:L312 A315:D315 F315 H315:L315 A319:D319 F319 H319:L319 A323:D323 F323 H323:L323 A331:D331 F331 H331:L331 A332:G332 I332:L332 A335:D335 F335 H335:L335 A336:G337 I336:L337 A359:D359 A346:D346 I346:L346 I343:L343 F346 A385:D385 A363:D363 L363 A350:D350 F350 H350:L350 A352:D352 F352 H352:L352 A354:D354 F354 H354:I354 K354:L354 A355:G355 I355:L355 F359 H359:L359 F363 H363:J363 A367:D367 F367 H367:L367 A368:G368 I368:L368 A371:D371 F371 H371:L371 A375:D375 F375 H375:L375 A378:D378 F378 H378:L378 A379:G379 I379:L379 A382:D382 F382 H382:L382 A393:D393 A387:D387 H387 F385 H385:L385 J387:L387 A389:D389 J389:L389 F387 H389 F389 A390:G392 I390:L391 A408:D408 A394:G394 I394:L394 J392:L392 L393 H393 C397:D397 F397 H397 J397:L397 A401:D401 F401 H401 J401:L401 A438 C409:F409 I409:L409 A405:D405 F405 H405 J405:L405 F408 H408 J408:L408 A413 F413 A417 F417 A420 F420 J413:L413 J417:L417 J420:L420 C417:D417 C420:D420 C413:D413 H413 H417 H420 A425:D425 F425 H425 J425:L425 A426:G426 I426:L426 A427:D427 H427 L427 A469 A440 L440 A428:G428 I428:L428 A431:D431 F431 H431:L431 A432:G434 I432:L434 F438 F440 H438 H440 J438:L438 J440 C438:D438 C440:D440 A445:D445 F445 H445:L445 A446:G449 I446:L449 A452:D452 F452 H452:L452 A454:D454 F454 H454:L454 A460:D460 F460 H460:L460 A462 F462 A464 F464 H462 H464 J464:L464 J462:L462 C462:D462 C464:D464 A466 J466:L466 F466 C466:D466 A467:G467 I467:L467 A470:G470 I470:L470 F469 H469 J469:L469 A562:D562 A482:D482 L482 C469:D469 H475:L475 A475:D476 H476:I476 H477 A477:A479 F478:F479 C477:D479 L476:L477 H478:L479 F482 H482 J482 A485:D485 F485 H485:L485 A488:D488 F488 H488:L488 A491:D491 F491 H491:L491 A494:D494 F494 H494:L494 A498:D498 F498 H498:L498 A502:D502 F502 H502:L502 A505:D505 F505 H505:L505 A508:D508 F508 H508:L508 A509:G511 I509:L511 A516:D516 F516 H516:L516 A520 F520 H520:L520 A525:D525 F525 H525:L525 A528:D528 F528 H528:L528 A532:D532 F532 H532:L532 A540 I540:L540 A542:D542 F542 H542:L542 A544:D544 F544 H544:L544 A546:D546 F546 H546:L546 A548:D548 F548 H548:L548 A551:D551 H551:L551 A553:D553 F553 H553:L553 A576:D576 A563 C563:G563 A559:D559 F559 H559:L559 F562 H562:L562 F540 C540:D540 I563:L563 C520:D520 A565:D565 F565 H565:L565 A567:D567 F567 H567:L567 A586:D586 A584 C584:D584 A721:L915 A590:D590 L590 A570:D570 F570 H570:L570 A572:D572 F572 H572:L572 A575 F575 H575:L575 C575:D575 H576:I576 L576 F584 H584:L584 F586 H586:L586 F590 H590:J590 A617:D617 A622:B622 D622 A226:D226 F226 A591:G591 I591:L591 A592:D592 H592:I592 L592 A596:D596 A600:D600 F600 H600:L600 F596 H596:L596 A604:D604 F604 H604:L604 A607:D607 F607 H607:L607 A608:G608 A612:D612 F612 H612:L612 I617:L617 I608:L608 F617 F622 H622:L622 A626:D626 F626 H626:L626 A627:G627 I627:L627 A629:D629 F629 H629:L629 A633:D633 F633 H633:L633 A634:G635 I634:L635 A640:D640 F640 H640:L640 A644:D644 F644 H644:L644 A647:D647 F647 H647:L647 A651:D651 F651 H651:L651 A654 C654:D654 F654 H654:L654 A657:D657 F657 H657:L657 A659:D659 F659 H659:L659 A662:D662 F662 H662:L662 A666:D666 F666 H666:L666 A670:D670 F670 H670:L670 A674:D674 F674 H674:L674 A678:D678 F678 H678:L678 A681:D681 F681 H681:L681 A684:D684 F684 H684:L684 A689:D689 F689 H689:L689 A692:D692 F692 H692:L692 A693:G693 I693:L693 A697:D697 F697 H697:L697 C702:D702 F702 H702:L702 C703:G703 I703:L703 A707:D707 F707 H707:L707 A708:G708 I708:L708 A713:D713 F713 H713:L713 A714:G715 I714:L715 A716:G716 A720:D720 F720 H720:L720 I716:L716" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L3 A50:D50 L37 G37:I37 G38:L38 B39:L39 B37:E38 A81 A56:D56 L56 A59:D59 J59:L59 A62:D62 J62:L62 H56 F59 F62 H59 H62 A53:D53 H53:I53 A5:L7 A4:E4 G4:L4 L53 F50 H50:L50 A19:L20 B10:D10 A11:D12 F10:F12 J10:L12 H10:H12 B17:D18 F17:F18 H17:H18 J17:L17 K18:L18 A28:G28 L21 F22:F24 J22:L24 A33:D36 L33 A21:D25 H21:H25 L25 A29:D29 H29:I29 L29 K28:L28 I28 F34:F36 J34:L36 H33:H36 A63:G63 I63:L63 A66:D66 F66 H66:L66 A67:A68 J67:L68 J72:L73 F72 F73:G73 F67:G68 C67:D68 H72 A72:A74 A84 I84:L84 C72:D74 A77 C77:D77 C81:D81 L74 J77:L77 J81:L81 F84:G84 F77 F81 H74 H77 H81 C84:D84 A85:D85 L85 A87 J87:L87 H85 F87 H87 C87:D87 A91:D91 F91 H91:L91 A97:G99 L98 A96:D96 F96 H96:L96 A122:D122 I97:L97 I98:J98 I99:L99 A101:D101 F101 A104:D104 H104:I104 J101:L101 H101 L104 A109:D109 H109:I109 L109 A113:G113 I113:L113 A117 F117 C117:D117 A121 C121:D121 F121 J117:L117 J121:L121 A138:D138 K126:L126 H117 H121 H122:I122 L122 A126:D127 H126:I127 L127 A128:G128 I128:L128 A130:D130 F130 H130:L130 A131:G132 I131:L132 A134:D134 F134 H134:L134 A142:D142 F142 H138 J138:L138 H142:L142 A143:G143 I143:L143 A144:D144 H144:I144 L144 A151:D151 F151 H151:L151 A155:F156 A152:G154 A157:G157 I152:L157 A159:D159 F159 H159:L159 A167:D167 A162:A163 C163:G163 C162:D162 J163:L163 L162 H162 A165:D165 F165 H165:L165 A181:L181 A172:D172 I172:L172 A168:G168 I168:L168 F167 H167:L167 F172 A176:D176 F176 H176:L176 A177:G179 I177:L179 A180:E180 G180:I180 L180 A206:D206 A182:G182 I182:L182 A188:D188 F188 H188:L188 A189:G189 I189:L189 F191 H191:L191 A191:D192 H192:I192 L192 F196 H196:L196 A196:D197 H197:I197 L197 A198:G198 I198:L198 A200:D200 F200 H200:L200 F202 H202:L202 A210:G210 A209:D209 H209:L209 A202:D203 H203:I203 L203 K227:L228 F206 H206:L206 F209 A213:F213 A212:G212 A211:F211 A214:G214 I210:L214 A217:D217 F217 H217 A220:D220 F220 H220 J217:L217 J220:L220 I226:L226 I227:I228 A227:G231 I229:L231 A233:D233 F233 H233:L233 A262:G262 A255:G258 K258:L258 A240:D240 F240 H240:L240 A241:A242 H241:I242 L241:L242 C241:D242 A245:D245 F245 H245:L245 A343:G343 A265:D265 L265 A246:G247 I246:L247 A251:D251 I251 A254:D254 I254 L251 L254 I255:L257 I258 A261:D261 F261 H261:L261 I262:L262 F265 H265:I265 A269:D269 F269 H269:L269 A272:D272 F272 H272:L272 A276:D276 F276 H276:L276 A279:D279 H279:L279 A283:D283 F283 H283:L283 C287:D287 F287 H287:L287 A291:D291 F291 H291:L291 A295:D295 F295 H295:L295 A298:D298 F298 H298:L298 A299:G299 I299:L299 A303:D303 F303 H303:L303 A305:D305 F305 H305:L305 A308:D308 F308 H308:L308 A311:D311 F311 H311:L311 A312:G312 I312:L312 A315:D315 F315 H315:L315 A319:D319 F319 H319:L319 A323:D323 F323 H323:L323 A331:D331 F331 H331:L331 A332:G332 I332:L332 A335:D335 F335 H335:L335 A336:G337 I336:L337 A359:D359 A346:D346 I346:L346 I343:L343 F346 A385:D385 A363:D363 L363 A350:D350 F350 H350:L350 A352:D352 F352 H352:L352 A354:D354 F354 H354:I354 K354:L354 A355:G355 I355:L355 F359 H359:L359 F363 H363:J363 A367:D367 F367 H367:L367 A368:G368 I368:L368 A371:D371 F371 H371:L371 A375:D375 F375 H375:L375 A378:D378 F378 H378:L378 A379:G379 I379:L379 A382:D382 F382 H382:L382 A393:D393 A387:D387 H387 F385 H385:L385 J387:L387 A389:D389 J389:L389 F387 H389 F389 A390:G392 I390:L391 A408:D408 A394:G394 I394:L394 J392:L392 L393 H393 C397:D397 F397 H397 J397:L397 A401:D401 F401 H401 J401:L401 A438 C409:F409 I409:L409 A405:D405 F405 H405 J405:L405 F408 H408 J408:L408 A413 F413 A417 F417 A420 F420 J413:L413 J417:L417 J420:L420 C417:D417 C420:D420 C413:D413 H413 H417 H420 A425:D425 F425 H425 J425:L425 A426:G426 I426:L426 A427:D427 H427 L427 A469 A440 L440 A428:G428 I428:L428 A431:D431 F431 H431:L431 A432:G434 I432:L434 F438 F440 H438 H440 J438:L438 J440 C438:D438 C440:D440 A445:D445 F445 H445:L445 A446:G449 I446:L449 A452:D452 F452 H452:L452 A454:D454 F454 H454:L454 A460:D460 F460 H460:L460 A462 F462 A464 F464 H462 H464 J464:L464 J462:L462 C462:D462 C464:D464 A466 J466:L466 F466 C466:D466 A467:G467 I467:L467 A470:G470 I470:L470 F469 H469 J469:L469 A562:D562 A482:D482 L482 C469:D469 H475:L475 A475:D476 H476:I476 H477 A477:A479 F478:F479 C477:D479 L476:L477 H478:L479 F482 H482 J482 A485:D485 F485 H485:L485 A488:D488 F488 H488:L488 A491:D491 F491 H491:L491 A494:D494 F494 H494:L494 A498:D498 F498 H498:L498 A502:D502 F502 H502:L502 A505:D505 F505 H505:L505 A508:D508 F508 H508:L508 A509:G511 I509:L511 A516:D516 F516 H516:L516 A520 F520 H520:L520 A525:D525 F525 H525:L525 A528:D528 F528 H528:L528 A532:D532 F532 H532:L532 A540 I540:L540 A542:D542 F542 H542:L542 A544:D544 F544 H544:L544 A546:D546 F546 H546:L546 A548:D548 F548 H548:L548 A551:D551 H551:L551 A553:D553 F553 H553:L553 A576:D576 A563 C563:G563 A559:D559 F559 H559:L559 F562 H562:L562 F540 C540:D540 I563:L563 C520:D520 A565:D565 F565 H565:L565 A567:D567 F567 H567:L567 A586:D586 A584 C584:D584 A729:L922 A590:D590 L590 A570:D570 F570 H570:L570 A572:D572 F572 H572:L572 A575 F575 H575:L575 C575:D575 H576:I576 L576 F584 H584:L584 F586 H586:L586 F590 H590:J590 A617:D617 A622:B622 D622 A226:D226 F226 A591:G591 I591:L591 A592:D592 H592:I592 L592 A596:D596 A600:D600 F600 H600:L600 F596 H596:L596 A604:D604 F604 H604:L604 A607:D607 F607 H607:L607 A608:G608 A612:D612 F612 H612:L612 I617:L617 I608:L608 F617 F622 H622:L622 A626:D626 F626 H626:L626 A627:G627 I627:L627 A629:D629 F629 H629:L629 A633:D633 F633 H633:L633 A634:G635 I634:L635 A640:D640 F640 H640:L640 A644:D644 F644 H644:L644 A647:D647 F647 H647:L647 A651:D651 F651 H651:L651 A654 C654:D654 F654 H654:L654 A657:D657 F657 H657:L657 A659:D659 F659 H659:L659 A662:D662 F662 H662:L662 A666:D666 F666 H666:L666 A670:D670 F670 H670:L670 A674:D674 F674 H674:L674 A678:D678 F678 H678:L678 A681:D681 F681 H681:L681 A684:D684 F684 H684:L684 A689:D689 F689 H689:L689 A692:D692 F692 H692:L692 A693:G693 I693:L693 A697:D697 F697 H697:L697 C702:D702 F702 H702:L702 C703:G703 I703:L703 A707:D707 F707 H707:L707 A708:G708 I708:L708 A713:D713 F713 H713:L713 A714:G715 I714:L715 A716:G716 A720:D720 F720 H720:L720 I716:L716 A728:D728 F728 H728:L728" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>